<commit_message>
docs(evie-ai): close phase1 implementation contract gaps
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -604,7 +604,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L28" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L32" headerRowCount="1">
   <autoFilter ref="A3:L24"/>
   <tableColumns count="12">
     <tableColumn id="1" name="任务ID"/>
@@ -656,7 +656,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F28" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F33" headerRowCount="1">
   <autoFilter ref="A3:F25"/>
   <tableColumns count="6">
     <tableColumn id="1" name="验证ID"/>
@@ -742,7 +742,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N84" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N95" headerRowCount="1">
   <autoFilter ref="A1:N84"/>
   <tableColumns count="14">
     <tableColumn id="1" name="用例ID"/>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>f5c8226a729288e68617a4956873eb462a6ed74f（文档分支基线）</t>
+          <t>07caca0（本轮可实施性修订前 HEAD；修订待提交）</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>• Specification/Plan 状态为 Approved；文档合并后才允许从最新 dev 创建 Slice 1 分支。</t>
+          <t>• Specification/Plan 五处可实施性缺口已补齐；Phase 1 计划用例更新为 94 条，Slice 1 仍待文档 PR 合并。</t>
         </is>
       </c>
       <c r="E19" s="22" t="n"/>
@@ -1376,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N84"/>
+  <dimension ref="A1:N95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4591,22 +4591,22 @@
       </c>
       <c r="F45" s="29" t="inlineStr">
         <is>
-          <t>跨项目访问拒绝</t>
+          <t>全部公开 API 仅 admin 访问 active project</t>
         </is>
       </c>
       <c r="G45" s="29" t="inlineStr">
         <is>
-          <t>principal 无目标项目权限</t>
+          <t>非 admin 分别调用列表/详情/版本历史/审核历史/写接口</t>
         </is>
       </c>
       <c r="H45" s="29" t="inlineStr">
         <is>
-          <t>调用查询/写 API</t>
+          <t>逐类调用公开 API</t>
         </is>
       </c>
       <c r="I45" s="29" t="inlineStr">
         <is>
-          <t>403 EVIE_PROJECT_SCOPE_FORBIDDEN</t>
+          <t>全部返回 403 EVIE_PROJECT_SCOPE_FORBIDDEN</t>
         </is>
       </c>
       <c r="J45" s="29" t="inlineStr">
@@ -6684,7 +6684,7 @@
       </c>
       <c r="G74" s="29" t="inlineStr">
         <is>
-          <t>新建/复用/版本/审核/删除/恢复</t>
+          <t>新建/复用/新版本/历史版本恢复/审核/删除/资产恢复</t>
         </is>
       </c>
       <c r="H74" s="29" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="I74" s="29" t="inlineStr">
         <is>
-          <t>返回批准的 201/200 状态</t>
+          <t>历史版本恢复与新版本返回 201，其余返回批准的 201/200 状态</t>
         </is>
       </c>
       <c r="J74" s="29" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="G76" s="29" t="inlineStr">
         <is>
-          <t>版本/审核/删除/恢复缺字段</t>
+          <t>新版本/历史版本恢复/审核/删除/资产恢复缺字段</t>
         </is>
       </c>
       <c r="H76" s="29" t="inlineStr">
@@ -7438,6 +7438,798 @@
         </is>
       </c>
       <c r="N84" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-084</t>
+        </is>
+      </c>
+      <c r="B85" s="29" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="C85" s="29" t="inlineStr">
+        <is>
+          <t>Fingerprint</t>
+        </is>
+      </c>
+      <c r="D85" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E85" s="29" t="inlineStr">
+        <is>
+          <t>D-05</t>
+        </is>
+      </c>
+      <c r="F85" s="29" t="inlineStr">
+        <is>
+          <t>Content fingerprint canonical JSON 稳定序列化</t>
+        </is>
+      </c>
+      <c r="G85" s="29" t="inlineStr">
+        <is>
+          <t>六个字段规范化结果相同但输入键顺序不同</t>
+        </is>
+      </c>
+      <c r="H85" s="29" t="inlineStr">
+        <is>
+          <t>按固定键名/键排序/UTF-8/无空白序列化并计算 SHA-256</t>
+        </is>
+      </c>
+      <c r="I85" s="29" t="inlineStr">
+        <is>
+          <t>跨进程得到相同字节流和指纹，不使用字符串拼接</t>
+        </is>
+      </c>
+      <c r="J85" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K85" s="29" t="inlineStr">
+        <is>
+          <t>单元</t>
+        </is>
+      </c>
+      <c r="L85" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="M85" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-05</t>
+        </is>
+      </c>
+      <c r="N85" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-085</t>
+        </is>
+      </c>
+      <c r="B86" s="29" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="C86" s="29" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="D86" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E86" s="29" t="inlineStr">
+        <is>
+          <t>D-06</t>
+        </is>
+      </c>
+      <c r="F86" s="29" t="inlineStr">
+        <is>
+          <t>conversion_status 合法集合不包含 failed</t>
+        </is>
+      </c>
+      <c r="G86" s="29" t="inlineStr">
+        <is>
+          <t>读取集中状态常量和状态迁移 Policy</t>
+        </is>
+      </c>
+      <c r="H86" s="29" t="inlineStr">
+        <is>
+          <t>枚举并验证全部合法值</t>
+        </is>
+      </c>
+      <c r="I86" s="29" t="inlineStr">
+        <is>
+          <t>仅含 not_started/processing/blocked/succeeded/stale；failed 被拒绝</t>
+        </is>
+      </c>
+      <c r="J86" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K86" s="29" t="inlineStr">
+        <is>
+          <t>单元</t>
+        </is>
+      </c>
+      <c r="L86" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_lifecycle_policy.py</t>
+        </is>
+      </c>
+      <c r="M86" s="29" t="inlineStr">
+        <is>
+          <t>Phase 0 常量已只读确认</t>
+        </is>
+      </c>
+      <c r="N86" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-086</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2</t>
+        </is>
+      </c>
+      <c r="C87" s="29" t="inlineStr">
+        <is>
+          <t>ORM</t>
+        </is>
+      </c>
+      <c r="D87" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E87" s="29" t="inlineStr">
+        <is>
+          <t>D-02/A-07</t>
+        </is>
+      </c>
+      <c r="F87" s="29" t="inlineStr">
+        <is>
+          <t>来源唯一约束固定为资产加来源身份</t>
+        </is>
+      </c>
+      <c r="G87" s="29" t="inlineStr">
+        <is>
+          <t>同资产、同 source_identity_hash 的重复来源</t>
+        </is>
+      </c>
+      <c r="H87" s="29" t="inlineStr">
+        <is>
+          <t>尝试插入重复来源</t>
+        </is>
+      </c>
+      <c r="I87" s="29" t="inlineStr">
+        <is>
+          <t>UNIQUE(test_asset_pk, source_identity_hash) 拒绝；唯一键不重复包含 source_type</t>
+        </is>
+      </c>
+      <c r="J87" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K87" s="29" t="inlineStr">
+        <is>
+          <t>数据库单元</t>
+        </is>
+      </c>
+      <c r="L87" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="M87" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：A-07</t>
+        </is>
+      </c>
+      <c r="N87" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-087</t>
+        </is>
+      </c>
+      <c r="B88" s="29" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C88" s="29" t="inlineStr">
+        <is>
+          <t>Idempotency</t>
+        </is>
+      </c>
+      <c r="D88" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E88" s="29" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="F88" s="29" t="inlineStr">
+        <is>
+          <t>过期 Idempotency-Key 可作为新请求复用</t>
+        </is>
+      </c>
+      <c r="G88" s="29" t="inlineStr">
+        <is>
+          <t>同 scope/key 的记录已过 expires_at</t>
+        </is>
+      </c>
+      <c r="H88" s="29" t="inlineStr">
+        <is>
+          <t>提交新的请求指纹</t>
+        </is>
+      </c>
+      <c r="I88" s="29" t="inlineStr">
+        <is>
+          <t>安全建立新幂等占用并按新请求处理</t>
+        </is>
+      </c>
+      <c r="J88" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K88" s="29" t="inlineStr">
+        <is>
+          <t>数据库单元</t>
+        </is>
+      </c>
+      <c r="L88" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_idempotency_repository.py</t>
+        </is>
+      </c>
+      <c r="M88" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-04</t>
+        </is>
+      </c>
+      <c r="N88" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-088</t>
+        </is>
+      </c>
+      <c r="B89" s="29" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C89" s="29" t="inlineStr">
+        <is>
+          <t>Idempotency并发</t>
+        </is>
+      </c>
+      <c r="D89" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E89" s="29" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="F89" s="29" t="inlineStr">
+        <is>
+          <t>过期清理与重新占用无并发窗口</t>
+        </is>
+      </c>
+      <c r="G89" s="29" t="inlineStr">
+        <is>
+          <t>两个 Session 同时清理并重用过期 key</t>
+        </is>
+      </c>
+      <c r="H89" s="29" t="inlineStr">
+        <is>
+          <t>并发执行 reclaim</t>
+        </is>
+      </c>
+      <c r="I89" s="29" t="inlineStr">
+        <is>
+          <t>数据库唯一性和事务保证只有一个新占用成功</t>
+        </is>
+      </c>
+      <c r="J89" s="29" t="inlineStr">
+        <is>
+          <t>PostgreSQL/SQLite</t>
+        </is>
+      </c>
+      <c r="K89" s="29" t="inlineStr">
+        <is>
+          <t>并发集成</t>
+        </is>
+      </c>
+      <c r="L89" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_idempotency_concurrency.py</t>
+        </is>
+      </c>
+      <c r="M89" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-04</t>
+        </is>
+      </c>
+      <c r="N89" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-089</t>
+        </is>
+      </c>
+      <c r="B90" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C90" s="29" t="inlineStr">
+        <is>
+          <t>Intake并发事务</t>
+        </is>
+      </c>
+      <c r="D90" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E90" s="29" t="inlineStr">
+        <is>
+          <t>D-03/D-05</t>
+        </is>
+      </c>
+      <c r="F90" s="29" t="inlineStr">
+        <is>
+          <t>新建 claim 唯一冲突后使用干净事务复用</t>
+        </is>
+      </c>
+      <c r="G90" s="29" t="inlineStr">
+        <is>
+          <t>两个不同 key 同内容并发且初始均未查到 claim</t>
+        </is>
+      </c>
+      <c r="H90" s="29" t="inlineStr">
+        <is>
+          <t>并发执行 Intake</t>
+        </is>
+      </c>
+      <c r="I90" s="29" t="inlineStr">
+        <is>
+          <t>失败新建事务全回滚；失败 Session 不再使用；新事务读取 claim 后完成复用</t>
+        </is>
+      </c>
+      <c r="J90" s="29" t="inlineStr">
+        <is>
+          <t>PostgreSQL/SQLite</t>
+        </is>
+      </c>
+      <c r="K90" s="29" t="inlineStr">
+        <is>
+          <t>并发集成</t>
+        </is>
+      </c>
+      <c r="L90" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_intake_concurrency.py</t>
+        </is>
+      </c>
+      <c r="M90" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-03/D-05</t>
+        </is>
+      </c>
+      <c r="N90" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-090</t>
+        </is>
+      </c>
+      <c r="B91" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2</t>
+        </is>
+      </c>
+      <c r="C91" s="29" t="inlineStr">
+        <is>
+          <t>Schema边界</t>
+        </is>
+      </c>
+      <c r="D91" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E91" s="29" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="F91" s="29" t="inlineStr">
+        <is>
+          <t>TestAssetVersion 严格排除非版本领域事实</t>
+        </is>
+      </c>
+      <c r="G91" s="29" t="inlineStr">
+        <is>
+          <t>构造包含 asset_code/current_version_pk/status/source/review/audit/idempotency/claim 的版本请求</t>
+        </is>
+      </c>
+      <c r="H91" s="29" t="inlineStr">
+        <is>
+          <t>执行 Pydantic 字段集合与拒绝测试</t>
+        </is>
+      </c>
+      <c r="I91" s="29" t="inlineStr">
+        <is>
+          <t>版本只接受 title/precondition/natural_steps/expected_result/priority/tags</t>
+        </is>
+      </c>
+      <c r="J91" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K91" s="29" t="inlineStr">
+        <is>
+          <t>结构</t>
+        </is>
+      </c>
+      <c r="L91" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="M91" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：A-10</t>
+        </is>
+      </c>
+      <c r="N91" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-091</t>
+        </is>
+      </c>
+      <c r="B92" s="29" t="inlineStr">
+        <is>
+          <t>Slice 8</t>
+        </is>
+      </c>
+      <c r="C92" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D92" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E92" s="29" t="inlineStr">
+        <is>
+          <t>D-06/D-11</t>
+        </is>
+      </c>
+      <c r="F92" s="29" t="inlineStr">
+        <is>
+          <t>历史版本恢复 API 创建新版本</t>
+        </is>
+      </c>
+      <c r="G92" s="29" t="inlineStr">
+        <is>
+          <t>资产存在历史版本且 row_version 有效</t>
+        </is>
+      </c>
+      <c r="H92" s="29" t="inlineStr">
+        <is>
+          <t>POST /versions/{version_id}/restore</t>
+        </is>
+      </c>
+      <c r="I92" s="29" t="inlineStr">
+        <is>
+          <t>201 返回新 version_id，current 指向新版本且历史行不变</t>
+        </is>
+      </c>
+      <c r="J92" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K92" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L92" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_api.py</t>
+        </is>
+      </c>
+      <c r="M92" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-06/D-11</t>
+        </is>
+      </c>
+      <c r="N92" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-092</t>
+        </is>
+      </c>
+      <c r="B93" s="29" t="inlineStr">
+        <is>
+          <t>Slice 8</t>
+        </is>
+      </c>
+      <c r="C93" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D93" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E93" s="29" t="inlineStr">
+        <is>
+          <t>D-06/D-11</t>
+        </is>
+      </c>
+      <c r="F93" s="29" t="inlineStr">
+        <is>
+          <t>历史版本恢复版本不存在与跨资产拒绝</t>
+        </is>
+      </c>
+      <c r="G93" s="29" t="inlineStr">
+        <is>
+          <t>version_id 不存在或属于其他 TestAsset</t>
+        </is>
+      </c>
+      <c r="H93" s="29" t="inlineStr">
+        <is>
+          <t>调用历史版本恢复 API</t>
+        </is>
+      </c>
+      <c r="I93" s="29" t="inlineStr">
+        <is>
+          <t>分别返回 EVIE_VERSION_NOT_FOUND / EVIE_VERSION_SCOPE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="J93" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K93" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L93" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_api.py</t>
+        </is>
+      </c>
+      <c r="M93" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-06/D-11</t>
+        </is>
+      </c>
+      <c r="N93" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-093</t>
+        </is>
+      </c>
+      <c r="B94" s="29" t="inlineStr">
+        <is>
+          <t>Slice 8</t>
+        </is>
+      </c>
+      <c r="C94" s="29" t="inlineStr">
+        <is>
+          <t>API安全</t>
+        </is>
+      </c>
+      <c r="D94" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E94" s="29" t="inlineStr">
+        <is>
+          <t>A-02/D-11</t>
+        </is>
+      </c>
+      <c r="F94" s="29" t="inlineStr">
+        <is>
+          <t>项目不存在与非 active 使用稳定错误码</t>
+        </is>
+      </c>
+      <c r="G94" s="29" t="inlineStr">
+        <is>
+          <t>admin 请求未知或 inactive project</t>
+        </is>
+      </c>
+      <c r="H94" s="29" t="inlineStr">
+        <is>
+          <t>调用任一公开 API</t>
+        </is>
+      </c>
+      <c r="I94" s="29" t="inlineStr">
+        <is>
+          <t>分别返回 EVIE_PROJECT_NOT_FOUND / EVIE_PROJECT_INACTIVE，不创建默认项目</t>
+        </is>
+      </c>
+      <c r="J94" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K94" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L94" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_api_safety.py</t>
+        </is>
+      </c>
+      <c r="M94" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：A-02</t>
+        </is>
+      </c>
+      <c r="N94" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-094</t>
+        </is>
+      </c>
+      <c r="B95" s="29" t="inlineStr">
+        <is>
+          <t>Slice 8</t>
+        </is>
+      </c>
+      <c r="C95" s="29" t="inlineStr">
+        <is>
+          <t>API错误</t>
+        </is>
+      </c>
+      <c r="D95" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E95" s="29" t="inlineStr">
+        <is>
+          <t>D-11/A-08</t>
+        </is>
+      </c>
+      <c r="F95" s="29" t="inlineStr">
+        <is>
+          <t>审核版本和数据完整性稳定错误映射</t>
+        </is>
+      </c>
+      <c r="G95" s="29" t="inlineStr">
+        <is>
+          <t>审核目标非 current version 或 Repository 检测到领域不一致</t>
+        </is>
+      </c>
+      <c r="H95" s="29" t="inlineStr">
+        <is>
+          <t>调用审核/查询 API</t>
+        </is>
+      </c>
+      <c r="I95" s="29" t="inlineStr">
+        <is>
+          <t>返回 EVIE_REVIEW_VERSION_NOT_CURRENT 或 EVIE_DATA_INTEGRITY_ERROR，不泄露 SQL/正文</t>
+        </is>
+      </c>
+      <c r="J95" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K95" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L95" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_api.py</t>
+        </is>
+      </c>
+      <c r="M95" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：A-08/D-11</t>
+        </is>
+      </c>
+      <c r="N95" s="29" t="inlineStr">
         <is>
           <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
         </is>
@@ -7458,7 +8250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9284,6 +10076,68 @@
       <c r="L31" s="12" t="inlineStr">
         <is>
           <t>文档合并后从最新 dev 创建 Slice 1 分支</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>DOC-06</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 可实施性评审</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>补齐 Specification/Plan 五处实施缺口</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>把已签字规则写成可直接实现且无歧义的合同</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>补齐 admin-only 读权限、Content Claim 新建并发顺序、conversion_status 合法集、非版本事实边界、历史版本恢复 API；同步非阻塞错误码/唯一约束/指纹/幂等语义</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Specification、Implementation Plan、Excel 测试台账</t>
+        </is>
+      </c>
+      <c r="H32" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>5 处缺口已闭合；未新增架构决策；Slice 1 仍等待文档 PR 合并</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>仅 docs/evie-ai；未修改 ORM、Migration、Service、API、数据库</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>docs/evie-ai-phase1-lifecycle / PR #5</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>完成文档一致性检查并更新 PR</t>
         </is>
       </c>
     </row>
@@ -9528,7 +10382,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
@@ -9801,7 +10654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10783,6 +11636,38 @@
       <c r="F32" s="12" t="inlineStr">
         <is>
           <t>D-01～D-14、A-01～A-10 无冲突；无待签字残留</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>DOC-V06</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 可实施性缺口同步审查</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Specification/Plan/Excel 一致性与 conversion_status 只读核对</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Phase 0 合法 conversion_status 不含 failed；5 处实施缺口和 4 项非阻塞合同已同步</t>
         </is>
       </c>
     </row>
@@ -13508,7 +14393,7 @@
       </c>
       <c r="F4" s="29" t="inlineStr">
         <is>
-          <t>77 passed, 11 warnings in 7.09s</t>
+          <t>77 passed, 11 warnings in 7.09s（代码未变，本轮未重跑）</t>
         </is>
       </c>
       <c r="G4" s="5" t="n"/>
@@ -13531,7 +14416,7 @@
         </is>
       </c>
       <c r="F5" s="29" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="6" t="n"/>

</xml_diff>

<commit_message>
docs(evie-ai): close phase1 concurrency and migration gaps
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -604,7 +604,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L32" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L33" headerRowCount="1">
   <autoFilter ref="A3:L24"/>
   <tableColumns count="12">
     <tableColumn id="1" name="任务ID"/>
@@ -656,7 +656,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F33" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F34" headerRowCount="1">
   <autoFilter ref="A3:F25"/>
   <tableColumns count="6">
     <tableColumn id="1" name="验证ID"/>
@@ -742,7 +742,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N95" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N98" headerRowCount="1">
   <autoFilter ref="A1:N84"/>
   <tableColumns count="14">
     <tableColumn id="1" name="用例ID"/>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>07caca0（本轮可实施性修订前 HEAD；修订待提交）</t>
+          <t>4a07745（本轮最终合同修订前 HEAD；修订待提交）</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>• Specification/Plan 五处可实施性缺口已补齐；Phase 1 计划用例更新为 94 条，Slice 1 仍待文档 PR 合并。</t>
+          <t>• 最终合同审查补齐完整 Intake 并发回退与 Migration 指纹冻结；Phase 1 计划用例更新为 97 条，Slice 1 仍待文档 PR 合并。</t>
         </is>
       </c>
       <c r="E19" s="22" t="n"/>
@@ -1376,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N95"/>
+  <dimension ref="A1:N98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="F90" s="29" t="inlineStr">
         <is>
-          <t>新建 claim 唯一冲突后使用干净事务复用</t>
+          <t>新建 claim 唯一冲突后从完整 Intake 重启</t>
         </is>
       </c>
       <c r="G90" s="29" t="inlineStr">
@@ -7841,12 +7841,12 @@
       </c>
       <c r="H90" s="29" t="inlineStr">
         <is>
-          <t>并发执行 Intake</t>
+          <t>回滚失败事务并用干净事务重校 scope/request fingerprint/幂等后重进 Intake</t>
         </is>
       </c>
       <c r="I90" s="29" t="inlineStr">
         <is>
-          <t>失败新建事务全回滚；失败 Session 不再使用；新事务读取 claim 后完成复用</t>
+          <t>同幂等请求重放原结果；否则读取 Content Claim 后复用；来源和审计不重复</t>
         </is>
       </c>
       <c r="J90" s="29" t="inlineStr">
@@ -8230,6 +8230,222 @@
         </is>
       </c>
       <c r="N95" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-095</t>
+        </is>
+      </c>
+      <c r="B96" s="29" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="C96" s="29" t="inlineStr">
+        <is>
+          <t>Migration确定性</t>
+        </is>
+      </c>
+      <c r="D96" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E96" s="29" t="inlineStr">
+        <is>
+          <t>D-13/A-06</t>
+        </is>
+      </c>
+      <c r="F96" s="29" t="inlineStr">
+        <is>
+          <t>Migration 使用冻结指纹算法与固定测试向量</t>
+        </is>
+      </c>
+      <c r="G96" s="29" t="inlineStr">
+        <is>
+          <t>存量资产和跨平台固定输入向量</t>
+        </is>
+      </c>
+      <c r="H96" s="29" t="inlineStr">
+        <is>
+          <t>执行 revision-local 规范化/canonical JSON/SHA-256</t>
+        </is>
+      </c>
+      <c r="I96" s="29" t="inlineStr">
+        <is>
+          <t>结果与发布时应用 Policy 相同，历史 revision 不导入可演进应用模块</t>
+        </is>
+      </c>
+      <c r="J96" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K96" s="29" t="inlineStr">
+        <is>
+          <t>迁移结构/集成</t>
+        </is>
+      </c>
+      <c r="L96" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="M96" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-13/A-06</t>
+        </is>
+      </c>
+      <c r="N96" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-096</t>
+        </is>
+      </c>
+      <c r="B97" s="29" t="inlineStr">
+        <is>
+          <t>Slice 3/4</t>
+        </is>
+      </c>
+      <c r="C97" s="29" t="inlineStr">
+        <is>
+          <t>来源一致性</t>
+        </is>
+      </c>
+      <c r="D97" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E97" s="29" t="inlineStr">
+        <is>
+          <t>A-04</t>
+        </is>
+      </c>
+      <c r="F97" s="29" t="inlineStr">
+        <is>
+          <t>无组合 FK 时来源主子异常 fail-closed</t>
+        </is>
+      </c>
+      <c r="G97" s="29" t="inlineStr">
+        <is>
+          <t>直接构造 requirement 缺子记录和 manual 存在子记录</t>
+        </is>
+      </c>
+      <c r="H97" s="29" t="inlineStr">
+        <is>
+          <t>通过 Repository 读取并执行 Migration 校验</t>
+        </is>
+      </c>
+      <c r="I97" s="29" t="inlineStr">
+        <is>
+          <t>Repository 与 Migration 均明确失败；Service 不产生该状态</t>
+        </is>
+      </c>
+      <c r="J97" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K97" s="29" t="inlineStr">
+        <is>
+          <t>数据库集成</t>
+        </is>
+      </c>
+      <c r="L97" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_source_integrity.py</t>
+        </is>
+      </c>
+      <c r="M97" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：A-04</t>
+        </is>
+      </c>
+      <c r="N97" s="29" t="inlineStr">
+        <is>
+          <t>Plan 明确不复制 source_type、不使用组合 FK。</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-097</t>
+        </is>
+      </c>
+      <c r="B98" s="29" t="inlineStr">
+        <is>
+          <t>Slice 8</t>
+        </is>
+      </c>
+      <c r="C98" s="29" t="inlineStr">
+        <is>
+          <t>API契约</t>
+        </is>
+      </c>
+      <c r="D98" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E98" s="29" t="inlineStr">
+        <is>
+          <t>D-06/D-11</t>
+        </is>
+      </c>
+      <c r="F98" s="29" t="inlineStr">
+        <is>
+          <t>历史版本恢复路径只接受 tav_ 公共 ID</t>
+        </is>
+      </c>
+      <c r="G98" s="29" t="inlineStr">
+        <is>
+          <t>分别使用合法 tav_ ID、内部整数和错误前缀</t>
+        </is>
+      </c>
+      <c r="H98" s="29" t="inlineStr">
+        <is>
+          <t>调用 /versions/{test_asset_version_id}/restore</t>
+        </is>
+      </c>
+      <c r="I98" s="29" t="inlineStr">
+        <is>
+          <t>合法公共 ID 进入 Service；内部 PK 和错误格式返回 422</t>
+        </is>
+      </c>
+      <c r="J98" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K98" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L98" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_api.py</t>
+        </is>
+      </c>
+      <c r="M98" s="29" t="inlineStr">
+        <is>
+          <t>合同已批准：D-06/D-11</t>
+        </is>
+      </c>
+      <c r="N98" s="29" t="inlineStr">
         <is>
           <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
         </is>
@@ -8250,7 +8466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10136,6 +10352,68 @@
         </is>
       </c>
       <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>完成文档一致性检查并更新 PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>DOC-07</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 最终合同审查</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>补齐 Intake 并发回退与 Migration 指纹冻结</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>消除幂等并发重复写风险和历史 Migration 非确定性风险</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>并发 Claim 冲突后从完整 Intake 重启；冻结 revision-local 指纹算法；版本路径使用公共 tav_ ID；Plan 明确不使用组合 FK及 fail-closed 测试</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Specification、Implementation Plan、README、Excel 测试台账</t>
+        </is>
+      </c>
+      <c r="H33" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>两项阻塞合同及两项非阻塞细化已同步；Specification 保持 Approved，Plan 进入 Final Review</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>仅 docs/evie-ai；未修改 ORM、Migration、Service、API、数据库</t>
+        </is>
+      </c>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>docs/evie-ai-phase1-lifecycle / PR #5</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
         <is>
           <t>完成文档一致性检查并更新 PR</t>
         </is>
@@ -10654,7 +10932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11668,6 +11946,38 @@
       <c r="F33" s="12" t="inlineStr">
         <is>
           <t>Phase 0 合法 conversion_status 不含 failed；5 处实施缺口和 4 项非阻塞合同已同步</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>DOC-V07</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>最终合同确定性审查</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Specification/Plan/README/Excel 交叉检查</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>并发回退不绕过幂等；Migration 指纹算法冻结；历史版本参数使用 tav_ 公共 ID；来源异常 fail-closed</t>
         </is>
       </c>
     </row>
@@ -14416,7 +14726,7 @@
         </is>
       </c>
       <c r="F5" s="29" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="6" t="n"/>

</xml_diff>

<commit_message>
docs(evie-ai): approve phase1 implementation plan
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -604,7 +604,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L33" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L34" headerRowCount="1">
   <autoFilter ref="A3:L24"/>
   <tableColumns count="12">
     <tableColumn id="1" name="任务ID"/>
@@ -656,7 +656,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F34" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F35" headerRowCount="1">
   <autoFilter ref="A3:F25"/>
   <tableColumns count="6">
     <tableColumn id="1" name="验证ID"/>
@@ -742,7 +742,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N98" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N113" headerRowCount="1">
   <autoFilter ref="A1:N84"/>
   <tableColumns count="14">
     <tableColumn id="1" name="用例ID"/>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>4a07745（本轮最终合同修订前 HEAD；修订待提交）</t>
+          <t>3fb07fa（本轮 Plan 最终定版前 HEAD；修订待提交）</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>• 最终合同审查补齐完整 Intake 并发回退与 Migration 指纹冻结；Phase 1 计划用例更新为 97 条，Slice 1 仍待文档 PR 合并。</t>
+          <t>• Implementation Plan 已纳入 P-01～P-06 并更新为 Approved；Phase 1 计划用例 112 条，Slice 1 仍待文档 PR 合并。</t>
         </is>
       </c>
       <c r="E19" s="22" t="n"/>
@@ -1376,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N98"/>
+  <dimension ref="A1:N113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8451,6 +8451,1086 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-098</t>
+        </is>
+      </c>
+      <c r="B99" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3</t>
+        </is>
+      </c>
+      <c r="C99" s="29" t="inlineStr">
+        <is>
+          <t>交付守卫</t>
+        </is>
+      </c>
+      <c r="D99" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E99" s="29" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="F99" s="29" t="inlineStr">
+        <is>
+          <t>ORM 与 Migration 原子 PR 交付</t>
+        </is>
+      </c>
+      <c r="G99" s="29" t="inlineStr">
+        <is>
+          <t>功能分支包含 Slice 2 ORM 变更</t>
+        </is>
+      </c>
+      <c r="H99" s="29" t="inlineStr">
+        <is>
+          <t>检查 PR 文件与切片门禁</t>
+        </is>
+      </c>
+      <c r="I99" s="29" t="inlineStr">
+        <is>
+          <t>缺少对应线性 Migration 时禁止合并；具备双数据库升级证据后才允许</t>
+        </is>
+      </c>
+      <c r="J99" s="29" t="inlineStr">
+        <is>
+          <t>CI/Git</t>
+        </is>
+      </c>
+      <c r="K99" s="29" t="inlineStr">
+        <is>
+          <t>结构</t>
+        </is>
+      </c>
+      <c r="L99" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_delivery_boundaries.py</t>
+        </is>
+      </c>
+      <c r="M99" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-01</t>
+        </is>
+      </c>
+      <c r="N99" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-099</t>
+        </is>
+      </c>
+      <c r="B100" s="29" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="C100" s="29" t="inlineStr">
+        <is>
+          <t>Idempotency Policy</t>
+        </is>
+      </c>
+      <c r="D100" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E100" s="29" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="F100" s="29" t="inlineStr">
+        <is>
+          <t>operation_type 固定枚举</t>
+        </is>
+      </c>
+      <c r="G100" s="29" t="inlineStr">
+        <is>
+          <t>六个批准操作和任意自由文本</t>
+        </is>
+      </c>
+      <c r="H100" s="29" t="inlineStr">
+        <is>
+          <t>解析 operation_type</t>
+        </is>
+      </c>
+      <c r="I100" s="29" t="inlineStr">
+        <is>
+          <t>仅接受六个固定值；Router 路径/函数名/自由文本被拒绝</t>
+        </is>
+      </c>
+      <c r="J100" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K100" s="29" t="inlineStr">
+        <is>
+          <t>单元</t>
+        </is>
+      </c>
+      <c r="L100" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_idempotency_policy.py</t>
+        </is>
+      </c>
+      <c r="M100" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-02</t>
+        </is>
+      </c>
+      <c r="N100" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-100</t>
+        </is>
+      </c>
+      <c r="B101" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3</t>
+        </is>
+      </c>
+      <c r="C101" s="29" t="inlineStr">
+        <is>
+          <t>ORM/Migration</t>
+        </is>
+      </c>
+      <c r="D101" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E101" s="29" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="F101" s="29" t="inlineStr">
+        <is>
+          <t>幂等完整 scope 唯一约束与显式名称</t>
+        </is>
+      </c>
+      <c r="G101" s="29" t="inlineStr">
+        <is>
+          <t>相同 project/operation/actor/key</t>
+        </is>
+      </c>
+      <c r="H101" s="29" t="inlineStr">
+        <is>
+          <t>并发或顺序插入两条记录</t>
+        </is>
+      </c>
+      <c r="I101" s="29" t="inlineStr">
+        <is>
+          <t>uq_test_asset_idempotency_scope_key 拒绝重复且名称小于 63 字节</t>
+        </is>
+      </c>
+      <c r="J101" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K101" s="29" t="inlineStr">
+        <is>
+          <t>数据库单元</t>
+        </is>
+      </c>
+      <c r="L101" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="M101" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-02</t>
+        </is>
+      </c>
+      <c r="N101" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-101</t>
+        </is>
+      </c>
+      <c r="B102" s="29" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C102" s="29" t="inlineStr">
+        <is>
+          <t>Idempotency CAS</t>
+        </is>
+      </c>
+      <c r="D102" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E102" s="29" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="F102" s="29" t="inlineStr">
+        <is>
+          <t>过期记录使用 generation CAS 重新占用</t>
+        </is>
+      </c>
+      <c r="G102" s="29" t="inlineStr">
+        <is>
+          <t>两个 Session 读取相同过期 generation</t>
+        </is>
+      </c>
+      <c r="H102" s="29" t="inlineStr">
+        <is>
+          <t>并发条件更新</t>
+        </is>
+      </c>
+      <c r="I102" s="29" t="inlineStr">
+        <is>
+          <t>仅一个递增 generation 并清空旧结果；失败方重读且不覆盖</t>
+        </is>
+      </c>
+      <c r="J102" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K102" s="29" t="inlineStr">
+        <is>
+          <t>并发集成</t>
+        </is>
+      </c>
+      <c r="L102" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_idempotency_concurrency.py</t>
+        </is>
+      </c>
+      <c r="M102" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-02</t>
+        </is>
+      </c>
+      <c r="N102" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-102</t>
+        </is>
+      </c>
+      <c r="B103" s="29" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C103" s="29" t="inlineStr">
+        <is>
+          <t>Idempotency并发</t>
+        </is>
+      </c>
+      <c r="D103" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E103" s="29" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="F103" s="29" t="inlineStr">
+        <is>
+          <t>不存在记录的并发插入回退</t>
+        </is>
+      </c>
+      <c r="G103" s="29" t="inlineStr">
+        <is>
+          <t>两个 Session 同 scope/key 且初始无记录</t>
+        </is>
+      </c>
+      <c r="H103" s="29" t="inlineStr">
+        <is>
+          <t>并发插入</t>
+        </is>
+      </c>
+      <c r="I103" s="29" t="inlineStr">
+        <is>
+          <t>唯一冲突事务回滚；干净事务重新检查并得到确定结果</t>
+        </is>
+      </c>
+      <c r="J103" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K103" s="29" t="inlineStr">
+        <is>
+          <t>并发集成</t>
+        </is>
+      </c>
+      <c r="L103" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_idempotency_concurrency.py</t>
+        </is>
+      </c>
+      <c r="M103" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-02</t>
+        </is>
+      </c>
+      <c r="N103" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-103</t>
+        </is>
+      </c>
+      <c r="B104" s="29" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C104" s="29" t="inlineStr">
+        <is>
+          <t>Idempotency结果</t>
+        </is>
+      </c>
+      <c r="D104" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E104" s="29" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="F104" s="29" t="inlineStr">
+        <is>
+          <t>重放返回不可变操作结果 Envelope</t>
+        </is>
+      </c>
+      <c r="G104" s="29" t="inlineStr">
+        <is>
+          <t>原操作完成后资产又被编辑或删除</t>
+        </is>
+      </c>
+      <c r="H104" s="29" t="inlineStr">
+        <is>
+          <t>使用相同 key 重放</t>
+        </is>
+      </c>
+      <c r="I104" s="29" t="inlineStr">
+        <is>
+          <t>返回原 status/IDs/flags/completed row_version，不被当前资产状态覆盖</t>
+        </is>
+      </c>
+      <c r="J104" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K104" s="29" t="inlineStr">
+        <is>
+          <t>服务集成</t>
+        </is>
+      </c>
+      <c r="L104" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_idempotency_replay.py</t>
+        </is>
+      </c>
+      <c r="M104" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-03</t>
+        </is>
+      </c>
+      <c r="N104" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-104</t>
+        </is>
+      </c>
+      <c r="B105" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/4</t>
+        </is>
+      </c>
+      <c r="C105" s="29" t="inlineStr">
+        <is>
+          <t>隐私边界</t>
+        </is>
+      </c>
+      <c r="D105" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E105" s="29" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="F105" s="29" t="inlineStr">
+        <is>
+          <t>幂等记录不保存自然语言正文</t>
+        </is>
+      </c>
+      <c r="G105" s="29" t="inlineStr">
+        <is>
+          <t>创建请求包含全部自然语言字段</t>
+        </is>
+      </c>
+      <c r="H105" s="29" t="inlineStr">
+        <is>
+          <t>检查幂等持久化记录</t>
+        </is>
+      </c>
+      <c r="I105" s="29" t="inlineStr">
+        <is>
+          <t>仅保存结果摘要，不含 title/precondition/natural_steps/expected_result/完整响应</t>
+        </is>
+      </c>
+      <c r="J105" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K105" s="29" t="inlineStr">
+        <is>
+          <t>数据库集成</t>
+        </is>
+      </c>
+      <c r="L105" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_idempotency_replay.py</t>
+        </is>
+      </c>
+      <c r="M105" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-03</t>
+        </is>
+      </c>
+      <c r="N105" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-105</t>
+        </is>
+      </c>
+      <c r="B106" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C106" s="29" t="inlineStr">
+        <is>
+          <t>Intake并发</t>
+        </is>
+      </c>
+      <c r="D106" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E106" s="29" t="inlineStr">
+        <is>
+          <t>P-04</t>
+        </is>
+      </c>
+      <c r="F106" s="29" t="inlineStr">
+        <is>
+          <t>PostgreSQL 两事务 Claim 竞态新 Session 读取获胜结果</t>
+        </is>
+      </c>
+      <c r="G106" s="29" t="inlineStr">
+        <is>
+          <t>两事务并发相同 content fingerprint</t>
+        </is>
+      </c>
+      <c r="H106" s="29" t="inlineStr">
+        <is>
+          <t>执行 Intake</t>
+        </is>
+      </c>
+      <c r="I106" s="29" t="inlineStr">
+        <is>
+          <t>失败 Session 回滚关闭；新 Session 完整重入并读取获胜 claim</t>
+        </is>
+      </c>
+      <c r="J106" s="29" t="inlineStr">
+        <is>
+          <t>PostgreSQL 16</t>
+        </is>
+      </c>
+      <c r="K106" s="29" t="inlineStr">
+        <is>
+          <t>并发集成</t>
+        </is>
+      </c>
+      <c r="L106" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_intake_concurrency.py</t>
+        </is>
+      </c>
+      <c r="M106" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-04</t>
+        </is>
+      </c>
+      <c r="N106" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-106</t>
+        </is>
+      </c>
+      <c r="B107" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C107" s="29" t="inlineStr">
+        <is>
+          <t>Intake并发</t>
+        </is>
+      </c>
+      <c r="D107" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E107" s="29" t="inlineStr">
+        <is>
+          <t>P-04</t>
+        </is>
+      </c>
+      <c r="F107" s="29" t="inlineStr">
+        <is>
+          <t>文件型 SQLite 多连接 Claim 竞态</t>
+        </is>
+      </c>
+      <c r="G107" s="29" t="inlineStr">
+        <is>
+          <t>两个独立连接并发相同 content fingerprint</t>
+        </is>
+      </c>
+      <c r="H107" s="29" t="inlineStr">
+        <is>
+          <t>执行 Intake</t>
+        </is>
+      </c>
+      <c r="I107" s="29" t="inlineStr">
+        <is>
+          <t>唯一约束/CAS 提供等价语义；新连接完成一次重入，无进程锁依赖</t>
+        </is>
+      </c>
+      <c r="J107" s="29" t="inlineStr">
+        <is>
+          <t>文件型 SQLite</t>
+        </is>
+      </c>
+      <c r="K107" s="29" t="inlineStr">
+        <is>
+          <t>并发集成</t>
+        </is>
+      </c>
+      <c r="L107" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_intake_concurrency.py</t>
+        </is>
+      </c>
+      <c r="M107" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-04</t>
+        </is>
+      </c>
+      <c r="N107" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-107</t>
+        </is>
+      </c>
+      <c r="B108" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C108" s="29" t="inlineStr">
+        <is>
+          <t>异常映射</t>
+        </is>
+      </c>
+      <c r="D108" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E108" s="29" t="inlineStr">
+        <is>
+          <t>P-04</t>
+        </is>
+      </c>
+      <c r="F108" s="29" t="inlineStr">
+        <is>
+          <t>非目标 IntegrityError 不误判为重复复用</t>
+        </is>
+      </c>
+      <c r="G108" s="29" t="inlineStr">
+        <is>
+          <t>制造无关 FK/Unique 约束错误</t>
+        </is>
+      </c>
+      <c r="H108" s="29" t="inlineStr">
+        <is>
+          <t>执行 Intake</t>
+        </is>
+      </c>
+      <c r="I108" s="29" t="inlineStr">
+        <is>
+          <t>fail-closed 为数据完整性错误，不进入 duplicate/idempotency 回退</t>
+        </is>
+      </c>
+      <c r="J108" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K108" s="29" t="inlineStr">
+        <is>
+          <t>服务集成</t>
+        </is>
+      </c>
+      <c r="L108" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_intake_errors.py</t>
+        </is>
+      </c>
+      <c r="M108" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-04</t>
+        </is>
+      </c>
+      <c r="N108" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-108</t>
+        </is>
+      </c>
+      <c r="B109" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C109" s="29" t="inlineStr">
+        <is>
+          <t>重试边界</t>
+        </is>
+      </c>
+      <c r="D109" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E109" s="29" t="inlineStr">
+        <is>
+          <t>P-04</t>
+        </is>
+      </c>
+      <c r="F109" s="29" t="inlineStr">
+        <is>
+          <t>Content Claim 完整重入最多一次</t>
+        </is>
+      </c>
+      <c r="G109" s="29" t="inlineStr">
+        <is>
+          <t>重入后仍无法读取获胜 claim或再次冲突</t>
+        </is>
+      </c>
+      <c r="H109" s="29" t="inlineStr">
+        <is>
+          <t>执行 Intake</t>
+        </is>
+      </c>
+      <c r="I109" s="29" t="inlineStr">
+        <is>
+          <t>第二次异常后 fail-closed，无无限循环，Session 均关闭</t>
+        </is>
+      </c>
+      <c r="J109" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K109" s="29" t="inlineStr">
+        <is>
+          <t>服务集成</t>
+        </is>
+      </c>
+      <c r="L109" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_intake_concurrency.py</t>
+        </is>
+      </c>
+      <c r="M109" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-04</t>
+        </is>
+      </c>
+      <c r="N109" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-109</t>
+        </is>
+      </c>
+      <c r="B110" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3</t>
+        </is>
+      </c>
+      <c r="C110" s="29" t="inlineStr">
+        <is>
+          <t>Phase0不变量</t>
+        </is>
+      </c>
+      <c r="D110" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E110" s="29" t="inlineStr">
+        <is>
+          <t>P-05</t>
+        </is>
+      </c>
+      <c r="F110" s="29" t="inlineStr">
+        <is>
+          <t>current_version_pk 保持 nullable 且无数据库 FK</t>
+        </is>
+      </c>
+      <c r="G110" s="29" t="inlineStr">
+        <is>
+          <t>反射 TestAsset ORM 与 Migration 结构</t>
+        </is>
+      </c>
+      <c r="H110" s="29" t="inlineStr">
+        <is>
+          <t>检查列和 ForeignKey</t>
+        </is>
+      </c>
+      <c r="I110" s="29" t="inlineStr">
+        <is>
+          <t>nullable=true 且不存在数据库 FK；归属仅由 Repository/Service 校验</t>
+        </is>
+      </c>
+      <c r="J110" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K110" s="29" t="inlineStr">
+        <is>
+          <t>结构</t>
+        </is>
+      </c>
+      <c r="L110" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="M110" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-05</t>
+        </is>
+      </c>
+      <c r="N110" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-110</t>
+        </is>
+      </c>
+      <c r="B111" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6/7</t>
+        </is>
+      </c>
+      <c r="C111" s="29" t="inlineStr">
+        <is>
+          <t>Audit矩阵</t>
+        </is>
+      </c>
+      <c r="D111" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E111" s="29" t="inlineStr">
+        <is>
+          <t>P-06</t>
+        </is>
+      </c>
+      <c r="F111" s="29" t="inlineStr">
+        <is>
+          <t>每个生命周期操作生成批准审计事件</t>
+        </is>
+      </c>
+      <c r="G111" s="29" t="inlineStr">
+        <is>
+          <t>逐项执行新建/复用/版本/恢复/审核/删除/恢复/空修改/重放</t>
+        </is>
+      </c>
+      <c r="H111" s="29" t="inlineStr">
+        <is>
+          <t>读取审计历史</t>
+        </is>
+      </c>
+      <c r="I111" s="29" t="inlineStr">
+        <is>
+          <t>事件类型和数量严格符合 P-06；空修改/幂等重放/非法转换无事件</t>
+        </is>
+      </c>
+      <c r="J111" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K111" s="29" t="inlineStr">
+        <is>
+          <t>服务集成</t>
+        </is>
+      </c>
+      <c r="L111" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_audit_events.py</t>
+        </is>
+      </c>
+      <c r="M111" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-06</t>
+        </is>
+      </c>
+      <c r="N111" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-111</t>
+        </is>
+      </c>
+      <c r="B112" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C112" s="29" t="inlineStr">
+        <is>
+          <t>Audit双事件</t>
+        </is>
+      </c>
+      <c r="D112" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E112" s="29" t="inlineStr">
+        <is>
+          <t>P-06</t>
+        </is>
+      </c>
+      <c r="F112" s="29" t="inlineStr">
+        <is>
+          <t>重复复用新增来源产生两个独立事件</t>
+        </is>
+      </c>
+      <c r="G112" s="29" t="inlineStr">
+        <is>
+          <t>重复内容且来源为新的真实来源</t>
+        </is>
+      </c>
+      <c r="H112" s="29" t="inlineStr">
+        <is>
+          <t>执行 Intake</t>
+        </is>
+      </c>
+      <c r="I112" s="29" t="inlineStr">
+        <is>
+          <t>source_added 与 exact_duplicate_reused 共享请求上下文但 audit_event_id 不同</t>
+        </is>
+      </c>
+      <c r="J112" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K112" s="29" t="inlineStr">
+        <is>
+          <t>服务集成</t>
+        </is>
+      </c>
+      <c r="L112" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_audit_events.py</t>
+        </is>
+      </c>
+      <c r="M112" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-06</t>
+        </is>
+      </c>
+      <c r="N112" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-112</t>
+        </is>
+      </c>
+      <c r="B113" s="29" t="inlineStr">
+        <is>
+          <t>Slice 8</t>
+        </is>
+      </c>
+      <c r="C113" s="29" t="inlineStr">
+        <is>
+          <t>API scope</t>
+        </is>
+      </c>
+      <c r="D113" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E113" s="29" t="inlineStr">
+        <is>
+          <t>A-02/P-04</t>
+        </is>
+      </c>
+      <c r="F113" s="29" t="inlineStr">
+        <is>
+          <t>project_code 传输和作用域查询合同</t>
+        </is>
+      </c>
+      <c r="G113" s="29" t="inlineStr">
+        <is>
+          <t>覆盖创建/列表/详情/版本/审核/删除/恢复和跨项目 ID</t>
+        </is>
+      </c>
+      <c r="H113" s="29" t="inlineStr">
+        <is>
+          <t>按合同位置传参并尝试跨项目访问</t>
+        </is>
+      </c>
+      <c r="I113" s="29" t="inlineStr">
+        <is>
+          <t>Body/Query 位置正确；实体按 project+public ID 查询；Requirement 四方项目一致</t>
+        </is>
+      </c>
+      <c r="J113" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K113" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L113" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_api_scope.py</t>
+        </is>
+      </c>
+      <c r="M113" s="29" t="inlineStr">
+        <is>
+          <t>Plan project scope</t>
+        </is>
+      </c>
+      <c r="N113" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8466,7 +9546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10416,6 +11496,68 @@
       <c r="L33" s="12" t="inlineStr">
         <is>
           <t>完成文档一致性检查并更新 PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>DOC-08</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 Implementation Plan 最终定版</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>纳入 P-01～P-06 实施级约束</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>闭合原子数据库交付、幂等并发、结果重放、竞态协调、Phase 0 不变量和审计矩阵</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>固定 Slice2/3 同 PR；operation/唯一约束/CAS；结果 Envelope；单次新 Session 重入；current_version 无 FK；审计矩阵；project scope 传输</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Implementation Plan、README、Excel 测试台账</t>
+        </is>
+      </c>
+      <c r="H34" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>Plan 状态更新为 Approved；架构/合同待签字项均为 0；Slice 1 仍待 PR 合并</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>仅 docs/evie-ai；未修改 Specification、ADR、代码、Migration 或数据库</t>
+        </is>
+      </c>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>docs/evie-ai-phase1-lifecycle / PR #5</t>
+        </is>
+      </c>
+      <c r="L34" s="12" t="inlineStr">
+        <is>
+          <t>完成三文档一致性检查并等待 PR 合并</t>
         </is>
       </c>
     </row>
@@ -10932,7 +12074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11978,6 +13120,38 @@
       <c r="F34" s="12" t="inlineStr">
         <is>
           <t>并发回退不绕过幂等；Migration 指纹算法冻结；历史版本参数使用 tav_ 公共 ID；来源异常 fail-closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>DOC-V08</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Implementation Plan 最终定版审查</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>ADR/Specification/Plan/README/Excel 交叉检查</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>P-01～P-06 与 project scope 规则已纳入；Plan=Approved；Slice 1 仍受文档合并门禁</t>
         </is>
       </c>
     </row>
@@ -14726,7 +15900,7 @@
         </is>
       </c>
       <c r="F5" s="29" t="n">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="6" t="n"/>

</xml_diff>

<commit_message>
docs(evie-ai): finalize phase1 lifecycle contract
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -604,7 +604,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L34" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L36" headerRowCount="1">
   <autoFilter ref="A3:L24"/>
   <tableColumns count="12">
     <tableColumn id="1" name="任务ID"/>
@@ -656,7 +656,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F35" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F37" headerRowCount="1">
   <autoFilter ref="A3:F25"/>
   <tableColumns count="6">
     <tableColumn id="1" name="验证ID"/>
@@ -671,7 +671,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DecisionLedger" displayName="DecisionLedger" ref="A3:F26" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DecisionLedger" displayName="DecisionLedger" ref="A3:F42" headerRowCount="1">
   <autoFilter ref="A3:F14"/>
   <tableColumns count="6">
     <tableColumn id="1" name="决策ID"/>
@@ -686,7 +686,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Phase1Signoffs" displayName="Phase1Signoffs" ref="A3:F22" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Phase1Signoffs" displayName="Phase1Signoffs" ref="A3:F29" headerRowCount="1">
   <autoFilter ref="A3:F17"/>
   <tableColumns count="6">
     <tableColumn id="1" name="编号"/>
@@ -701,7 +701,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="FollowupLedger" displayName="FollowupLedger" ref="A3:G16" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="FollowupLedger" displayName="FollowupLedger" ref="A3:G17" headerRowCount="1">
   <autoFilter ref="A3:G14"/>
   <tableColumns count="7">
     <tableColumn id="1" name="编号"/>
@@ -742,7 +742,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N113" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EvieAiPhase1PlannedTests" displayName="EvieAiPhase1PlannedTests" ref="A1:N135" headerRowCount="1">
   <autoFilter ref="A1:N84"/>
   <tableColumns count="14">
     <tableColumn id="1" name="用例ID"/>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>3fb07fa（本轮 Plan 最终定版前 HEAD；修订待提交）</t>
+          <t>8c76784（A-11/P-09 最终文档同步前 HEAD；修订待提交）</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>• Implementation Plan 已纳入 P-01～P-06 并更新为 Approved；Phase 1 计划用例 112 条，Slice 1 仍待文档 PR 合并。</t>
+          <t>• A-11 已批准并同步：user_public_id=usr_&lt;uuid4hex32&gt;，P-01～P-09 已闭合；计划用例 134 条，Slice 1 仍待文档 PR 合并。</t>
         </is>
       </c>
       <c r="E19" s="22" t="n"/>
@@ -1376,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N113"/>
+  <dimension ref="A1:N135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9531,6 +9531,1590 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-113</t>
+        </is>
+      </c>
+      <c r="B114" s="29" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="C114" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D114" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E114" s="29" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="F114" s="29" t="inlineStr">
+        <is>
+          <t>v1 canonical JSON 固定测试向量</t>
+        </is>
+      </c>
+      <c r="G114" s="29" t="inlineStr">
+        <is>
+          <t>固定各 operation 的请求语义输入</t>
+        </is>
+      </c>
+      <c r="H114" s="29" t="inlineStr">
+        <is>
+          <t>计算 request fingerprint</t>
+        </is>
+      </c>
+      <c r="I114" s="29" t="inlineStr">
+        <is>
+          <t>输出与冻结 SHA-256 测试向量一致</t>
+        </is>
+      </c>
+      <c r="J114" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K114" s="29" t="inlineStr">
+        <is>
+          <t>单元</t>
+        </is>
+      </c>
+      <c r="L114" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="M114" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-07</t>
+        </is>
+      </c>
+      <c r="N114" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-114</t>
+        </is>
+      </c>
+      <c r="B115" s="29" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="C115" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D115" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E115" s="29" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="F115" s="29" t="inlineStr">
+        <is>
+          <t>字典顺序和进程重启不改变请求指纹</t>
+        </is>
+      </c>
+      <c r="G115" s="29" t="inlineStr">
+        <is>
+          <t>相同业务字段使用不同字典顺序并跨进程执行</t>
+        </is>
+      </c>
+      <c r="H115" s="29" t="inlineStr">
+        <is>
+          <t>计算 request fingerprint</t>
+        </is>
+      </c>
+      <c r="I115" s="29" t="inlineStr">
+        <is>
+          <t>所有结果完全一致</t>
+        </is>
+      </c>
+      <c r="J115" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/跨进程</t>
+        </is>
+      </c>
+      <c r="K115" s="29" t="inlineStr">
+        <is>
+          <t>单元</t>
+        </is>
+      </c>
+      <c r="L115" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="M115" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-07</t>
+        </is>
+      </c>
+      <c r="N115" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-115</t>
+        </is>
+      </c>
+      <c r="B116" s="29" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="C116" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D116" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E116" s="29" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="F116" s="29" t="inlineStr">
+        <is>
+          <t>逐操作字段纳入与排除合同</t>
+        </is>
+      </c>
+      <c r="G116" s="29" t="inlineStr">
+        <is>
+          <t>覆盖六种 operation 且改变 scope/追踪字段</t>
+        </is>
+      </c>
+      <c r="H116" s="29" t="inlineStr">
+        <is>
+          <t>比较 request fingerprint</t>
+        </is>
+      </c>
+      <c r="I116" s="29" t="inlineStr">
+        <is>
+          <t>业务语义字段改变则不同；project/actor/channel/key/request_id/time 改变不影响</t>
+        </is>
+      </c>
+      <c r="J116" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K116" s="29" t="inlineStr">
+        <is>
+          <t>参数化单元</t>
+        </is>
+      </c>
+      <c r="L116" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="M116" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-07</t>
+        </is>
+      </c>
+      <c r="N116" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-116</t>
+        </is>
+      </c>
+      <c r="B117" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2</t>
+        </is>
+      </c>
+      <c r="C117" s="29" t="inlineStr">
+        <is>
+          <t>Schema边界</t>
+        </is>
+      </c>
+      <c r="D117" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E117" s="29" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="F117" s="29" t="inlineStr">
+        <is>
+          <t>客户端不能提交 request_fingerprint</t>
+        </is>
+      </c>
+      <c r="G117" s="29" t="inlineStr">
+        <is>
+          <t>向所有公开写 Schema 注入 request_fingerprint</t>
+        </is>
+      </c>
+      <c r="H117" s="29" t="inlineStr">
+        <is>
+          <t>执行 Pydantic 校验</t>
+        </is>
+      </c>
+      <c r="I117" s="29" t="inlineStr">
+        <is>
+          <t>字段被拒绝或忽略策略符合显式禁止合同，不进入 Service</t>
+        </is>
+      </c>
+      <c r="J117" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K117" s="29" t="inlineStr">
+        <is>
+          <t>单元</t>
+        </is>
+      </c>
+      <c r="L117" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="M117" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-07</t>
+        </is>
+      </c>
+      <c r="N117" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-117</t>
+        </is>
+      </c>
+      <c r="B118" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3</t>
+        </is>
+      </c>
+      <c r="C118" s="29" t="inlineStr">
+        <is>
+          <t>幂等历史</t>
+        </is>
+      </c>
+      <c r="D118" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E118" s="29" t="inlineStr">
+        <is>
+          <t>P-08</t>
+        </is>
+      </c>
+      <c r="F118" s="29" t="inlineStr">
+        <is>
+          <t>Review/Audit 不强 FK 到可重用幂等行</t>
+        </is>
+      </c>
+      <c r="G118" s="29" t="inlineStr">
+        <is>
+          <t>反射模型与 Migration FK</t>
+        </is>
+      </c>
+      <c r="H118" s="29" t="inlineStr">
+        <is>
+          <t>检查关联结构</t>
+        </is>
+      </c>
+      <c r="I118" s="29" t="inlineStr">
+        <is>
+          <t>无指向 idempotency record 的永久强 FK；存在四项快照字段</t>
+        </is>
+      </c>
+      <c r="J118" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K118" s="29" t="inlineStr">
+        <is>
+          <t>结构</t>
+        </is>
+      </c>
+      <c r="L118" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="M118" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-08</t>
+        </is>
+      </c>
+      <c r="N118" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-118</t>
+        </is>
+      </c>
+      <c r="B119" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6/7</t>
+        </is>
+      </c>
+      <c r="C119" s="29" t="inlineStr">
+        <is>
+          <t>幂等历史</t>
+        </is>
+      </c>
+      <c r="D119" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E119" s="29" t="inlineStr">
+        <is>
+          <t>P-08</t>
+        </is>
+      </c>
+      <c r="F119" s="29" t="inlineStr">
+        <is>
+          <t>幂等快照与领域历史同事务写入且不保存原始 key</t>
+        </is>
+      </c>
+      <c r="G119" s="29" t="inlineStr">
+        <is>
+          <t>执行审核及审计写入</t>
+        </is>
+      </c>
+      <c r="H119" s="29" t="inlineStr">
+        <is>
+          <t>读取 Review/Audit</t>
+        </is>
+      </c>
+      <c r="I119" s="29" t="inlineStr">
+        <is>
+          <t>保存 operation/scope hash/key hash/generation；无原始 Idempotency-Key</t>
+        </is>
+      </c>
+      <c r="J119" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K119" s="29" t="inlineStr">
+        <is>
+          <t>服务集成</t>
+        </is>
+      </c>
+      <c r="L119" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_idempotency_history.py</t>
+        </is>
+      </c>
+      <c r="M119" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-08</t>
+        </is>
+      </c>
+      <c r="N119" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-119</t>
+        </is>
+      </c>
+      <c r="B120" s="29" t="inlineStr">
+        <is>
+          <t>Slice 4/7</t>
+        </is>
+      </c>
+      <c r="C120" s="29" t="inlineStr">
+        <is>
+          <t>幂等历史</t>
+        </is>
+      </c>
+      <c r="D120" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E120" s="29" t="inlineStr">
+        <is>
+          <t>P-08</t>
+        </is>
+      </c>
+      <c r="F120" s="29" t="inlineStr">
+        <is>
+          <t>过期重用新 generation 不改变历史归属</t>
+        </is>
+      </c>
+      <c r="G120" s="29" t="inlineStr">
+        <is>
+          <t>完成操作后使幂等记录过期并以同 key 新 generation 重用</t>
+        </is>
+      </c>
+      <c r="H120" s="29" t="inlineStr">
+        <is>
+          <t>比较重用前后 Review/Audit</t>
+        </is>
+      </c>
+      <c r="I120" s="29" t="inlineStr">
+        <is>
+          <t>既有快照保持原 operation/hash/generation</t>
+        </is>
+      </c>
+      <c r="J120" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K120" s="29" t="inlineStr">
+        <is>
+          <t>数据库集成</t>
+        </is>
+      </c>
+      <c r="L120" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_idempotency_history.py</t>
+        </is>
+      </c>
+      <c r="M120" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-08</t>
+        </is>
+      </c>
+      <c r="N120" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-120</t>
+        </is>
+      </c>
+      <c r="B121" s="29" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C121" s="29" t="inlineStr">
+        <is>
+          <t>Audit双事件</t>
+        </is>
+      </c>
+      <c r="D121" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E121" s="29" t="inlineStr">
+        <is>
+          <t>P-06/P-08</t>
+        </is>
+      </c>
+      <c r="F121" s="29" t="inlineStr">
+        <is>
+          <t>双审计事件共享幂等快照但 ID 独立</t>
+        </is>
+      </c>
+      <c r="G121" s="29" t="inlineStr">
+        <is>
+          <t>重复复用并新增来源</t>
+        </is>
+      </c>
+      <c r="H121" s="29" t="inlineStr">
+        <is>
+          <t>读取两个 AuditEvent</t>
+        </is>
+      </c>
+      <c r="I121" s="29" t="inlineStr">
+        <is>
+          <t>四项幂等快照一致，audit_event_id 各自唯一</t>
+        </is>
+      </c>
+      <c r="J121" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K121" s="29" t="inlineStr">
+        <is>
+          <t>服务集成</t>
+        </is>
+      </c>
+      <c r="L121" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_audit_events.py</t>
+        </is>
+      </c>
+      <c r="M121" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-06/P-08</t>
+        </is>
+      </c>
+      <c r="N121" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-121</t>
+        </is>
+      </c>
+      <c r="B122" s="29" t="inlineStr">
+        <is>
+          <t>Slice 5/8</t>
+        </is>
+      </c>
+      <c r="C122" s="29" t="inlineStr">
+        <is>
+          <t>授权防枚举</t>
+        </is>
+      </c>
+      <c r="D122" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E122" s="29" t="inlineStr">
+        <is>
+          <t>P-09/A-02</t>
+        </is>
+      </c>
+      <c r="F122" s="29" t="inlineStr">
+        <is>
+          <t>先校验全局 admin 再查询项目</t>
+        </is>
+      </c>
+      <c r="G122" s="29" t="inlineStr">
+        <is>
+          <t>非 admin 请求存在/不存在/非 active 项目</t>
+        </is>
+      </c>
+      <c r="H122" s="29" t="inlineStr">
+        <is>
+          <t>调用所有 EvieAi API</t>
+        </is>
+      </c>
+      <c r="I122" s="29" t="inlineStr">
+        <is>
+          <t>均返回 403 EVIE_PROJECT_SCOPE_FORBIDDEN，不泄露项目状态</t>
+        </is>
+      </c>
+      <c r="J122" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K122" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L122" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_api_scope.py</t>
+        </is>
+      </c>
+      <c r="M122" s="29" t="inlineStr">
+        <is>
+          <t>Plan P-09</t>
+        </is>
+      </c>
+      <c r="N122" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-122</t>
+        </is>
+      </c>
+      <c r="B123" s="29" t="inlineStr">
+        <is>
+          <t>Slice 5</t>
+        </is>
+      </c>
+      <c r="C123" s="29" t="inlineStr">
+        <is>
+          <t>Actor identity</t>
+        </is>
+      </c>
+      <c r="D123" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E123" s="29" t="inlineStr">
+        <is>
+          <t>P-09</t>
+        </is>
+      </c>
+      <c r="F123" s="29" t="inlineStr">
+        <is>
+          <t>RequestActorContext 使用批准的稳定身份字段</t>
+        </is>
+      </c>
+      <c r="G123" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准，认证 principal 提供合法 user_public_id</t>
+        </is>
+      </c>
+      <c r="H123" s="29" t="inlineStr">
+        <is>
+          <t>生成 actor identity</t>
+        </is>
+      </c>
+      <c r="I123" s="29" t="inlineStr">
+        <is>
+          <t>严格为 user:&lt;user_public_id&gt;，不使用可变/临时/内部字段</t>
+        </is>
+      </c>
+      <c r="J123" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/认证集成</t>
+        </is>
+      </c>
+      <c r="K123" s="29" t="inlineStr">
+        <is>
+          <t>单元+集成</t>
+        </is>
+      </c>
+      <c r="L123" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_actor_context.py</t>
+        </is>
+      </c>
+      <c r="M123" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准；文档 PR 合并后实施</t>
+        </is>
+      </c>
+      <c r="N123" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-123</t>
+        </is>
+      </c>
+      <c r="B124" s="29" t="inlineStr">
+        <is>
+          <t>Slice 0</t>
+        </is>
+      </c>
+      <c r="C124" s="29" t="inlineStr">
+        <is>
+          <t>文档架构守卫</t>
+        </is>
+      </c>
+      <c r="D124" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E124" s="29" t="inlineStr">
+        <is>
+          <t>C-04</t>
+        </is>
+      </c>
+      <c r="F124" s="29" t="inlineStr">
+        <is>
+          <t>唯一当前阶段权威声明</t>
+        </is>
+      </c>
+      <c r="G124" s="29" t="inlineStr">
+        <is>
+          <t>扫描 EvieAi 权威文档阶段标记与链接</t>
+        </is>
+      </c>
+      <c r="H124" s="29" t="inlineStr">
+        <is>
+          <t>校验 current/frozen historical 状态</t>
+        </is>
+      </c>
+      <c r="I124" s="29" t="inlineStr">
+        <is>
+          <t>仅 Phase 1 文档声明当前阶段；Phase 0 明确为冻结历史基线且链接阶段矩阵</t>
+        </is>
+      </c>
+      <c r="J124" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K124" s="29" t="inlineStr">
+        <is>
+          <t>静态文档</t>
+        </is>
+      </c>
+      <c r="L124" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_document_authority.py</t>
+        </is>
+      </c>
+      <c r="M124" s="29" t="inlineStr">
+        <is>
+          <t>C-04 已关闭</t>
+        </is>
+      </c>
+      <c r="N124" s="29" t="inlineStr">
+        <is>
+          <t>计划自动化守卫，防止后续阶段声明再次漂移。</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-124</t>
+        </is>
+      </c>
+      <c r="B125" s="29" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="C125" s="29" t="inlineStr">
+        <is>
+          <t>User ID</t>
+        </is>
+      </c>
+      <c r="D125" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E125" s="29" t="inlineStr">
+        <is>
+          <t>A-11/P-09</t>
+        </is>
+      </c>
+      <c r="F125" s="29" t="inlineStr">
+        <is>
+          <t>usr_ 公共 ID 格式与唯一性</t>
+        </is>
+      </c>
+      <c r="G125" s="29" t="inlineStr">
+        <is>
+          <t>固定 uuid4 并批量生成 1000 个 ID</t>
+        </is>
+      </c>
+      <c r="H125" s="29" t="inlineStr">
+        <is>
+          <t>调用统一 ID generator</t>
+        </is>
+      </c>
+      <c r="I125" s="29" t="inlineStr">
+        <is>
+          <t>格式严格 usr_&lt;32位小写hex&gt; 且批量无重复</t>
+        </is>
+      </c>
+      <c r="J125" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="K125" s="29" t="inlineStr">
+        <is>
+          <t>单元</t>
+        </is>
+      </c>
+      <c r="L125" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py</t>
+        </is>
+      </c>
+      <c r="M125" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准</t>
+        </is>
+      </c>
+      <c r="N125" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-125</t>
+        </is>
+      </c>
+      <c r="B126" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3</t>
+        </is>
+      </c>
+      <c r="C126" s="29" t="inlineStr">
+        <is>
+          <t>User ORM</t>
+        </is>
+      </c>
+      <c r="D126" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E126" s="29" t="inlineStr">
+        <is>
+          <t>A-11/P-01</t>
+        </is>
+      </c>
+      <c r="F126" s="29" t="inlineStr">
+        <is>
+          <t>User.user_public_id ORM 与数据库约束</t>
+        </is>
+      </c>
+      <c r="G126" s="29" t="inlineStr">
+        <is>
+          <t>反射 User 模型和迁移后结构</t>
+        </is>
+      </c>
+      <c r="H126" s="29" t="inlineStr">
+        <is>
+          <t>检查字段/nullable/unique</t>
+        </is>
+      </c>
+      <c r="I126" s="29" t="inlineStr">
+        <is>
+          <t>字段最终 NOT NULL、全局 UNIQUE、内部 id 仍为 Integer PK</t>
+        </is>
+      </c>
+      <c r="J126" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K126" s="29" t="inlineStr">
+        <is>
+          <t>结构</t>
+        </is>
+      </c>
+      <c r="L126" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_identity.py</t>
+        </is>
+      </c>
+      <c r="M126" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 原子 PR</t>
+        </is>
+      </c>
+      <c r="N126" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-126</t>
+        </is>
+      </c>
+      <c r="B127" s="29" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="C127" s="29" t="inlineStr">
+        <is>
+          <t>User Migration</t>
+        </is>
+      </c>
+      <c r="D127" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E127" s="29" t="inlineStr">
+        <is>
+          <t>A-11/D-13</t>
+        </is>
+      </c>
+      <c r="F127" s="29" t="inlineStr">
+        <is>
+          <t>SQLite 存量用户无损回填</t>
+        </is>
+      </c>
+      <c r="G127" s="29" t="inlineStr">
+        <is>
+          <t>121000 SQLite 含多名存量用户</t>
+        </is>
+      </c>
+      <c r="H127" s="29" t="inlineStr">
+        <is>
+          <t>upgrade 到 Phase 1 head</t>
+        </is>
+      </c>
+      <c r="I127" s="29" t="inlineStr">
+        <is>
+          <t>每名用户获得唯一合法 usr_ ID，旧认证字段和记录不变</t>
+        </is>
+      </c>
+      <c r="J127" s="29" t="inlineStr">
+        <is>
+          <t>SQLite foreign_keys=ON</t>
+        </is>
+      </c>
+      <c r="K127" s="29" t="inlineStr">
+        <is>
+          <t>Migration集成</t>
+        </is>
+      </c>
+      <c r="L127" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_user_identity_migration.py</t>
+        </is>
+      </c>
+      <c r="M127" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 原子 PR</t>
+        </is>
+      </c>
+      <c r="N127" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-127</t>
+        </is>
+      </c>
+      <c r="B128" s="29" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="C128" s="29" t="inlineStr">
+        <is>
+          <t>User Migration</t>
+        </is>
+      </c>
+      <c r="D128" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E128" s="29" t="inlineStr">
+        <is>
+          <t>A-11/D-13</t>
+        </is>
+      </c>
+      <c r="F128" s="29" t="inlineStr">
+        <is>
+          <t>PostgreSQL 存量用户无损回填</t>
+        </is>
+      </c>
+      <c r="G128" s="29" t="inlineStr">
+        <is>
+          <t>121000 PostgreSQL 含多名存量用户</t>
+        </is>
+      </c>
+      <c r="H128" s="29" t="inlineStr">
+        <is>
+          <t>upgrade 到 Phase 1 head</t>
+        </is>
+      </c>
+      <c r="I128" s="29" t="inlineStr">
+        <is>
+          <t>每名用户获得唯一合法 usr_ ID，NOT NULL/UNIQUE 生效</t>
+        </is>
+      </c>
+      <c r="J128" s="29" t="inlineStr">
+        <is>
+          <t>PostgreSQL 16</t>
+        </is>
+      </c>
+      <c r="K128" s="29" t="inlineStr">
+        <is>
+          <t>Migration集成</t>
+        </is>
+      </c>
+      <c r="L128" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_user_identity_migration.py</t>
+        </is>
+      </c>
+      <c r="M128" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 原子 PR</t>
+        </is>
+      </c>
+      <c r="N128" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-128</t>
+        </is>
+      </c>
+      <c r="B129" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/5</t>
+        </is>
+      </c>
+      <c r="C129" s="29" t="inlineStr">
+        <is>
+          <t>User创建</t>
+        </is>
+      </c>
+      <c r="D129" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E129" s="29" t="inlineStr">
+        <is>
+          <t>A-11</t>
+        </is>
+      </c>
+      <c r="F129" s="29" t="inlineStr">
+        <is>
+          <t>新用户自动生成公共 ID</t>
+        </is>
+      </c>
+      <c r="G129" s="29" t="inlineStr">
+        <is>
+          <t>通过现有受支持用户创建路径创建用户</t>
+        </is>
+      </c>
+      <c r="H129" s="29" t="inlineStr">
+        <is>
+          <t>读取 principal/User</t>
+        </is>
+      </c>
+      <c r="I129" s="29" t="inlineStr">
+        <is>
+          <t>服务端生成唯一合法 user_public_id，客户端不能控制</t>
+        </is>
+      </c>
+      <c r="J129" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K129" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L129" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_user_identity.py</t>
+        </is>
+      </c>
+      <c r="M129" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准</t>
+        </is>
+      </c>
+      <c r="N129" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-129</t>
+        </is>
+      </c>
+      <c r="B130" s="29" t="inlineStr">
+        <is>
+          <t>Slice 5</t>
+        </is>
+      </c>
+      <c r="C130" s="29" t="inlineStr">
+        <is>
+          <t>Actor稳定性</t>
+        </is>
+      </c>
+      <c r="D130" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E130" s="29" t="inlineStr">
+        <is>
+          <t>A-11/P-09</t>
+        </is>
+      </c>
+      <c r="F130" s="29" t="inlineStr">
+        <is>
+          <t>username 修改不改变 actor 身份</t>
+        </is>
+      </c>
+      <c r="G130" s="29" t="inlineStr">
+        <is>
+          <t>已有 user_public_id 的用户先后修改 username</t>
+        </is>
+      </c>
+      <c r="H130" s="29" t="inlineStr">
+        <is>
+          <t>两次生成 RequestActorContext</t>
+        </is>
+      </c>
+      <c r="I130" s="29" t="inlineStr">
+        <is>
+          <t>两次均为相同 user:&lt;user_public_id&gt;</t>
+        </is>
+      </c>
+      <c r="J130" s="29" t="inlineStr">
+        <is>
+          <t>认证集成</t>
+        </is>
+      </c>
+      <c r="K130" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L130" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_actor_identity.py</t>
+        </is>
+      </c>
+      <c r="M130" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准</t>
+        </is>
+      </c>
+      <c r="N130" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-130</t>
+        </is>
+      </c>
+      <c r="B131" s="29" t="inlineStr">
+        <is>
+          <t>Slice 5</t>
+        </is>
+      </c>
+      <c r="C131" s="29" t="inlineStr">
+        <is>
+          <t>JWT兼容</t>
+        </is>
+      </c>
+      <c r="D131" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E131" s="29" t="inlineStr">
+        <is>
+          <t>A-11/P-09</t>
+        </is>
+      </c>
+      <c r="F131" s="29" t="inlineStr">
+        <is>
+          <t>现有 JWT sub 继续认证并暴露公共 ID</t>
+        </is>
+      </c>
+      <c r="G131" s="29" t="inlineStr">
+        <is>
+          <t>使用 sub=内部 User.id 的现有 token</t>
+        </is>
+      </c>
+      <c r="H131" s="29" t="inlineStr">
+        <is>
+          <t>执行认证解析</t>
+        </is>
+      </c>
+      <c r="I131" s="29" t="inlineStr">
+        <is>
+          <t>认证成功；principal 同时提供合法 user_public_id；token 无需改版</t>
+        </is>
+      </c>
+      <c r="J131" s="29" t="inlineStr">
+        <is>
+          <t>认证集成</t>
+        </is>
+      </c>
+      <c r="K131" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L131" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_auth_compatibility.py</t>
+        </is>
+      </c>
+      <c r="M131" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准</t>
+        </is>
+      </c>
+      <c r="N131" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-131</t>
+        </is>
+      </c>
+      <c r="B132" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/6/7/8</t>
+        </is>
+      </c>
+      <c r="C132" s="29" t="inlineStr">
+        <is>
+          <t>隐私边界</t>
+        </is>
+      </c>
+      <c r="D132" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E132" s="29" t="inlineStr">
+        <is>
+          <t>A-11/P-08</t>
+        </is>
+      </c>
+      <c r="F132" s="29" t="inlineStr">
+        <is>
+          <t>API 与历史事实不暴露内部 User.id</t>
+        </is>
+      </c>
+      <c r="G132" s="29" t="inlineStr">
+        <is>
+          <t>执行 Source/Review/Audit/幂等写入并查询 API</t>
+        </is>
+      </c>
+      <c r="H132" s="29" t="inlineStr">
+        <is>
+          <t>检查持久化和响应</t>
+        </is>
+      </c>
+      <c r="I132" s="29" t="inlineStr">
+        <is>
+          <t>仅保存/返回 user:&lt;user_public_id&gt; 快照，无内部 User.id</t>
+        </is>
+      </c>
+      <c r="J132" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL/API</t>
+        </is>
+      </c>
+      <c r="K132" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L132" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_actor_identity.py</t>
+        </is>
+      </c>
+      <c r="M132" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准</t>
+        </is>
+      </c>
+      <c r="N132" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-132</t>
+        </is>
+      </c>
+      <c r="B133" s="29" t="inlineStr">
+        <is>
+          <t>Slice 5/8</t>
+        </is>
+      </c>
+      <c r="C133" s="29" t="inlineStr">
+        <is>
+          <t>Actor防伪</t>
+        </is>
+      </c>
+      <c r="D133" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E133" s="29" t="inlineStr">
+        <is>
+          <t>A-11/P-09</t>
+        </is>
+      </c>
+      <c r="F133" s="29" t="inlineStr">
+        <is>
+          <t>请求正文不能伪造 actor且缺失公共 ID fail-closed</t>
+        </is>
+      </c>
+      <c r="G133" s="29" t="inlineStr">
+        <is>
+          <t>提交 actor 覆盖字段；构造缺失/非法 user_public_id principal</t>
+        </is>
+      </c>
+      <c r="H133" s="29" t="inlineStr">
+        <is>
+          <t>调用写 API</t>
+        </is>
+      </c>
+      <c r="I133" s="29" t="inlineStr">
+        <is>
+          <t>覆盖字段被拒绝；缺失/非法身份明确拒绝且不回退</t>
+        </is>
+      </c>
+      <c r="J133" s="29" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="K133" s="29" t="inlineStr">
+        <is>
+          <t>集成</t>
+        </is>
+      </c>
+      <c r="L133" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_actor_identity.py</t>
+        </is>
+      </c>
+      <c r="M133" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准</t>
+        </is>
+      </c>
+      <c r="N133" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-133</t>
+        </is>
+      </c>
+      <c r="B134" s="29" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="C134" s="29" t="inlineStr">
+        <is>
+          <t>Downgrade保护</t>
+        </is>
+      </c>
+      <c r="D134" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E134" s="29" t="inlineStr">
+        <is>
+          <t>A-11/A-05/D-13</t>
+        </is>
+      </c>
+      <c r="F134" s="29" t="inlineStr">
+        <is>
+          <t>用户公共身份 downgrade fail-closed</t>
+        </is>
+      </c>
+      <c r="G134" s="29" t="inlineStr">
+        <is>
+          <t>数据库存在 User 或公共 actor 历史事实</t>
+        </is>
+      </c>
+      <c r="H134" s="29" t="inlineStr">
+        <is>
+          <t>尝试 downgrade 到无法表达 user_public_id 的 revision</t>
+        </is>
+      </c>
+      <c r="I134" s="29" t="inlineStr">
+        <is>
+          <t>明确拒绝，结构和数据不变；空库无身份事实路径按合同验证</t>
+        </is>
+      </c>
+      <c r="J134" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K134" s="29" t="inlineStr">
+        <is>
+          <t>Migration集成</t>
+        </is>
+      </c>
+      <c r="L134" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_user_identity_migration.py</t>
+        </is>
+      </c>
+      <c r="M134" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 原子 PR</t>
+        </is>
+      </c>
+      <c r="N134" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-PLAN-134</t>
+        </is>
+      </c>
+      <c r="B135" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/5</t>
+        </is>
+      </c>
+      <c r="C135" s="29" t="inlineStr">
+        <is>
+          <t>User identity immutability</t>
+        </is>
+      </c>
+      <c r="D135" s="35" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+      <c r="E135" s="29" t="inlineStr">
+        <is>
+          <t>A-11</t>
+        </is>
+      </c>
+      <c r="F135" s="29" t="inlineStr">
+        <is>
+          <t>user_public_id 创建后不可修改</t>
+        </is>
+      </c>
+      <c r="G135" s="29" t="inlineStr">
+        <is>
+          <t>已有合法公共 ID 的用户</t>
+        </is>
+      </c>
+      <c r="H135" s="29" t="inlineStr">
+        <is>
+          <t>尝试经 Schema/Service 修改公共 ID并执行 username/role/status 更新</t>
+        </is>
+      </c>
+      <c r="I135" s="29" t="inlineStr">
+        <is>
+          <t>公共 ID 修改请求被拒绝；其他用户字段变化后 user_public_id 保持不变</t>
+        </is>
+      </c>
+      <c r="J135" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL/API</t>
+        </is>
+      </c>
+      <c r="K135" s="29" t="inlineStr">
+        <is>
+          <t>单元+集成</t>
+        </is>
+      </c>
+      <c r="L135" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/integration/evie_ai/test_evie_ai_user_identity.py</t>
+        </is>
+      </c>
+      <c r="M135" s="29" t="inlineStr">
+        <is>
+          <t>A-11 已批准</t>
+        </is>
+      </c>
+      <c r="N135" s="29" t="inlineStr">
+        <is>
+          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9546,7 +11130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11558,6 +13142,130 @@
       <c r="L34" s="12" t="inlineStr">
         <is>
           <t>完成三文档一致性检查并等待 PR 合并</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>DOC-09</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 最终实施澄清</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>纳入 P-07～P-09 并关闭 C-04</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>冻结请求指纹和幂等快照语义，核验认证 principal 稳定身份，消除阶段文档漂移</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>计划补入 P-07/P-08；只读核验 User/JWT/auth 后记录 P-09 身份合同阻塞；Phase 0 文档标记历史冻结基线</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Implementation Plan、README、Architecture Baseline、Phase 0 历史基线、Excel 测试台账</t>
+        </is>
+      </c>
+      <c r="H35" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>P-07/P-08/C-04 已闭合；A-11 已批准并关闭 P-09</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>仅 docs/evie-ai；未修改认证模型、ORM、Migration、Service、API 或数据库</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
+        <is>
+          <t>docs/evie-ai-phase1-lifecycle / PR #5</t>
+        </is>
+      </c>
+      <c r="L35" s="12" t="inlineStr">
+        <is>
+          <t>提交并合并 Slice 0 文档 PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>DOC-10</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 身份合同签字</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>批准并同步 A-11 用户稳定公共身份</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>为 actor、Source、Review、Audit 和幂等作用域建立不可变公共用户身份</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>固定 user_public_id=usr_&lt;uuid4hex32&gt;；JWT sub 保持内部 ID；同步 ORM/Migration/Policy/principal 切片及测试合同</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>AGENTS、ADR、Specification、Implementation Plan、阶段追踪、Excel</t>
+        </is>
+      </c>
+      <c r="H36" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>A-01～A-11 Accepted；P-01～P-09 已闭合；Plan=Approved</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>仅文档和测试台账；未修改 User ORM、Migration、JWT、Service、API 或数据库</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>用户 2026-07-15 明确确认 / PR #5</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>审查并合并文档 PR 后从最新 dev 创建 Slice 1 分支</t>
         </is>
       </c>
     </row>
@@ -12074,7 +13782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13152,6 +14860,70 @@
       <c r="F35" s="12" t="inlineStr">
         <is>
           <t>P-01～P-06 与 project scope 规则已纳入；Plan=Approved；Slice 1 仍受文档合并门禁</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>DOC-V09</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>P-07～P-09 与 C-04 实施澄清审查</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Plan/README/Baseline/Phase0 文档、User 模型、JWT principal 与 Excel 交叉核验</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>passed; A-11 approved</t>
+        </is>
+      </c>
+      <c r="E36" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>缺口已由 A-11 正式闭合；未退化使用内部 PK 或可变 username</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>DOC-V10</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>A-11 身份合同一致性审查</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>AGENTS/ADR/Specification/Plan/README/Baseline/Traceability/Excel 交叉检查</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>usr_ ID、JWT 兼容、actor 快照、双数据库回填和 downgrade 保护已形成一致实施合同</t>
         </is>
       </c>
     </row>
@@ -13183,7 +14955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14357,6 +16129,134 @@
       <c r="F38" s="12" t="inlineStr">
         <is>
           <t>实施不得自行改变</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>请求指纹</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>按 operation_type 使用 v1 canonical JSON + UTF-8 + SHA-256；客户端不得提交</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>已纳入计划</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>Implementation Plan P-07</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>固定测试向量；不得混入幂等 scope 和追踪字段</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>P-08</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>幂等关联快照</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Review/Audit 保存 operation/scope hash/key hash/generation 快照，不强 FK 到可重用幂等行</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>已纳入计划</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>Implementation Plan P-08</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>不保存原始 Idempotency-Key；历史归属不可随 generation 改变</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>P-09</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>认证主体稳定身份</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>A-11 批准 user_public_id=usr_&lt;uuid4hex32&gt;；actor=user:&lt;user_public_id&gt;；JWT sub 保持内部 ID</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>已闭合</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>A-11 / Implementation Plan P-09</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>缺失或非法公共 ID fail-closed；不得退化使用其他字段</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>A-11</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>用户稳定公共身份</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>User.user_public_id 全局唯一且不可修改；actor 固定 user:&lt;user_public_id&gt;；存量线性迁移回填</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="inlineStr">
+        <is>
+          <t>已批准</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>ADR-0001 / 规格合同</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>内部 User.id 不作为 actor；JWT sub 兼容保留；公共身份历史快照不可重写</t>
         </is>
       </c>
     </row>
@@ -14388,7 +16288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15208,6 +17108,70 @@
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15 用户明确签字</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>P-09</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>认证主体稳定身份合同修订</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>由 A-11 固定 user_public_id、JWT 兼容和 actor 规范化合同</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>已闭合</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>实施阻塞已解除</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15 用户明确批准 A-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>A-11</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>用户稳定公共身份合同</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>user_public_id=usr_&lt;uuid4hex32&gt;；actor=user:&lt;user_public_id&gt;；存量回填；JWT sub 兼容</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>已批准</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>合同阻塞已解除</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>2026-07-15 用户明确签字</t>
         </is>
@@ -15241,7 +17205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15544,12 +17508,12 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>权威规格批准后更新“当前阶段 Phase 0”描述</t>
+          <t>Phase 0 文档已标记为冻结历史基线并链接当前 Phase 1 阶段矩阵</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
@@ -15559,7 +17523,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>不得在签字前提前改写</t>
+          <t>不得修改 Phase 0 冻结架构规则</t>
         </is>
       </c>
     </row>
@@ -15782,6 +17746,43 @@
       <c r="G16" s="12" t="inlineStr">
         <is>
           <t>后续门禁为文档提交/审查/合并</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>NEXT-14</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>完成 P-09 认证主体稳定身份合同修订</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>A-11 已批准并同步 ADR/Specification/Plan/测试台账</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>用户 2026-07-15 明确确认 A-11</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>下一门禁为文档 PR 合并，不授权在 docs 分支实施代码</t>
         </is>
       </c>
     </row>
@@ -15813,7 +17814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -15900,7 +17901,7 @@
         </is>
       </c>
       <c r="F5" s="29" t="n">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="6" t="n"/>
@@ -16196,6 +18197,13 @@
       <c r="A28" s="32" t="inlineStr">
         <is>
           <t>5. Candidate、structurer、Compiler、Runner 不得进入 EvieAi 自然语言资产测试事实源。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>6. A-11 已签字；P-09 计划用例解除合同阻塞，但仍须等待 Slice 0 文档 PR 合并后实施。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(evie-ai): close phase1 slice0
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -604,7 +604,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L36" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskLedger" displayName="TaskLedger" ref="A3:L37" headerRowCount="1">
   <autoFilter ref="A3:L24"/>
   <tableColumns count="12">
     <tableColumn id="1" name="任务ID"/>
@@ -656,7 +656,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F37" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F38" headerRowCount="1">
   <autoFilter ref="A3:F25"/>
   <tableColumns count="6">
     <tableColumn id="1" name="验证ID"/>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>docs/evie-ai-phase1-lifecycle</t>
+          <t>codex/evie-ai-phase1-slice0-closeout</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>8c76784（A-11/P-09 最终文档同步前 HEAD；修订待提交）</t>
+          <t>adb2b2b（PR #5 合并后的 dev 基线；closeout 修订待提交）</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>• A-11 已批准并同步：user_public_id=usr_&lt;uuid4hex32&gt;，P-01～P-09 已闭合；计划用例 134 条，Slice 1 仍待文档 PR 合并。</t>
+          <t>• A-01～A-11 与 P-01～P-09 已闭合；PR #5 已合并到 dev@adb2b2b；计划用例 134 条，Slice 1 允许启动。</t>
         </is>
       </c>
       <c r="E19" s="22" t="n"/>
@@ -11130,7 +11130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13266,6 +13266,68 @@
       <c r="L36" s="12" t="inlineStr">
         <is>
           <t>审查并合并文档 PR 后从最新 dev 创建 Slice 1 分支</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>DOC-11</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>Slice 0 收口</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>PR #5 合并后阶段状态收口</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>消除文档仍声称待合并的状态漂移</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>将 README/Baseline/Specification/Plan/Traceability 更新为 PR #5 已合并并允许 Slice 1</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>5 份权威状态文档与 Excel</t>
+        </is>
+      </c>
+      <c r="H37" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>dev@adb2b2b 已包含 Slice 0；Slice 1 启动门禁解除</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>仅状态收口；不修改合同、代码或数据库</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>codex/evie-ai-phase1-slice0-closeout</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>合并 closeout 后从最新 dev 创建 Slice 1 分支</t>
         </is>
       </c>
     </row>
@@ -13510,6 +13572,58 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>PR #5</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>docs(evie-ai): approve phase1 asset lifecycle contract</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>docs/evie-ai-phase1-lifecycle</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>已合并</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15 13:09:45 +08:00</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>adb2b2b</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>8 commits</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>ADR/Specification/Plan、A-11 用户身份合同、P-01～P-09、Excel 测试台账</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>https://github.com/Chloeqq/ai-test-platform/pull/5</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
@@ -13782,7 +13896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14924,6 +15038,38 @@
       <c r="F37" s="12" t="inlineStr">
         <is>
           <t>usr_ ID、JWT 兼容、actor 快照、双数据库回填和 downgrade 保护已形成一致实施合同</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>DOC-V11</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>PR #5 合并后状态一致性</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>dev@adb2b2b、PR #5 merged 状态与五份权威文档</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>不再存在“权威文档待合并”冲突；Slice 1 允许启动</t>
         </is>
       </c>
     </row>
@@ -17693,22 +17839,22 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>确认 diff、Excel 临时文件排除、提交并创建 docs PR</t>
+          <t>PR #5 已合并到 dev@adb2b2b；closeout 负责更新合并后状态</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>当前 docs 分支</t>
+          <t>PR #5 / adb2b2b</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>文档合并后再创建 Slice 1 功能分支</t>
+          <t>后续只允许按 Plan 从 Slice 1 开始</t>
         </is>
       </c>
     </row>
@@ -17854,7 +18000,7 @@
       </c>
       <c r="F3" s="29" t="inlineStr">
         <is>
-          <t>docs/evie-ai-phase1-lifecycle</t>
+          <t>codex/evie-ai-phase1-slice0-closeout</t>
         </is>
       </c>
       <c r="G3" s="5" t="n"/>
@@ -17914,7 +18060,7 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>dev@f5c8226</t>
+          <t>dev@adb2b2b</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>

</xml_diff>

<commit_message>
docs(evie-ai): update phase1 slice1 test ledger
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -21,12 +21,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任务明细'!$A$3:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Git与PR'!$A$8:$C$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'验证记录'!$A$3:$F$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'验证记录'!$A$3:$F$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'决策与约束'!$A$3:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Phase1签字项'!$A$3:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'后续事项'!$A$3:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'已实现测试用例'!$A$1:$P$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Phase1计划用例'!$A$1:$N$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'已实现测试用例'!$A$1:$P$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Phase1计划用例'!$A$1:$N$135</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -656,7 +656,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F38" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLedger" displayName="ValidationLedger" ref="A3:F42" headerRowCount="1">
   <autoFilter ref="A3:F25"/>
   <tableColumns count="6">
     <tableColumn id="1" name="验证ID"/>
@@ -717,7 +717,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="EvieAiImplementedTests" displayName="EvieAiImplementedTests" ref="A1:P78" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="EvieAiImplementedTests" displayName="EvieAiImplementedTests" ref="A1:P123" headerRowCount="1">
   <autoFilter ref="A1:P78"/>
   <tableColumns count="16">
     <tableColumn id="1" name="用例ID"/>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="D2" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E2" s="29" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="N2" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：tar_/tae_ 格式参数化节点；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D3" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E3" s="29" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="N3" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：tar_/tae_ 唯一性参数化节点；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="D4" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E4" s="29" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="N4" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_content_normalization_preserves_meaning_and_stabilizes_tags；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="D5" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E5" s="29" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="N5" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_content_normalization_preserves_meaning_and_stabilizes_tags；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="D6" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E6" s="29" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="N6" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_content_normalization_preserves_meaning_and_stabilizes_tags；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="D7" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E7" s="29" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="N7" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_content_normalization_preserves_meaning_and_stabilizes_tags；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="D8" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E8" s="29" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="N8" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_review_policy_allows_approved_transitions（4 nodes）；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="D9" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E9" s="29" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="N9" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_review_policy_rejects_invalid_or_unexplained_transitions（4 nodes）；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="D10" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E10" s="29" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="N10" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_idempotency_retention_defaults_to_seven_days；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="D11" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E11" s="29" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="N11" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_idempotency_retention_accepts_positive_environment_override；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="D12" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E12" s="29" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="N12" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_idempotency_retention_rejects_invalid_environment_values（3 nodes）；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="D13" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E13" s="29" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="N13" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_requirement_source_identity_matches_frozen_vector；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="D14" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E14" s="29" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="N14" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_manual_source_identity_changes_with_real_source_semantics；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="D15" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E15" s="29" t="inlineStr">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_asset_code_policy.py</t>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
         </is>
       </c>
       <c r="M15" s="29" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="N15" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_asset_code_for_new_asset_is_its_public_id / reject invalid；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="D85" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E85" s="29" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="N85" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：content frozen vector + canonical mapping order；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="D86" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E86" s="29" t="inlineStr">
@@ -7573,7 +7573,7 @@
       </c>
       <c r="L86" s="29" t="inlineStr">
         <is>
-          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_lifecycle_policy.py</t>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_constants.py</t>
         </is>
       </c>
       <c r="M86" s="29" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="N86" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_conversion_status_does_not_include_failed；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -8541,7 +8541,7 @@
       </c>
       <c r="D100" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E100" s="29" t="inlineStr">
@@ -8581,7 +8581,7 @@
       </c>
       <c r="L100" s="29" t="inlineStr">
         <is>
-          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_idempotency_policy.py</t>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_constants.py</t>
         </is>
       </c>
       <c r="M100" s="29" t="inlineStr">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="N100" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：test_phase1_protocol_enums_have_only_approved_values；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -9549,7 +9549,7 @@
       </c>
       <c r="D114" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E114" s="29" t="inlineStr">
@@ -9599,7 +9599,7 @@
       </c>
       <c r="N114" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：create vector + six operation frozen vectors；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -9621,7 +9621,7 @@
       </c>
       <c r="D115" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E115" s="29" t="inlineStr">
@@ -9671,7 +9671,7 @@
       </c>
       <c r="N115" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：canonical mapping order + subprocess restart；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -9693,7 +9693,7 @@
       </c>
       <c r="D116" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E116" s="29" t="inlineStr">
@@ -9743,7 +9743,7 @@
       </c>
       <c r="N116" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：six-operation field sensitivity + excluded input fields；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -10341,7 +10341,7 @@
       </c>
       <c r="D125" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E125" s="29" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="N125" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>实际覆盖：usr_ 格式/唯一性 + actor identity；2026-07-15 EvieAi 定向 96 passed。</t>
         </is>
       </c>
     </row>
@@ -11116,7 +11116,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N84"/>
+  <autoFilter ref="A1:N135"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13896,7 +13896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15073,8 +15073,136 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>SL1-V01</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1 EvieAi 定向测试</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>pytest -q tests/unit/evie_ai</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>96 passed</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>纯 Policy、ID、Settings、错误及架构边界全部通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>SL1-V02</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1 全量单元回归</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>pytest -q tests/unit --tb=no</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>550 passed, 32 failed</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>通过（存在已知旧链失败）</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>32 个失败均属于冻结旧 Workbench/生成链</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>SL1-V03</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>失败节点基线对比</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>当前分支 vs e111f21 临时 worktree</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>diff exit 0</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>基线 32 个失败节点与当前完全一致；新增失败 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>SL1-V04</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>Slice 1 静态和范围检查</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Ruff + py_compile + git diff/scope audit</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>未触及 ORM、Migration、Repository、Service、Router、认证模型或旧链</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F25"/>
+  <autoFilter ref="A3:F42"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -18000,7 +18128,7 @@
       </c>
       <c r="F3" s="29" t="inlineStr">
         <is>
-          <t>codex/evie-ai-phase1-slice0-closeout</t>
+          <t>codex/evie-ai-phase1-slice1-policies</t>
         </is>
       </c>
       <c r="G3" s="5" t="n"/>
@@ -18013,7 +18141,7 @@
         </is>
       </c>
       <c r="B4" s="29" t="n">
-        <v>77</v>
+        <v>122</v>
       </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
@@ -18024,7 +18152,7 @@
       </c>
       <c r="F4" s="29" t="inlineStr">
         <is>
-          <t>77 passed, 11 warnings in 7.09s（代码未变，本轮未重跑）</t>
+          <t>EvieAi 96 passed；全量 550 passed, 32 known legacy failures；新增失败 0</t>
         </is>
       </c>
       <c r="G4" s="5" t="n"/>
@@ -18037,7 +18165,7 @@
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="6" t="n"/>
@@ -18060,7 +18188,7 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>dev@adb2b2b</t>
+          <t>dev@e111f21 + Slice 1 未提交工作区</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -18129,11 +18257,11 @@
       <c r="D11" s="31" t="n"/>
       <c r="E11" s="31" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="F11" s="31" t="n">
-        <v>83</v>
+        <v>21</v>
       </c>
       <c r="G11" s="31" t="n"/>
       <c r="H11" s="31" t="n"/>
@@ -18151,11 +18279,11 @@
       <c r="D12" s="31" t="n"/>
       <c r="E12" s="31" t="inlineStr">
         <is>
-          <t>待签字</t>
+          <t>待实现</t>
         </is>
       </c>
       <c r="F12" s="31" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="G12" s="31" t="n"/>
       <c r="H12" s="31" t="n"/>
@@ -18167,7 +18295,7 @@
         </is>
       </c>
       <c r="B13" s="31" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C13" s="31" t="n"/>
       <c r="D13" s="31" t="n"/>
@@ -18243,11 +18371,11 @@
     <row r="18">
       <c r="A18" s="31" t="inlineStr">
         <is>
-          <t>冻结结构兼容性</t>
+          <t>冻结结构/标识符/Bootstrap</t>
         </is>
       </c>
       <c r="B18" s="31" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="31" t="n"/>
@@ -18263,7 +18391,7 @@
         </is>
       </c>
       <c r="B19" s="31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="31" t="n"/>
@@ -18275,11 +18403,11 @@
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
         <is>
-          <t>标识符守卫</t>
+          <t>Phase 1 常量/配置/错误</t>
         </is>
       </c>
       <c r="B20" s="31" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C20" s="31" t="n"/>
       <c r="D20" s="31" t="n"/>
@@ -18291,11 +18419,11 @@
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
-          <t>确定性 Bootstrap</t>
+          <t>Phase 1 纯 Policy</t>
         </is>
       </c>
       <c r="B21" s="31" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C21" s="31" t="n"/>
       <c r="D21" s="31" t="n"/>
@@ -18349,7 +18477,7 @@
     <row r="29">
       <c r="A29" s="32" t="inlineStr">
         <is>
-          <t>6. A-11 已签字；P-09 计划用例解除合同阻塞，但仍须等待 Slice 0 文档 PR 合并后实施。</t>
+          <t>6. Slice 0 已合并；Slice 1 Policy/ID 测试已实现并通过，代码尚未提交。</t>
         </is>
       </c>
     </row>
@@ -18385,7 +18513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P78"/>
+  <dimension ref="A1:P123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -18520,7 +18648,7 @@
         </is>
       </c>
       <c r="G2" s="29" t="n">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="H2" s="29" t="inlineStr">
         <is>
@@ -18600,7 +18728,7 @@
         </is>
       </c>
       <c r="G3" s="29" t="n">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="H3" s="29" t="inlineStr">
         <is>
@@ -18680,7 +18808,7 @@
         </is>
       </c>
       <c r="G4" s="29" t="n">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H4" s="29" t="inlineStr">
         <is>
@@ -18760,7 +18888,7 @@
         </is>
       </c>
       <c r="G5" s="29" t="n">
-        <v>119</v>
+        <v>158</v>
       </c>
       <c r="H5" s="29" t="inlineStr">
         <is>
@@ -18840,7 +18968,7 @@
         </is>
       </c>
       <c r="G6" s="29" t="n">
-        <v>127</v>
+        <v>166</v>
       </c>
       <c r="H6" s="29" t="inlineStr">
         <is>
@@ -18920,7 +19048,7 @@
         </is>
       </c>
       <c r="G7" s="29" t="n">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="H7" s="29" t="inlineStr">
         <is>
@@ -19000,7 +19128,7 @@
         </is>
       </c>
       <c r="G8" s="29" t="n">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="H8" s="29" t="inlineStr">
         <is>
@@ -19080,7 +19208,7 @@
         </is>
       </c>
       <c r="G9" s="29" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="H9" s="29" t="inlineStr">
         <is>
@@ -19160,7 +19288,7 @@
         </is>
       </c>
       <c r="G10" s="29" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="H10" s="29" t="inlineStr">
         <is>
@@ -19240,7 +19368,7 @@
         </is>
       </c>
       <c r="G11" s="29" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="H11" s="29" t="inlineStr">
         <is>
@@ -19320,7 +19448,7 @@
         </is>
       </c>
       <c r="G12" s="29" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="H12" s="29" t="inlineStr">
         <is>
@@ -19400,7 +19528,7 @@
         </is>
       </c>
       <c r="G13" s="29" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="H13" s="29" t="inlineStr">
         <is>
@@ -19480,7 +19608,7 @@
         </is>
       </c>
       <c r="G14" s="29" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="H14" s="29" t="inlineStr">
         <is>
@@ -19560,7 +19688,7 @@
         </is>
       </c>
       <c r="G15" s="29" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="H15" s="29" t="inlineStr">
         <is>
@@ -19640,7 +19768,7 @@
         </is>
       </c>
       <c r="G16" s="29" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="H16" s="29" t="inlineStr">
         <is>
@@ -19720,7 +19848,7 @@
         </is>
       </c>
       <c r="G17" s="29" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="H17" s="29" t="inlineStr">
         <is>
@@ -19800,7 +19928,7 @@
         </is>
       </c>
       <c r="G18" s="29" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="H18" s="29" t="inlineStr">
         <is>
@@ -19880,7 +20008,7 @@
         </is>
       </c>
       <c r="G19" s="29" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="H19" s="29" t="inlineStr">
         <is>
@@ -24648,8 +24776,3608 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-078</t>
+        </is>
+      </c>
+      <c r="B79" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C79" s="29" t="inlineStr">
+        <is>
+          <t>架构守卫</t>
+        </is>
+      </c>
+      <c r="D79" s="29" t="inlineStr">
+        <is>
+          <t>静态/架构单元测试</t>
+        </is>
+      </c>
+      <c r="E79" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F79" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_architecture_boundaries.py</t>
+        </is>
+      </c>
+      <c r="G79" s="29" t="n">
+        <v>109</v>
+      </c>
+      <c r="H79" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_architecture_boundaries.py::test_evie_ai_policies_do_not_depend_on_stateful_application_layers</t>
+        </is>
+      </c>
+      <c r="I79" s="29" t="inlineStr">
+        <is>
+          <t>纯 Policy 禁止依赖有状态应用层</t>
+        </is>
+      </c>
+      <c r="J79" s="29" t="inlineStr">
+        <is>
+          <t>验证 Policy 与 ORM/Repository/Service/Router/SQLAlchemy 的依赖隔离。</t>
+        </is>
+      </c>
+      <c r="K79" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L79" s="29" t="inlineStr">
+        <is>
+          <t>AST 扫描无禁止依赖。</t>
+        </is>
+      </c>
+      <c r="M79" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/AST</t>
+        </is>
+      </c>
+      <c r="N79" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O79" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P79" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 架构边界；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-079</t>
+        </is>
+      </c>
+      <c r="B80" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C80" s="29" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="D80" s="29" t="inlineStr">
+        <is>
+          <t>配置单元测试</t>
+        </is>
+      </c>
+      <c r="E80" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F80" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py</t>
+        </is>
+      </c>
+      <c r="G80" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="H80" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py::test_idempotency_retention_defaults_to_seven_days</t>
+        </is>
+      </c>
+      <c r="I80" s="29" t="inlineStr">
+        <is>
+          <t>幂等保留期默认 7 天</t>
+        </is>
+      </c>
+      <c r="J80" s="29" t="inlineStr">
+        <is>
+          <t>验证未配置环境变量时 Settings 使用唯一批准默认值。</t>
+        </is>
+      </c>
+      <c r="K80" s="29" t="inlineStr">
+        <is>
+          <t>monkeypatch 隔离环境变量</t>
+        </is>
+      </c>
+      <c r="L80" s="29" t="inlineStr">
+        <is>
+          <t>配置值为 7。</t>
+        </is>
+      </c>
+      <c r="M80" s="29" t="inlineStr">
+        <is>
+          <t>环境变量隔离</t>
+        </is>
+      </c>
+      <c r="N80" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O80" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P80" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-009；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-080</t>
+        </is>
+      </c>
+      <c r="B81" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C81" s="29" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="D81" s="29" t="inlineStr">
+        <is>
+          <t>配置单元测试</t>
+        </is>
+      </c>
+      <c r="E81" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F81" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py</t>
+        </is>
+      </c>
+      <c r="G81" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="H81" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py::test_idempotency_retention_accepts_positive_environment_override</t>
+        </is>
+      </c>
+      <c r="I81" s="29" t="inlineStr">
+        <is>
+          <t>幂等保留期接受正整数覆盖</t>
+        </is>
+      </c>
+      <c r="J81" s="29" t="inlineStr">
+        <is>
+          <t>验证 Settings 接受合法正整数环境配置。</t>
+        </is>
+      </c>
+      <c r="K81" s="29" t="inlineStr">
+        <is>
+          <t>monkeypatch 隔离环境变量</t>
+        </is>
+      </c>
+      <c r="L81" s="29" t="inlineStr">
+        <is>
+          <t>配置值使用显式覆盖值。</t>
+        </is>
+      </c>
+      <c r="M81" s="29" t="inlineStr">
+        <is>
+          <t>环境变量隔离</t>
+        </is>
+      </c>
+      <c r="N81" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O81" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P81" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-010；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-081</t>
+        </is>
+      </c>
+      <c r="B82" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C82" s="29" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="D82" s="29" t="inlineStr">
+        <is>
+          <t>配置单元测试</t>
+        </is>
+      </c>
+      <c r="E82" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F82" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py</t>
+        </is>
+      </c>
+      <c r="G82" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="H82" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py::test_idempotency_retention_rejects_invalid_environment_values[0]</t>
+        </is>
+      </c>
+      <c r="I82" s="29" t="inlineStr">
+        <is>
+          <t>幂等保留期拒绝非法值｜0</t>
+        </is>
+      </c>
+      <c r="J82" s="29" t="inlineStr">
+        <is>
+          <t>验证 0、负数和非整数均 fail-closed。</t>
+        </is>
+      </c>
+      <c r="K82" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：0</t>
+        </is>
+      </c>
+      <c r="L82" s="29" t="inlineStr">
+        <is>
+          <t>Settings 构造明确失败。</t>
+        </is>
+      </c>
+      <c r="M82" s="29" t="inlineStr">
+        <is>
+          <t>环境变量隔离</t>
+        </is>
+      </c>
+      <c r="N82" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O82" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P82" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-011；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-082</t>
+        </is>
+      </c>
+      <c r="B83" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C83" s="29" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="D83" s="29" t="inlineStr">
+        <is>
+          <t>配置单元测试</t>
+        </is>
+      </c>
+      <c r="E83" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F83" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py</t>
+        </is>
+      </c>
+      <c r="G83" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="H83" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py::test_idempotency_retention_rejects_invalid_environment_values[-1]</t>
+        </is>
+      </c>
+      <c r="I83" s="29" t="inlineStr">
+        <is>
+          <t>幂等保留期拒绝非法值｜-1</t>
+        </is>
+      </c>
+      <c r="J83" s="29" t="inlineStr">
+        <is>
+          <t>验证 0、负数和非整数均 fail-closed。</t>
+        </is>
+      </c>
+      <c r="K83" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：-1</t>
+        </is>
+      </c>
+      <c r="L83" s="29" t="inlineStr">
+        <is>
+          <t>Settings 构造明确失败。</t>
+        </is>
+      </c>
+      <c r="M83" s="29" t="inlineStr">
+        <is>
+          <t>环境变量隔离</t>
+        </is>
+      </c>
+      <c r="N83" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O83" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P83" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-011；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-083</t>
+        </is>
+      </c>
+      <c r="B84" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C84" s="29" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="D84" s="29" t="inlineStr">
+        <is>
+          <t>配置单元测试</t>
+        </is>
+      </c>
+      <c r="E84" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F84" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py</t>
+        </is>
+      </c>
+      <c r="G84" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="H84" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_config.py::test_idempotency_retention_rejects_invalid_environment_values[not-an-integer]</t>
+        </is>
+      </c>
+      <c r="I84" s="29" t="inlineStr">
+        <is>
+          <t>幂等保留期拒绝非法值｜not-an-integer</t>
+        </is>
+      </c>
+      <c r="J84" s="29" t="inlineStr">
+        <is>
+          <t>验证 0、负数和非整数均 fail-closed。</t>
+        </is>
+      </c>
+      <c r="K84" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：not-an-integer</t>
+        </is>
+      </c>
+      <c r="L84" s="29" t="inlineStr">
+        <is>
+          <t>Settings 构造明确失败。</t>
+        </is>
+      </c>
+      <c r="M84" s="29" t="inlineStr">
+        <is>
+          <t>环境变量隔离</t>
+        </is>
+      </c>
+      <c r="N84" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O84" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P84" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-011；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-084</t>
+        </is>
+      </c>
+      <c r="B85" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C85" s="29" t="inlineStr">
+        <is>
+          <t>协议常量</t>
+        </is>
+      </c>
+      <c r="D85" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E85" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F85" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_constants.py</t>
+        </is>
+      </c>
+      <c r="G85" s="29" t="n">
+        <v>23</v>
+      </c>
+      <c r="H85" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_constants.py::test_phase1_protocol_enums_have_only_approved_values</t>
+        </is>
+      </c>
+      <c r="I85" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 协议枚举只包含批准值</t>
+        </is>
+      </c>
+      <c r="J85" s="29" t="inlineStr">
+        <is>
+          <t>验证来源、operation、审核操作和审计事件均集中定义。</t>
+        </is>
+      </c>
+      <c r="K85" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L85" s="29" t="inlineStr">
+        <is>
+          <t>枚举集合与批准合同完全一致。</t>
+        </is>
+      </c>
+      <c r="M85" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N85" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O85" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P85" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-099；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-085</t>
+        </is>
+      </c>
+      <c r="B86" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C86" s="29" t="inlineStr">
+        <is>
+          <t>协议常量</t>
+        </is>
+      </c>
+      <c r="D86" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E86" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F86" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_constants.py</t>
+        </is>
+      </c>
+      <c r="G86" s="29" t="n">
+        <v>47</v>
+      </c>
+      <c r="H86" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_constants.py::test_conversion_status_does_not_include_failed</t>
+        </is>
+      </c>
+      <c r="I86" s="29" t="inlineStr">
+        <is>
+          <t>conversion_status 不包含 failed</t>
+        </is>
+      </c>
+      <c r="J86" s="29" t="inlineStr">
+        <is>
+          <t>验证合法状态集合沿用批准的 Phase 0 合同。</t>
+        </is>
+      </c>
+      <c r="K86" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L86" s="29" t="inlineStr">
+        <is>
+          <t>仅包含 not_started/processing/blocked/succeeded/stale。</t>
+        </is>
+      </c>
+      <c r="M86" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N86" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O86" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P86" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-085；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-086</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C87" s="29" t="inlineStr">
+        <is>
+          <t>内容指纹</t>
+        </is>
+      </c>
+      <c r="D87" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E87" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F87" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G87" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="H87" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py::test_content_normalization_preserves_meaning_and_stabilizes_tags</t>
+        </is>
+      </c>
+      <c r="I87" s="29" t="inlineStr">
+        <is>
+          <t>自然语言内容规范化与 Tags 稳定化</t>
+        </is>
+      </c>
+      <c r="J87" s="29" t="inlineStr">
+        <is>
+          <t>验证 NFC、换行、字段空白、内部空格和 tags 规则。</t>
+        </is>
+      </c>
+      <c r="K87" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L87" s="29" t="inlineStr">
+        <is>
+          <t>得到批准的规范化内容且不语义改写。</t>
+        </is>
+      </c>
+      <c r="M87" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N87" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O87" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P87" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-003～006；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-087</t>
+        </is>
+      </c>
+      <c r="B88" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C88" s="29" t="inlineStr">
+        <is>
+          <t>内容指纹</t>
+        </is>
+      </c>
+      <c r="D88" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E88" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F88" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G88" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="H88" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py::test_content_fingerprint_matches_frozen_vector</t>
+        </is>
+      </c>
+      <c r="I88" s="29" t="inlineStr">
+        <is>
+          <t>Content fingerprint 固定测试向量</t>
+        </is>
+      </c>
+      <c r="J88" s="29" t="inlineStr">
+        <is>
+          <t>验证 canonical JSON UTF-8 SHA-256 冻结算法。</t>
+        </is>
+      </c>
+      <c r="K88" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L88" s="29" t="inlineStr">
+        <is>
+          <t>输出与冻结 SHA-256 向量一致。</t>
+        </is>
+      </c>
+      <c r="M88" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N88" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O88" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P88" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-084；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-088</t>
+        </is>
+      </c>
+      <c r="B89" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C89" s="29" t="inlineStr">
+        <is>
+          <t>内容指纹</t>
+        </is>
+      </c>
+      <c r="D89" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E89" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F89" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G89" s="29" t="n">
+        <v>41</v>
+      </c>
+      <c r="H89" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py::test_canonical_json_is_independent_of_mapping_order</t>
+        </is>
+      </c>
+      <c r="I89" s="29" t="inlineStr">
+        <is>
+          <t>Canonical JSON 不受字典顺序影响</t>
+        </is>
+      </c>
+      <c r="J89" s="29" t="inlineStr">
+        <is>
+          <t>验证固定键排序、紧凑 JSON 和 UTF-8 字节流。</t>
+        </is>
+      </c>
+      <c r="K89" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L89" s="29" t="inlineStr">
+        <is>
+          <t>不同字典顺序得到相同字节流。</t>
+        </is>
+      </c>
+      <c r="M89" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N89" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O89" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P89" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-084/114；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-089</t>
+        </is>
+      </c>
+      <c r="B90" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C90" s="29" t="inlineStr">
+        <is>
+          <t>内容指纹</t>
+        </is>
+      </c>
+      <c r="D90" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E90" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F90" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G90" s="29" t="n">
+        <v>49</v>
+      </c>
+      <c r="H90" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_content_fingerprint.py::test_incomplete_natural_language_content_remains_fingerprintable</t>
+        </is>
+      </c>
+      <c r="I90" s="29" t="inlineStr">
+        <is>
+          <t>不完整自然语言内容仍可计算指纹</t>
+        </is>
+      </c>
+      <c r="J90" s="29" t="inlineStr">
+        <is>
+          <t>验证低质量或不完整内容不会被 Policy 阻止进入资产流程。</t>
+        </is>
+      </c>
+      <c r="K90" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L90" s="29" t="inlineStr">
+        <is>
+          <t>空白自然语言字段仍得到合法 SHA-256。</t>
+        </is>
+      </c>
+      <c r="M90" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N90" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O90" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P90" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 自然语言资产硬边界；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-090</t>
+        </is>
+      </c>
+      <c r="B91" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C91" s="29" t="inlineStr">
+        <is>
+          <t>结构化错误</t>
+        </is>
+      </c>
+      <c r="D91" s="29" t="inlineStr">
+        <is>
+          <t>契约单元测试</t>
+        </is>
+      </c>
+      <c r="E91" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F91" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_errors.py</t>
+        </is>
+      </c>
+      <c r="G91" s="29" t="n">
+        <v>31</v>
+      </c>
+      <c r="H91" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_errors.py::test_stable_error_code_set_matches_phase1_contract</t>
+        </is>
+      </c>
+      <c r="I91" s="29" t="inlineStr">
+        <is>
+          <t>稳定错误码集合符合 Phase 1 合同</t>
+        </is>
+      </c>
+      <c r="J91" s="29" t="inlineStr">
+        <is>
+          <t>验证错误码集中定义且无遗漏或漂移。</t>
+        </is>
+      </c>
+      <c r="K91" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L91" s="29" t="inlineStr">
+        <is>
+          <t>错误码集合与 Specification 一致。</t>
+        </is>
+      </c>
+      <c r="M91" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N91" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O91" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P91" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 C-05/稳定错误合同；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-091</t>
+        </is>
+      </c>
+      <c r="B92" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C92" s="29" t="inlineStr">
+        <is>
+          <t>结构化错误</t>
+        </is>
+      </c>
+      <c r="D92" s="29" t="inlineStr">
+        <is>
+          <t>契约单元测试</t>
+        </is>
+      </c>
+      <c r="E92" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F92" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_errors.py</t>
+        </is>
+      </c>
+      <c r="G92" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="H92" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_errors.py::test_domain_error_exposes_structured_contract_without_transport_logic</t>
+        </is>
+      </c>
+      <c r="I92" s="29" t="inlineStr">
+        <is>
+          <t>领域错误提供稳定结构且不耦合传输层</t>
+        </is>
+      </c>
+      <c r="J92" s="29" t="inlineStr">
+        <is>
+          <t>验证 code/domain/stage/retryable/trace 等字段。</t>
+        </is>
+      </c>
+      <c r="K92" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L92" s="29" t="inlineStr">
+        <is>
+          <t>结构化错误字段完整且无 Router 依赖。</t>
+        </is>
+      </c>
+      <c r="M92" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N92" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O92" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P92" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 C-05/稳定错误合同；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-092</t>
+        </is>
+      </c>
+      <c r="B93" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C93" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D93" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E93" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F93" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G93" s="29" t="n">
+        <v>13</v>
+      </c>
+      <c r="H93" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_user_public_id_and_actor_use_approved_stable_identity</t>
+        </is>
+      </c>
+      <c r="I93" s="29" t="inlineStr">
+        <is>
+          <t>用户公共 ID 生成标准 actor 身份</t>
+        </is>
+      </c>
+      <c r="J93" s="29" t="inlineStr">
+        <is>
+          <t>验证 actor 固定为 user:&lt;user_public_id&gt;。</t>
+        </is>
+      </c>
+      <c r="K93" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L93" s="29" t="inlineStr">
+        <is>
+          <t>合法 usr_ ID 规范化为稳定公共 actor。</t>
+        </is>
+      </c>
+      <c r="M93" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N93" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O93" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P93" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 A-11/P-09；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-093</t>
+        </is>
+      </c>
+      <c r="B94" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C94" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D94" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E94" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F94" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G94" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="H94" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_invalid_user_public_identity_fails_closed[None]</t>
+        </is>
+      </c>
+      <c r="I94" s="29" t="inlineStr">
+        <is>
+          <t>非法或缺失用户公共身份 fail-closed｜None</t>
+        </is>
+      </c>
+      <c r="J94" s="29" t="inlineStr">
+        <is>
+          <t>验证不得退化使用 username、内部 PK 或其他可变身份。</t>
+        </is>
+      </c>
+      <c r="K94" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：None</t>
+        </is>
+      </c>
+      <c r="L94" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_DATA_INTEGRITY_ERROR。</t>
+        </is>
+      </c>
+      <c r="M94" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N94" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O94" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P94" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 A-11/P-09；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-094</t>
+        </is>
+      </c>
+      <c r="B95" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C95" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D95" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E95" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F95" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G95" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="H95" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_invalid_user_public_identity_fails_closed[]</t>
+        </is>
+      </c>
+      <c r="I95" s="29" t="inlineStr">
+        <is>
+          <t>非法或缺失用户公共身份 fail-closed｜空字符串</t>
+        </is>
+      </c>
+      <c r="J95" s="29" t="inlineStr">
+        <is>
+          <t>验证不得退化使用 username、内部 PK 或其他可变身份。</t>
+        </is>
+      </c>
+      <c r="K95" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：空字符串</t>
+        </is>
+      </c>
+      <c r="L95" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_DATA_INTEGRITY_ERROR。</t>
+        </is>
+      </c>
+      <c r="M95" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N95" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O95" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P95" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 A-11/P-09；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-095</t>
+        </is>
+      </c>
+      <c r="B96" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C96" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D96" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E96" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F96" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G96" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="H96" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_invalid_user_public_identity_fails_closed[usr_short]</t>
+        </is>
+      </c>
+      <c r="I96" s="29" t="inlineStr">
+        <is>
+          <t>非法或缺失用户公共身份 fail-closed｜usr_short</t>
+        </is>
+      </c>
+      <c r="J96" s="29" t="inlineStr">
+        <is>
+          <t>验证不得退化使用 username、内部 PK 或其他可变身份。</t>
+        </is>
+      </c>
+      <c r="K96" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：usr_short</t>
+        </is>
+      </c>
+      <c r="L96" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_DATA_INTEGRITY_ERROR。</t>
+        </is>
+      </c>
+      <c r="M96" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N96" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O96" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P96" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 A-11/P-09；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-096</t>
+        </is>
+      </c>
+      <c r="B97" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C97" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D97" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E97" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F97" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G97" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="H97" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_invalid_user_public_identity_fails_closed[USR_0123456789abcdef0123456789abcdef]</t>
+        </is>
+      </c>
+      <c r="I97" s="29" t="inlineStr">
+        <is>
+          <t>非法或缺失用户公共身份 fail-closed｜USR_0123456789abcdef0123456789abcdef</t>
+        </is>
+      </c>
+      <c r="J97" s="29" t="inlineStr">
+        <is>
+          <t>验证不得退化使用 username、内部 PK 或其他可变身份。</t>
+        </is>
+      </c>
+      <c r="K97" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：USR_0123456789abcdef0123456789abcdef</t>
+        </is>
+      </c>
+      <c r="L97" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_DATA_INTEGRITY_ERROR。</t>
+        </is>
+      </c>
+      <c r="M97" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N97" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O97" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P97" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 A-11/P-09；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-097</t>
+        </is>
+      </c>
+      <c r="B98" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C98" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D98" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E98" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F98" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G98" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="H98" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_invalid_user_public_identity_fails_closed[123]</t>
+        </is>
+      </c>
+      <c r="I98" s="29" t="inlineStr">
+        <is>
+          <t>非法或缺失用户公共身份 fail-closed｜123</t>
+        </is>
+      </c>
+      <c r="J98" s="29" t="inlineStr">
+        <is>
+          <t>验证不得退化使用 username、内部 PK 或其他可变身份。</t>
+        </is>
+      </c>
+      <c r="K98" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：123</t>
+        </is>
+      </c>
+      <c r="L98" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_DATA_INTEGRITY_ERROR。</t>
+        </is>
+      </c>
+      <c r="M98" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N98" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O98" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P98" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 A-11/P-09；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-098</t>
+        </is>
+      </c>
+      <c r="B99" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C99" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D99" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E99" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F99" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G99" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="H99" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_asset_code_for_new_asset_is_its_public_id</t>
+        </is>
+      </c>
+      <c r="I99" s="29" t="inlineStr">
+        <is>
+          <t>新资产 asset_code 等于 test_asset_id</t>
+        </is>
+      </c>
+      <c r="J99" s="29" t="inlineStr">
+        <is>
+          <t>验证 A-01 服务端权威 asset_code Policy。</t>
+        </is>
+      </c>
+      <c r="K99" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L99" s="29" t="inlineStr">
+        <is>
+          <t>返回原 test_asset_id。</t>
+        </is>
+      </c>
+      <c r="M99" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N99" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O99" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P99" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-014；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-099</t>
+        </is>
+      </c>
+      <c r="B100" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C100" s="29" t="inlineStr">
+        <is>
+          <t>身份与 AssetCode Policy</t>
+        </is>
+      </c>
+      <c r="D100" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E100" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F100" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py</t>
+        </is>
+      </c>
+      <c r="G100" s="29" t="n">
+        <v>36</v>
+      </c>
+      <c r="H100" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_identity_policies.py::test_asset_code_policy_rejects_non_asset_identity</t>
+        </is>
+      </c>
+      <c r="I100" s="29" t="inlineStr">
+        <is>
+          <t>AssetCode Policy 拒绝非资产 ID</t>
+        </is>
+      </c>
+      <c r="J100" s="29" t="inlineStr">
+        <is>
+          <t>验证客户端或错误身份不能伪造 asset_code。</t>
+        </is>
+      </c>
+      <c r="K100" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L100" s="29" t="inlineStr">
+        <is>
+          <t>结构化数据完整性错误。</t>
+        </is>
+      </c>
+      <c r="M100" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N100" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O100" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P100" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-014；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-100</t>
+        </is>
+      </c>
+      <c r="B101" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C101" s="29" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D101" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E101" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F101" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py</t>
+        </is>
+      </c>
+      <c r="G101" s="29" t="n">
+        <v>53</v>
+      </c>
+      <c r="H101" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py::test_evie_ai_public_ids_have_expected_format[generate_user_public_id-usr-^usr_[0-9a-f]{32}$]</t>
+        </is>
+      </c>
+      <c r="I101" s="29" t="inlineStr">
+        <is>
+          <t>usr_ 用户公共 ID 格式｜generate_user_public_id-usr-^usr_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="J101" s="29" t="inlineStr">
+        <is>
+          <t>验证 usr_ 用户公共 ID 使用完整 uuid4hex32。</t>
+        </is>
+      </c>
+      <c r="K101" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：generate_user_public_id-usr-^usr_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="L101" s="29" t="inlineStr">
+        <is>
+          <t>前缀正确，后缀为 32 位小写十六进制。</t>
+        </is>
+      </c>
+      <c r="M101" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N101" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O101" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P101" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-001/124；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-101</t>
+        </is>
+      </c>
+      <c r="B102" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C102" s="29" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D102" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E102" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F102" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py</t>
+        </is>
+      </c>
+      <c r="G102" s="29" t="n">
+        <v>53</v>
+      </c>
+      <c r="H102" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py::test_evie_ai_public_ids_have_expected_format[generate_test_asset_review_id-tar-^tar_[0-9a-f]{32}$]</t>
+        </is>
+      </c>
+      <c r="I102" s="29" t="inlineStr">
+        <is>
+          <t>tar_ 审核记录 ID 格式｜generate_test_asset_review_id-tar-^tar_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="J102" s="29" t="inlineStr">
+        <is>
+          <t>验证 tar_ 审核记录 ID 使用完整 uuid4hex32。</t>
+        </is>
+      </c>
+      <c r="K102" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：generate_test_asset_review_id-tar-^tar_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="L102" s="29" t="inlineStr">
+        <is>
+          <t>前缀正确，后缀为 32 位小写十六进制。</t>
+        </is>
+      </c>
+      <c r="M102" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N102" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O102" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P102" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-001/124；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-102</t>
+        </is>
+      </c>
+      <c r="B103" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C103" s="29" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D103" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E103" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F103" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py</t>
+        </is>
+      </c>
+      <c r="G103" s="29" t="n">
+        <v>53</v>
+      </c>
+      <c r="H103" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py::test_evie_ai_public_ids_have_expected_format[generate_test_asset_audit_event_id-tae-^tae_[0-9a-f]{32}$]</t>
+        </is>
+      </c>
+      <c r="I103" s="29" t="inlineStr">
+        <is>
+          <t>tae_ 审计事件 ID 格式｜generate_test_asset_audit_event_id-tae-^tae_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="J103" s="29" t="inlineStr">
+        <is>
+          <t>验证 tae_ 审计事件 ID 使用完整 uuid4hex32。</t>
+        </is>
+      </c>
+      <c r="K103" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：generate_test_asset_audit_event_id-tae-^tae_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="L103" s="29" t="inlineStr">
+        <is>
+          <t>前缀正确，后缀为 32 位小写十六进制。</t>
+        </is>
+      </c>
+      <c r="M103" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N103" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O103" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P103" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-001/124；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-103</t>
+        </is>
+      </c>
+      <c r="B104" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C104" s="29" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D104" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E104" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F104" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py</t>
+        </is>
+      </c>
+      <c r="G104" s="29" t="n">
+        <v>65</v>
+      </c>
+      <c r="H104" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py::test_evie_ai_public_ids_are_unique[generate_user_public_id-usr-^usr_[0-9a-f]{32}$]</t>
+        </is>
+      </c>
+      <c r="I104" s="29" t="inlineStr">
+        <is>
+          <t>usr_ 用户公共 ID 1000 次抽样唯一性｜generate_user_public_id-usr-^usr_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="J104" s="29" t="inlineStr">
+        <is>
+          <t>验证 usr_ 用户公共 ID 批量生成不重复。</t>
+        </is>
+      </c>
+      <c r="K104" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：generate_user_public_id-usr-^usr_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="L104" s="29" t="inlineStr">
+        <is>
+          <t>1000 个生成值全部唯一。</t>
+        </is>
+      </c>
+      <c r="M104" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N104" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O104" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P104" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-002/124；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-104</t>
+        </is>
+      </c>
+      <c r="B105" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C105" s="29" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D105" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E105" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F105" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py</t>
+        </is>
+      </c>
+      <c r="G105" s="29" t="n">
+        <v>65</v>
+      </c>
+      <c r="H105" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py::test_evie_ai_public_ids_are_unique[generate_test_asset_review_id-tar-^tar_[0-9a-f]{32}$]</t>
+        </is>
+      </c>
+      <c r="I105" s="29" t="inlineStr">
+        <is>
+          <t>tar_ 审核记录 ID 1000 次抽样唯一性｜generate_test_asset_review_id-tar-^tar_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="J105" s="29" t="inlineStr">
+        <is>
+          <t>验证 tar_ 审核记录 ID 批量生成不重复。</t>
+        </is>
+      </c>
+      <c r="K105" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：generate_test_asset_review_id-tar-^tar_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="L105" s="29" t="inlineStr">
+        <is>
+          <t>1000 个生成值全部唯一。</t>
+        </is>
+      </c>
+      <c r="M105" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N105" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O105" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P105" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-002/124；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-105</t>
+        </is>
+      </c>
+      <c r="B106" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C106" s="29" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D106" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E106" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F106" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py</t>
+        </is>
+      </c>
+      <c r="G106" s="29" t="n">
+        <v>65</v>
+      </c>
+      <c r="H106" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_ids.py::test_evie_ai_public_ids_are_unique[generate_test_asset_audit_event_id-tae-^tae_[0-9a-f]{32}$]</t>
+        </is>
+      </c>
+      <c r="I106" s="29" t="inlineStr">
+        <is>
+          <t>tae_ 审计事件 ID 1000 次抽样唯一性｜generate_test_asset_audit_event_id-tae-^tae_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="J106" s="29" t="inlineStr">
+        <is>
+          <t>验证 tae_ 审计事件 ID 批量生成不重复。</t>
+        </is>
+      </c>
+      <c r="K106" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：generate_test_asset_audit_event_id-tae-^tae_[0-9a-f]{32}$</t>
+        </is>
+      </c>
+      <c r="L106" s="29" t="inlineStr">
+        <is>
+          <t>1000 个生成值全部唯一。</t>
+        </is>
+      </c>
+      <c r="M106" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N106" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O106" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P106" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-002/124；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-106</t>
+        </is>
+      </c>
+      <c r="B107" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C107" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D107" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E107" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F107" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G107" s="29" t="n">
+        <v>43</v>
+      </c>
+      <c r="H107" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py::test_create_asset_request_fingerprint_matches_frozen_vector</t>
+        </is>
+      </c>
+      <c r="I107" s="29" t="inlineStr">
+        <is>
+          <t>create_asset request fingerprint 固定向量</t>
+        </is>
+      </c>
+      <c r="J107" s="29" t="inlineStr">
+        <is>
+          <t>验证 v1 canonical JSON 请求指纹。</t>
+        </is>
+      </c>
+      <c r="K107" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L107" s="29" t="inlineStr">
+        <is>
+          <t>输出与冻结 SHA-256 向量一致。</t>
+        </is>
+      </c>
+      <c r="M107" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/部分子进程</t>
+        </is>
+      </c>
+      <c r="N107" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O107" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P107" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-113；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-107</t>
+        </is>
+      </c>
+      <c r="B108" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C108" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D108" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E108" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F108" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G108" s="29" t="n">
+        <v>54</v>
+      </c>
+      <c r="H108" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py::test_all_six_operation_fingerprints_are_stable_and_field_sensitive</t>
+        </is>
+      </c>
+      <c r="I108" s="29" t="inlineStr">
+        <is>
+          <t>六种 operation 请求指纹固定且字段敏感</t>
+        </is>
+      </c>
+      <c r="J108" s="29" t="inlineStr">
+        <is>
+          <t>逐项验证六种批准 operation 的冻结向量和关键字段变化。</t>
+        </is>
+      </c>
+      <c r="K108" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L108" s="29" t="inlineStr">
+        <is>
+          <t>六个冻结向量一致；关键字段变化均改变指纹。</t>
+        </is>
+      </c>
+      <c r="M108" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/部分子进程</t>
+        </is>
+      </c>
+      <c r="N108" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O108" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P108" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-113/115；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-108</t>
+        </is>
+      </c>
+      <c r="B109" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C109" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D109" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E109" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F109" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G109" s="29" t="n">
+        <v>166</v>
+      </c>
+      <c r="H109" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py::test_scope_and_transport_fields_are_not_accepted_by_fingerprint_inputs</t>
+        </is>
+      </c>
+      <c r="I109" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint 排除 scope 与传输字段</t>
+        </is>
+      </c>
+      <c r="J109" s="29" t="inlineStr">
+        <is>
+          <t>验证 project/actor/channel/key/request/time 不进入指纹输入。</t>
+        </is>
+      </c>
+      <c r="K109" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L109" s="29" t="inlineStr">
+        <is>
+          <t>输入合同不包含所有禁止字段。</t>
+        </is>
+      </c>
+      <c r="M109" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/部分子进程</t>
+        </is>
+      </c>
+      <c r="N109" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O109" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P109" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-115；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-109</t>
+        </is>
+      </c>
+      <c r="B110" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C110" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D110" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E110" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F110" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G110" s="29" t="n">
+        <v>185</v>
+      </c>
+      <c r="H110" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py::test_request_fingerprint_rejects_invalid_source_and_concurrency_contracts</t>
+        </is>
+      </c>
+      <c r="I110" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint 拒绝非法来源与并发合同</t>
+        </is>
+      </c>
+      <c r="J110" s="29" t="inlineStr">
+        <is>
+          <t>验证来源组合和 expected_row_version fail-closed。</t>
+        </is>
+      </c>
+      <c r="K110" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L110" s="29" t="inlineStr">
+        <is>
+          <t>非法输入明确失败。</t>
+        </is>
+      </c>
+      <c r="M110" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/部分子进程</t>
+        </is>
+      </c>
+      <c r="N110" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O110" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P110" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-115；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-110</t>
+        </is>
+      </c>
+      <c r="B111" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C111" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint</t>
+        </is>
+      </c>
+      <c r="D111" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E111" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F111" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py</t>
+        </is>
+      </c>
+      <c r="G111" s="29" t="n">
+        <v>214</v>
+      </c>
+      <c r="H111" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_request_fingerprint.py::test_request_fingerprint_is_stable_across_process_restarts</t>
+        </is>
+      </c>
+      <c r="I111" s="29" t="inlineStr">
+        <is>
+          <t>Request fingerprint 跨进程稳定</t>
+        </is>
+      </c>
+      <c r="J111" s="29" t="inlineStr">
+        <is>
+          <t>验证进程重启不改变 v1 SHA-256。</t>
+        </is>
+      </c>
+      <c r="K111" s="29" t="inlineStr">
+        <is>
+          <t>两个独立 Python 子进程</t>
+        </is>
+      </c>
+      <c r="L111" s="29" t="inlineStr">
+        <is>
+          <t>两次独立进程输出同一冻结向量。</t>
+        </is>
+      </c>
+      <c r="M111" s="29" t="inlineStr">
+        <is>
+          <t>无数据库/部分子进程</t>
+        </is>
+      </c>
+      <c r="N111" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O111" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P111" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-114；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-111</t>
+        </is>
+      </c>
+      <c r="B112" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C112" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D112" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E112" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F112" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G112" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="H112" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_allows_approved_transitions[pending-approve-approved]</t>
+        </is>
+      </c>
+      <c r="I112" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy 允许已批准状态转换｜pending-approve-approved</t>
+        </is>
+      </c>
+      <c r="J112" s="29" t="inlineStr">
+        <is>
+          <t>验证 pending approve/reject 及 approved/rejected reopen。</t>
+        </is>
+      </c>
+      <c r="K112" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：pending-approve-approved</t>
+        </is>
+      </c>
+      <c r="L112" s="29" t="inlineStr">
+        <is>
+          <t>返回合同规定的新状态。</t>
+        </is>
+      </c>
+      <c r="M112" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N112" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O112" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P112" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-007；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-112</t>
+        </is>
+      </c>
+      <c r="B113" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C113" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D113" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E113" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F113" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G113" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="H113" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_allows_approved_transitions[pending-reject-rejected]</t>
+        </is>
+      </c>
+      <c r="I113" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy 允许已批准状态转换｜pending-reject-rejected</t>
+        </is>
+      </c>
+      <c r="J113" s="29" t="inlineStr">
+        <is>
+          <t>验证 pending approve/reject 及 approved/rejected reopen。</t>
+        </is>
+      </c>
+      <c r="K113" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：pending-reject-rejected</t>
+        </is>
+      </c>
+      <c r="L113" s="29" t="inlineStr">
+        <is>
+          <t>返回合同规定的新状态。</t>
+        </is>
+      </c>
+      <c r="M113" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N113" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O113" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P113" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-007；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-113</t>
+        </is>
+      </c>
+      <c r="B114" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C114" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D114" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E114" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F114" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G114" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="H114" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_allows_approved_transitions[approved-reopen-pending]</t>
+        </is>
+      </c>
+      <c r="I114" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy 允许已批准状态转换｜approved-reopen-pending</t>
+        </is>
+      </c>
+      <c r="J114" s="29" t="inlineStr">
+        <is>
+          <t>验证 pending approve/reject 及 approved/rejected reopen。</t>
+        </is>
+      </c>
+      <c r="K114" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：approved-reopen-pending</t>
+        </is>
+      </c>
+      <c r="L114" s="29" t="inlineStr">
+        <is>
+          <t>返回合同规定的新状态。</t>
+        </is>
+      </c>
+      <c r="M114" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N114" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O114" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P114" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-007；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-114</t>
+        </is>
+      </c>
+      <c r="B115" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C115" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D115" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E115" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F115" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G115" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="H115" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_allows_approved_transitions[rejected-reopen-pending]</t>
+        </is>
+      </c>
+      <c r="I115" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy 允许已批准状态转换｜rejected-reopen-pending</t>
+        </is>
+      </c>
+      <c r="J115" s="29" t="inlineStr">
+        <is>
+          <t>验证 pending approve/reject 及 approved/rejected reopen。</t>
+        </is>
+      </c>
+      <c r="K115" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：rejected-reopen-pending</t>
+        </is>
+      </c>
+      <c r="L115" s="29" t="inlineStr">
+        <is>
+          <t>返回合同规定的新状态。</t>
+        </is>
+      </c>
+      <c r="M115" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N115" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O115" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P115" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-007；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-115</t>
+        </is>
+      </c>
+      <c r="B116" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C116" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D116" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E116" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F116" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G116" s="29" t="n">
+        <v>52</v>
+      </c>
+      <c r="H116" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_reopen_is_an_action_not_a_review_status</t>
+        </is>
+      </c>
+      <c r="I116" s="29" t="inlineStr">
+        <is>
+          <t>Reopen 是审核操作而非状态</t>
+        </is>
+      </c>
+      <c r="J116" s="29" t="inlineStr">
+        <is>
+          <t>验证审核状态仍只有 pending/approved/rejected。</t>
+        </is>
+      </c>
+      <c r="K116" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L116" s="29" t="inlineStr">
+        <is>
+          <t>reopen 仅存在于操作枚举。</t>
+        </is>
+      </c>
+      <c r="M116" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N116" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O116" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P116" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 D-07；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-116</t>
+        </is>
+      </c>
+      <c r="B117" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C117" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D117" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E117" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F117" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G117" s="29" t="n">
+        <v>66</v>
+      </c>
+      <c r="H117" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_rejects_invalid_or_unexplained_transitions[approved-approve-None]</t>
+        </is>
+      </c>
+      <c r="I117" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy 拒绝非法或缺少原因的转换｜approved-approve-None</t>
+        </is>
+      </c>
+      <c r="J117" s="29" t="inlineStr">
+        <is>
+          <t>验证重复/非法转换及 reject/reopen reason 规则。</t>
+        </is>
+      </c>
+      <c r="K117" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：approved-approve-None</t>
+        </is>
+      </c>
+      <c r="L117" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_INVALID_REVIEW_TRANSITION。</t>
+        </is>
+      </c>
+      <c r="M117" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N117" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O117" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P117" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-008；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-117</t>
+        </is>
+      </c>
+      <c r="B118" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C118" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D118" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E118" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F118" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G118" s="29" t="n">
+        <v>66</v>
+      </c>
+      <c r="H118" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_rejects_invalid_or_unexplained_transitions[pending-reopen-why]</t>
+        </is>
+      </c>
+      <c r="I118" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy 拒绝非法或缺少原因的转换｜pending-reopen-why</t>
+        </is>
+      </c>
+      <c r="J118" s="29" t="inlineStr">
+        <is>
+          <t>验证重复/非法转换及 reject/reopen reason 规则。</t>
+        </is>
+      </c>
+      <c r="K118" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：pending-reopen-why</t>
+        </is>
+      </c>
+      <c r="L118" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_INVALID_REVIEW_TRANSITION。</t>
+        </is>
+      </c>
+      <c r="M118" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N118" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O118" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P118" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-008；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-118</t>
+        </is>
+      </c>
+      <c r="B119" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C119" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D119" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E119" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F119" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G119" s="29" t="n">
+        <v>66</v>
+      </c>
+      <c r="H119" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_rejects_invalid_or_unexplained_transitions[pending-reject-  ]</t>
+        </is>
+      </c>
+      <c r="I119" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">审核 Policy 拒绝非法或缺少原因的转换｜pending-reject-  </t>
+        </is>
+      </c>
+      <c r="J119" s="29" t="inlineStr">
+        <is>
+          <t>验证重复/非法转换及 reject/reopen reason 规则。</t>
+        </is>
+      </c>
+      <c r="K119" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">参数化输入：pending-reject-  </t>
+        </is>
+      </c>
+      <c r="L119" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_INVALID_REVIEW_TRANSITION。</t>
+        </is>
+      </c>
+      <c r="M119" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N119" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O119" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P119" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-008；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-119</t>
+        </is>
+      </c>
+      <c r="B120" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C120" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy</t>
+        </is>
+      </c>
+      <c r="D120" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E120" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F120" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py</t>
+        </is>
+      </c>
+      <c r="G120" s="29" t="n">
+        <v>66</v>
+      </c>
+      <c r="H120" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_review_policy.py::test_review_policy_rejects_invalid_or_unexplained_transitions[rejected-reopen-None]</t>
+        </is>
+      </c>
+      <c r="I120" s="29" t="inlineStr">
+        <is>
+          <t>审核 Policy 拒绝非法或缺少原因的转换｜rejected-reopen-None</t>
+        </is>
+      </c>
+      <c r="J120" s="29" t="inlineStr">
+        <is>
+          <t>验证重复/非法转换及 reject/reopen reason 规则。</t>
+        </is>
+      </c>
+      <c r="K120" s="29" t="inlineStr">
+        <is>
+          <t>参数化输入：rejected-reopen-None</t>
+        </is>
+      </c>
+      <c r="L120" s="29" t="inlineStr">
+        <is>
+          <t>抛出 EVIE_INVALID_REVIEW_TRANSITION。</t>
+        </is>
+      </c>
+      <c r="M120" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N120" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O120" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P120" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-008；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-120</t>
+        </is>
+      </c>
+      <c r="B121" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C121" s="29" t="inlineStr">
+        <is>
+          <t>来源身份</t>
+        </is>
+      </c>
+      <c r="D121" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E121" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F121" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_source_policy.py</t>
+        </is>
+      </c>
+      <c r="G121" s="29" t="n">
+        <v>13</v>
+      </c>
+      <c r="H121" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_source_policy.py::test_requirement_source_identity_matches_frozen_vector</t>
+        </is>
+      </c>
+      <c r="I121" s="29" t="inlineStr">
+        <is>
+          <t>Requirement 来源身份固定向量</t>
+        </is>
+      </c>
+      <c r="J121" s="29" t="inlineStr">
+        <is>
+          <t>验证公共 Requirement/Version canonical JSON SHA-256。</t>
+        </is>
+      </c>
+      <c r="K121" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L121" s="29" t="inlineStr">
+        <is>
+          <t>输出与冻结来源身份向量一致。</t>
+        </is>
+      </c>
+      <c r="M121" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N121" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O121" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P121" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-012；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-121</t>
+        </is>
+      </c>
+      <c r="B122" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C122" s="29" t="inlineStr">
+        <is>
+          <t>来源身份</t>
+        </is>
+      </c>
+      <c r="D122" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E122" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F122" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_source_policy.py</t>
+        </is>
+      </c>
+      <c r="G122" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="H122" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_source_policy.py::test_manual_source_identity_changes_with_real_source_semantics</t>
+        </is>
+      </c>
+      <c r="I122" s="29" t="inlineStr">
+        <is>
+          <t>Manual 来源身份区分真实 Intake</t>
+        </is>
+      </c>
+      <c r="J122" s="29" t="inlineStr">
+        <is>
+          <t>验证幂等 key 等真实来源语义变化产生不同来源身份。</t>
+        </is>
+      </c>
+      <c r="K122" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L122" s="29" t="inlineStr">
+        <is>
+          <t>基础向量稳定且来源语义变化后 hash 不同。</t>
+        </is>
+      </c>
+      <c r="M122" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N122" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O122" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P122" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 EVIE-PLAN-013；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-122</t>
+        </is>
+      </c>
+      <c r="B123" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 1</t>
+        </is>
+      </c>
+      <c r="C123" s="29" t="inlineStr">
+        <is>
+          <t>来源身份</t>
+        </is>
+      </c>
+      <c r="D123" s="29" t="inlineStr">
+        <is>
+          <t>纯函数单元测试</t>
+        </is>
+      </c>
+      <c r="E123" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F123" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_source_policy.py</t>
+        </is>
+      </c>
+      <c r="G123" s="29" t="n">
+        <v>48</v>
+      </c>
+      <c r="H123" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_source_policy.py::test_source_identity_rejects_malformed_authoritative_inputs</t>
+        </is>
+      </c>
+      <c r="I123" s="29" t="inlineStr">
+        <is>
+          <t>来源身份拒绝非法权威输入</t>
+        </is>
+      </c>
+      <c r="J123" s="29" t="inlineStr">
+        <is>
+          <t>验证错误 Requirement 或 actor 身份 fail-closed。</t>
+        </is>
+      </c>
+      <c r="K123" s="29" t="inlineStr">
+        <is>
+          <t>无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L123" s="29" t="inlineStr">
+        <is>
+          <t>非法输入明确失败。</t>
+        </is>
+      </c>
+      <c r="M123" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N123" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O123" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P123" s="29" t="inlineStr">
+        <is>
+          <t>覆盖 A-07；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P78"/>
+  <autoFilter ref="A1:P123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
docs(evie-ai): record slice2-3 compatibility and validation
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -2493,7 +2493,7 @@
       </c>
       <c r="D16" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E16" s="29" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="N16" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
       </c>
       <c r="D17" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E17" s="29" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="N17" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="D18" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E18" s="29" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="N18" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="D19" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E19" s="29" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="N19" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="D20" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E20" s="29" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="N20" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="D21" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E21" s="29" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="N21" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="D22" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E22" s="29" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="N22" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="D23" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E23" s="29" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="N23" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="D24" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E24" s="29" t="inlineStr">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="N24" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="D25" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E25" s="29" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="N25" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="D26" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E26" s="29" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="N26" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="D27" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E27" s="29" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="N27" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="D28" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E28" s="29" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="N28" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="D29" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E29" s="29" t="inlineStr">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="N29" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="D30" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E30" s="29" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="N30" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="D31" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已验证（待自动化）</t>
         </is>
       </c>
       <c r="E31" s="29" t="inlineStr">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="N31" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>2026-07-15 真实 PostgreSQL 16 手工隔离验证通过；后续补 CI 自动化。</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="D32" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E32" s="29" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="N32" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="D33" s="36" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E33" s="29" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="N33" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D34" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E34" s="29" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="N34" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="D35" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E35" s="29" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="N35" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -7605,7 +7605,7 @@
       </c>
       <c r="D87" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E87" s="29" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="N87" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -7893,7 +7893,7 @@
       </c>
       <c r="D91" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E91" s="29" t="inlineStr">
@@ -7943,7 +7943,7 @@
       </c>
       <c r="N91" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -8253,7 +8253,7 @@
       </c>
       <c r="D96" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E96" s="29" t="inlineStr">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="N96" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -8325,7 +8325,7 @@
       </c>
       <c r="D97" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E97" s="29" t="inlineStr">
@@ -8375,7 +8375,7 @@
       </c>
       <c r="N97" s="29" t="inlineStr">
         <is>
-          <t>Plan 明确不复制 source_type、不使用组合 FK。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="D99" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E99" s="29" t="inlineStr">
@@ -8519,7 +8519,7 @@
       </c>
       <c r="N99" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8613,7 @@
       </c>
       <c r="D101" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E101" s="29" t="inlineStr">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="N101" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -8901,7 +8901,7 @@
       </c>
       <c r="D105" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E105" s="29" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="N105" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="D110" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E110" s="29" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="N110" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -9765,7 +9765,7 @@
       </c>
       <c r="D117" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E117" s="29" t="inlineStr">
@@ -9815,7 +9815,7 @@
       </c>
       <c r="N117" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -9837,7 +9837,7 @@
       </c>
       <c r="D118" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E118" s="29" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="N118" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -10413,7 +10413,7 @@
       </c>
       <c r="D126" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E126" s="29" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="N126" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -10485,7 +10485,7 @@
       </c>
       <c r="D127" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E127" s="29" t="inlineStr">
@@ -10535,7 +10535,7 @@
       </c>
       <c r="N127" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -10557,7 +10557,7 @@
       </c>
       <c r="D128" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已验证（待自动化）</t>
         </is>
       </c>
       <c r="E128" s="29" t="inlineStr">
@@ -10607,7 +10607,7 @@
       </c>
       <c r="N128" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>2026-07-15 真实 PostgreSQL 16 手工隔离验证通过；后续补 CI 自动化。</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="D129" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E129" s="29" t="inlineStr">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="N129" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -10989,7 +10989,7 @@
       </c>
       <c r="D134" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="E134" s="29" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="N134" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已有自动化节点覆盖；2026-07-15 定向 156 passed。</t>
         </is>
       </c>
     </row>
@@ -11061,7 +11061,7 @@
       </c>
       <c r="D135" s="35" t="inlineStr">
         <is>
-          <t>待实现</t>
+          <t>部分实现</t>
         </is>
       </c>
       <c r="E135" s="29" t="inlineStr">
@@ -11111,7 +11111,7 @@
       </c>
       <c r="N135" s="29" t="inlineStr">
         <is>
-          <t>尚未生成测试代码；实施时必须保持节点与本表可追踪。</t>
+          <t>Slice 2/3 已覆盖部分合同；剩余场景按后续切片或专用集成测试补齐。</t>
         </is>
       </c>
     </row>
@@ -11130,7 +11130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13328,6 +13328,130 @@
       <c r="L37" s="12" t="inlineStr">
         <is>
           <t>合并 closeout 后从最新 dev 创建 Slice 1 分支</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>SL23-01</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>ORM、Schema 与线性 Migration 原子交付</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>在同一分支/PR交付 Phase 1 生命周期持久化结构，保持 frozen baseline 不变</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>完成 User public ID、通用来源/Requirement 子表、幂等/Claim/Review/Audit 模型与 Schema；新增 20260715_100000 Migration、确定性回填、fail-closed upgrade/downgrade</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Slice 2 commit b33844b；Slice 3 工作区；SQLite/PostgreSQL 16 验证</t>
+        </is>
+      </c>
+      <c r="H38" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>定向 156 passed；全量相对 0aeedde 新增失败 0；PostgreSQL 16 升降级和存量回填通过</t>
+        </is>
+      </c>
+      <c r="J38" s="12" t="inlineStr">
+        <is>
+          <t>不修改 120000/121000/frozen baseline；不实现 Service、Router、完整 Slice 4 Repository</t>
+        </is>
+      </c>
+      <c r="K38" s="12" t="inlineStr">
+        <is>
+          <t>b33844b / 77c92fe</t>
+        </is>
+      </c>
+      <c r="L38" s="12" t="inlineStr">
+        <is>
+          <t>提交文档台账并创建 Slice 2/3 原子 PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>P11-01</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 兼容适配</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>Requirement 来源 Repository 主/子表兼容</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>退役主表 Requirement 专用列后保证 Phase 0 Repository 在中间版本仍可运行</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>保留 add_source 调用合同；写入通用 TestAssetSource 后 flush，再写 TestAssetRequirementSource；读取路径移除退役属性依赖；事务由上层持有</t>
+        </is>
+      </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>test_asset_repository.py、Repository 单测、PostgreSQL 16 手工事务验证</t>
+        </is>
+      </c>
+      <c r="H39" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>一次调用产生主/子两条关联记录；外层 rollback 同时清除；无 commit/rollback/独立 Session</t>
+        </is>
+      </c>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>仅批准的 P-11；不实现 Idempotency/Claim/Review/Audit/Intake Repository</t>
+        </is>
+      </c>
+      <c r="K39" s="12" t="inlineStr">
+        <is>
+          <t>77c92fe / 用户 2026-07-15 批准</t>
+        </is>
+      </c>
+      <c r="L39" s="12" t="inlineStr">
+        <is>
+          <t>随 Slice 2/3 原子 PR 审查合并</t>
         </is>
       </c>
     </row>
@@ -13896,7 +14020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15198,6 +15322,134 @@
       <c r="F42" s="12" t="inlineStr">
         <is>
           <t>未触及 ORM、Migration、Repository、Service、Router、认证模型或旧链</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>SL23-V01</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>Slice 2/3 EvieAi 与数据库基线定向回归</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>pytest：EvieAi + Alembic guard + bootstrap + identifier + deterministic baseline</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>156 passed</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>SQLite Migration、ORM、Schema、Repository、冻结基线和架构边界全部通过；29 warnings 为既有弃用提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>SL23-V02</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>Slice 2/3 全量失败节点基线对比</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>当前分支 vs 0aeedde detached worktree；相同 pytest tests/unit --tb=no</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>当前 584 passed/32 failed；基线 550 passed/32 failed；failure diff=0</t>
+        </is>
+      </c>
+      <c r="E44" s="24" t="inlineStr">
+        <is>
+          <t>通过（存在已知旧链失败）</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>32 个失败节点完全一致；Slice 2/3 新增失败 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>SL23-V03</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>Phase 1 Migration 真实 PostgreSQL 16 验证</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>隔离 Docker PostgreSQL 16：fresh bootstrap、121000↔head、存量回填、downgrade fail-closed</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>user_public_id、Requirement 来源子表、Content Claim 回填正确；业务事实存在时 downgrade 拒绝且无部分降级</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>P11-V01</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>P-11 Repository 主/子表事务验证</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>SQLite 12 个 Repository 测试 + PostgreSQL 16 外层事务强制 rollback</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>主/子记录同事务；FK 正确；rollback 后均不存在；Repository 无 commit/rollback/独立 Session</t>
         </is>
       </c>
     </row>
@@ -15229,7 +15481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16531,6 +16783,38 @@
       <c r="F42" s="12" t="inlineStr">
         <is>
           <t>内部 User.id 不作为 actor；JWT sub 兼容保留；公共身份历史快照不可重写</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>P-11</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>Requirement 来源 Repository 结构兼容适配</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>Slice 2/3 可最小适配既有 add_source 主/子表写入与直接读取，保持调用合同；不提前实施其他 Slice 4 Repository</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>已批准并实施</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>用户 2026-07-15 明确批准 / Implementation Plan P-11</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Repository 不 commit/rollback/建 Session；仅允许 flush；主子表由外层同一事务提交或回滚</t>
         </is>
       </c>
     </row>
@@ -16562,7 +16846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17448,6 +17732,38 @@
       <c r="F29" s="12" t="inlineStr">
         <is>
           <t>2026-07-15 用户明确签字</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>P-11</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Requirement 来源 Repository 兼容适配</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>退役主表旧列后最小适配主表+Requirement 子表既有读写路径</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>已批准</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Slice 2/3 Repository 新增失败阻塞已解除</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15 用户明确批准；不得扩大为完整 Slice 4 Repository</t>
         </is>
       </c>
     </row>
@@ -18128,7 +18444,7 @@
       </c>
       <c r="F3" s="29" t="inlineStr">
         <is>
-          <t>codex/evie-ai-phase1-slice1-policies</t>
+          <t>codex/evie-ai-phase1-slice2-3-database</t>
         </is>
       </c>
       <c r="G3" s="5" t="n"/>
@@ -18141,7 +18457,7 @@
         </is>
       </c>
       <c r="B4" s="29" t="n">
-        <v>122</v>
+        <v>156</v>
       </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
@@ -18152,7 +18468,7 @@
       </c>
       <c r="F4" s="29" t="inlineStr">
         <is>
-          <t>EvieAi 96 passed；全量 550 passed, 32 known legacy failures；新增失败 0</t>
+          <t>定向 156 passed；全量 584 passed, 32 known legacy failures；相对 0aeedde 新增失败 0</t>
         </is>
       </c>
       <c r="G4" s="5" t="n"/>
@@ -18165,7 +18481,7 @@
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="6" t="n"/>
@@ -18188,7 +18504,7 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>dev@e111f21 + Slice 1 未提交工作区</t>
+          <t>dev@7b0957b + Slice 2 b33844b + Slice 3 77c92fe</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -18200,7 +18516,7 @@
       </c>
       <c r="F6" s="29" t="inlineStr">
         <is>
-          <t>20260713_121000</t>
+          <t>20260715_100000</t>
         </is>
       </c>
       <c r="G6" s="5" t="n"/>
@@ -18261,7 +18577,7 @@
         </is>
       </c>
       <c r="F11" s="31" t="n">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="G11" s="31" t="n"/>
       <c r="H11" s="31" t="n"/>
@@ -18283,7 +18599,7 @@
         </is>
       </c>
       <c r="F12" s="31" t="n">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="G12" s="31" t="n"/>
       <c r="H12" s="31" t="n"/>
@@ -18299,8 +18615,14 @@
       </c>
       <c r="C13" s="31" t="n"/>
       <c r="D13" s="31" t="n"/>
-      <c r="E13" s="31" t="n"/>
-      <c r="F13" s="31" t="n"/>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>部分实现</t>
+        </is>
+      </c>
+      <c r="F13" s="31" t="n">
+        <v>8</v>
+      </c>
       <c r="G13" s="31" t="n"/>
       <c r="H13" s="31" t="n"/>
     </row>
@@ -18311,12 +18633,18 @@
         </is>
       </c>
       <c r="B14" s="31" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C14" s="31" t="n"/>
       <c r="D14" s="31" t="n"/>
-      <c r="E14" s="31" t="n"/>
-      <c r="F14" s="31" t="n"/>
+      <c r="E14" s="31" t="inlineStr">
+        <is>
+          <t>已验证（待自动化）</t>
+        </is>
+      </c>
+      <c r="F14" s="31" t="n">
+        <v>2</v>
+      </c>
       <c r="G14" s="31" t="n"/>
       <c r="H14" s="31" t="n"/>
     </row>
@@ -18327,7 +18655,7 @@
         </is>
       </c>
       <c r="B15" s="31" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C15" s="31" t="n"/>
       <c r="D15" s="31" t="n"/>
@@ -18343,7 +18671,7 @@
         </is>
       </c>
       <c r="B16" s="31" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C16" s="31" t="n"/>
       <c r="D16" s="31" t="n"/>
@@ -18359,7 +18687,7 @@
         </is>
       </c>
       <c r="B17" s="31" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="31" t="n"/>
@@ -18375,7 +18703,7 @@
         </is>
       </c>
       <c r="B18" s="31" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="31" t="n"/>
@@ -18432,6 +18760,16 @@
       <c r="G21" s="31" t="n"/>
       <c r="H21" s="31" t="n"/>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>User/JWT 兼容</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" s="30" t="inlineStr">
         <is>
@@ -18477,7 +18815,7 @@
     <row r="29">
       <c r="A29" s="32" t="inlineStr">
         <is>
-          <t>6. Slice 0 已合并；Slice 1 Policy/ID 测试已实现并通过，代码尚未提交。</t>
+          <t>6. Slice 2/3 已实现并完成代码提交：当前 156 个相关 pytest 节点；7 个旧节点保留为历史替换记录。</t>
         </is>
       </c>
     </row>
@@ -18513,7 +18851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P123"/>
+  <dimension ref="A1:P164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -18959,7 +19297,7 @@
       </c>
       <c r="E6" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F6" s="29" t="inlineStr">
@@ -19007,12 +19345,12 @@
       </c>
       <c r="O6" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P6" s="29" t="inlineStr">
         <is>
-          <t>本次定向执行：77 passed；参数化节点按实际 pytest node 维护。</t>
+          <t>已由 Phase 1 通用来源/Requirement 子表架构守卫替代</t>
         </is>
       </c>
     </row>
@@ -19119,7 +19457,7 @@
       </c>
       <c r="E8" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F8" s="29" t="inlineStr">
@@ -19167,12 +19505,12 @@
       </c>
       <c r="O8" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P8" s="29" t="inlineStr">
         <is>
-          <t>本次定向执行：77 passed；参数化节点按实际 pytest node 维护。</t>
+          <t>已由 Phase 1 全部必需 FK 命名守卫替代</t>
         </is>
       </c>
     </row>
@@ -22239,7 +22577,7 @@
       </c>
       <c r="E47" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F47" s="29" t="inlineStr">
@@ -22287,12 +22625,12 @@
       </c>
       <c r="O47" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P47" s="29" t="inlineStr">
         <is>
-          <t>本次定向执行：77 passed；参数化节点按实际 pytest node 维护。</t>
+          <t>已由 Intake 身份与治理字段拒绝合同替代</t>
         </is>
       </c>
     </row>
@@ -22319,7 +22657,7 @@
       </c>
       <c r="E48" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F48" s="29" t="inlineStr">
@@ -22367,12 +22705,12 @@
       </c>
       <c r="O48" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P48" s="29" t="inlineStr">
         <is>
-          <t>本次定向执行：77 passed；参数化节点按实际 pytest node 维护。</t>
+          <t>已由自然语言内容 Schema 合同替代</t>
         </is>
       </c>
     </row>
@@ -22399,7 +22737,7 @@
       </c>
       <c r="E49" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F49" s="29" t="inlineStr">
@@ -22447,12 +22785,12 @@
       </c>
       <c r="O49" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P49" s="29" t="inlineStr">
         <is>
-          <t>本次定向执行：77 passed；参数化节点按实际 pytest node 维护。</t>
+          <t>已由自然语言内容机器字段拒绝合同替代</t>
         </is>
       </c>
     </row>
@@ -22479,7 +22817,7 @@
       </c>
       <c r="E50" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F50" s="29" t="inlineStr">
@@ -22527,12 +22865,12 @@
       </c>
       <c r="O50" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P50" s="29" t="inlineStr">
         <is>
-          <t>本次定向执行：77 passed；参数化节点按实际 pytest node 维护。</t>
+          <t>已由来源 discriminated union 合同替代</t>
         </is>
       </c>
     </row>
@@ -22879,7 +23217,7 @@
       </c>
       <c r="E55" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F55" s="29" t="inlineStr">
@@ -22927,12 +23265,12 @@
       </c>
       <c r="O55" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P55" s="29" t="inlineStr">
         <is>
-          <t>本次定向执行：77 passed；参数化节点按实际 pytest node 维护。</t>
+          <t>已由 legacy override 不替代 deterministic bootstrap 合同替代</t>
         </is>
       </c>
     </row>
@@ -28373,6 +28711,3286 @@
       <c r="P123" s="29" t="inlineStr">
         <is>
           <t>覆盖 A-07；Slice 1 定向执行 96 passed；相对 e111f21 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-123</t>
+        </is>
+      </c>
+      <c r="B124" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C124" s="29" t="inlineStr">
+        <is>
+          <t>架构守卫</t>
+        </is>
+      </c>
+      <c r="D124" s="29" t="inlineStr">
+        <is>
+          <t>静态/结构单元测试</t>
+        </is>
+      </c>
+      <c r="E124" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F124" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_architecture_boundaries.py</t>
+        </is>
+      </c>
+      <c r="G124" s="29" t="n">
+        <v>171</v>
+      </c>
+      <c r="H124" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_architecture_boundaries.py::test_phase1_source_schema_separates_common_and_requirement_facts</t>
+        </is>
+      </c>
+      <c r="I124" s="29" t="inlineStr">
+        <is>
+          <t>phase1 source schema separates common and requirement facts</t>
+        </is>
+      </c>
+      <c r="J124" s="29" t="inlineStr">
+        <is>
+          <t>验证：phase1 source schema separates common and requirement facts。</t>
+        </is>
+      </c>
+      <c r="K124" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L124" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M124" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N124" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O124" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P124" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-124</t>
+        </is>
+      </c>
+      <c r="B125" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C125" s="29" t="inlineStr">
+        <is>
+          <t>架构守卫</t>
+        </is>
+      </c>
+      <c r="D125" s="29" t="inlineStr">
+        <is>
+          <t>静态/结构单元测试</t>
+        </is>
+      </c>
+      <c r="E125" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F125" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_architecture_boundaries.py</t>
+        </is>
+      </c>
+      <c r="G125" s="29" t="n">
+        <v>203</v>
+      </c>
+      <c r="H125" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_architecture_boundaries.py::test_required_foreign_keys_are_explicit_and_named</t>
+        </is>
+      </c>
+      <c r="I125" s="29" t="inlineStr">
+        <is>
+          <t>required foreign keys are explicit and named</t>
+        </is>
+      </c>
+      <c r="J125" s="29" t="inlineStr">
+        <is>
+          <t>验证：required foreign keys are explicit and named。</t>
+        </is>
+      </c>
+      <c r="K125" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L125" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M125" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N125" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O125" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P125" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-125</t>
+        </is>
+      </c>
+      <c r="B126" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C126" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D126" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E126" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F126" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G126" s="29" t="n">
+        <v>426</v>
+      </c>
+      <c r="H126" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_all_evie_ai_schema_identifiers_fit_postgresql_limit</t>
+        </is>
+      </c>
+      <c r="I126" s="29" t="inlineStr">
+        <is>
+          <t>all evie ai schema identifiers fit postgresql limit</t>
+        </is>
+      </c>
+      <c r="J126" s="29" t="inlineStr">
+        <is>
+          <t>验证：all evie ai schema identifiers fit postgresql limit。</t>
+        </is>
+      </c>
+      <c r="K126" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L126" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M126" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N126" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O126" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P126" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-126</t>
+        </is>
+      </c>
+      <c r="B127" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C127" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D127" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E127" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F127" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G127" s="29" t="n">
+        <v>444</v>
+      </c>
+      <c r="H127" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_content_claim_database_uniqueness_is_enforced</t>
+        </is>
+      </c>
+      <c r="I127" s="29" t="inlineStr">
+        <is>
+          <t>content claim database uniqueness is enforced</t>
+        </is>
+      </c>
+      <c r="J127" s="29" t="inlineStr">
+        <is>
+          <t>验证：content claim database uniqueness is enforced。</t>
+        </is>
+      </c>
+      <c r="K127" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L127" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M127" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N127" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O127" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P127" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-127</t>
+        </is>
+      </c>
+      <c r="B128" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C128" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D128" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E128" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F128" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G128" s="29" t="n">
+        <v>413</v>
+      </c>
+      <c r="H128" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_governance_records_do_not_duplicate_natural_language_content</t>
+        </is>
+      </c>
+      <c r="I128" s="29" t="inlineStr">
+        <is>
+          <t>governance records do not duplicate natural language content</t>
+        </is>
+      </c>
+      <c r="J128" s="29" t="inlineStr">
+        <is>
+          <t>验证：governance records do not duplicate natural language content。</t>
+        </is>
+      </c>
+      <c r="K128" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L128" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M128" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N128" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O128" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P128" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-128</t>
+        </is>
+      </c>
+      <c r="B129" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C129" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D129" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E129" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F129" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G129" s="29" t="n">
+        <v>308</v>
+      </c>
+      <c r="H129" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_phase1_source_models_separate_common_and_requirement_fields</t>
+        </is>
+      </c>
+      <c r="I129" s="29" t="inlineStr">
+        <is>
+          <t>phase1 source models separate common and requirement fields</t>
+        </is>
+      </c>
+      <c r="J129" s="29" t="inlineStr">
+        <is>
+          <t>验证：phase1 source models separate common and requirement fields。</t>
+        </is>
+      </c>
+      <c r="K129" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L129" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M129" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N129" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O129" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P129" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-129</t>
+        </is>
+      </c>
+      <c r="B130" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C130" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D130" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E130" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F130" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G130" s="29" t="n">
+        <v>377</v>
+      </c>
+      <c r="H130" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_phase1_state_checks_use_central_contract_values</t>
+        </is>
+      </c>
+      <c r="I130" s="29" t="inlineStr">
+        <is>
+          <t>phase1 state checks use central contract values</t>
+        </is>
+      </c>
+      <c r="J130" s="29" t="inlineStr">
+        <is>
+          <t>验证：phase1 state checks use central contract values。</t>
+        </is>
+      </c>
+      <c r="K130" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L130" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M130" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N130" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O130" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P130" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-130</t>
+        </is>
+      </c>
+      <c r="B131" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C131" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D131" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E131" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F131" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G131" s="29" t="n">
+        <v>326</v>
+      </c>
+      <c r="H131" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_phase1_uniqueness_contracts_are_present</t>
+        </is>
+      </c>
+      <c r="I131" s="29" t="inlineStr">
+        <is>
+          <t>phase1 uniqueness contracts are present</t>
+        </is>
+      </c>
+      <c r="J131" s="29" t="inlineStr">
+        <is>
+          <t>验证：phase1 uniqueness contracts are present。</t>
+        </is>
+      </c>
+      <c r="K131" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L131" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M131" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N131" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O131" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P131" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-131</t>
+        </is>
+      </c>
+      <c r="B132" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C132" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D132" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E132" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F132" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G132" s="29" t="n">
+        <v>352</v>
+      </c>
+      <c r="H132" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_review_and_audit_store_idempotency_snapshots_without_strong_fk</t>
+        </is>
+      </c>
+      <c r="I132" s="29" t="inlineStr">
+        <is>
+          <t>review and audit store idempotency snapshots without strong fk</t>
+        </is>
+      </c>
+      <c r="J132" s="29" t="inlineStr">
+        <is>
+          <t>验证：review and audit store idempotency snapshots without strong fk。</t>
+        </is>
+      </c>
+      <c r="K132" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L132" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M132" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N132" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O132" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P132" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-132</t>
+        </is>
+      </c>
+      <c r="B133" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C133" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D133" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E133" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F133" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G133" s="29" t="n">
+        <v>390</v>
+      </c>
+      <c r="H133" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_test_asset_version_has_only_approved_content_fields</t>
+        </is>
+      </c>
+      <c r="I133" s="29" t="inlineStr">
+        <is>
+          <t>test asset version has only approved content fields</t>
+        </is>
+      </c>
+      <c r="J133" s="29" t="inlineStr">
+        <is>
+          <t>验证：test asset version has only approved content fields。</t>
+        </is>
+      </c>
+      <c r="K133" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L133" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M133" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N133" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O133" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P133" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-133</t>
+        </is>
+      </c>
+      <c r="B134" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C134" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D134" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E134" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F134" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G134" s="29" t="n">
+        <v>384</v>
+      </c>
+      <c r="H134" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_user_public_id_has_no_implicit_generator_default</t>
+        </is>
+      </c>
+      <c r="I134" s="29" t="inlineStr">
+        <is>
+          <t>user public id has no implicit generator default</t>
+        </is>
+      </c>
+      <c r="J134" s="29" t="inlineStr">
+        <is>
+          <t>验证：user public id has no implicit generator default。</t>
+        </is>
+      </c>
+      <c r="K134" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L134" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M134" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N134" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O134" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P134" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-134</t>
+        </is>
+      </c>
+      <c r="B135" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C135" s="29" t="inlineStr">
+        <is>
+          <t>ORM/约束</t>
+        </is>
+      </c>
+      <c r="D135" s="29" t="inlineStr">
+        <is>
+          <t>结构/数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E135" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F135" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py</t>
+        </is>
+      </c>
+      <c r="G135" s="29" t="n">
+        <v>365</v>
+      </c>
+      <c r="H135" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_models.py::test_user_public_id_is_required_and_uniquely_constrained</t>
+        </is>
+      </c>
+      <c r="I135" s="29" t="inlineStr">
+        <is>
+          <t>user public id is required and uniquely constrained</t>
+        </is>
+      </c>
+      <c r="J135" s="29" t="inlineStr">
+        <is>
+          <t>验证：user public id is required and uniquely constrained。</t>
+        </is>
+      </c>
+      <c r="K135" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L135" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M135" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/结构反射</t>
+        </is>
+      </c>
+      <c r="N135" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O135" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P135" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-135</t>
+        </is>
+      </c>
+      <c r="B136" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C136" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D136" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E136" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F136" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G136" s="29" t="n">
+        <v>386</v>
+      </c>
+      <c r="H136" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_downgrade_with_public_user_identity_fails_without_schema_change</t>
+        </is>
+      </c>
+      <c r="I136" s="29" t="inlineStr">
+        <is>
+          <t>downgrade with public user identity fails without schema change</t>
+        </is>
+      </c>
+      <c r="J136" s="29" t="inlineStr">
+        <is>
+          <t>验证：downgrade with public user identity fails without schema change。</t>
+        </is>
+      </c>
+      <c r="K136" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L136" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M136" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N136" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O136" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P136" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-136</t>
+        </is>
+      </c>
+      <c r="B137" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C137" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D137" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E137" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F137" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G137" s="29" t="n">
+        <v>315</v>
+      </c>
+      <c r="H137" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_duplicate_active_assets_fail_closed_before_schema_changes</t>
+        </is>
+      </c>
+      <c r="I137" s="29" t="inlineStr">
+        <is>
+          <t>duplicate active assets fail closed before schema changes</t>
+        </is>
+      </c>
+      <c r="J137" s="29" t="inlineStr">
+        <is>
+          <t>验证：duplicate active assets fail closed before schema changes。</t>
+        </is>
+      </c>
+      <c r="K137" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L137" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M137" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N137" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O137" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P137" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-137</t>
+        </is>
+      </c>
+      <c r="B138" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C138" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D138" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E138" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F138" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G138" s="29" t="n">
+        <v>359</v>
+      </c>
+      <c r="H138" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_empty_database_can_downgrade_and_upgrade_again</t>
+        </is>
+      </c>
+      <c r="I138" s="29" t="inlineStr">
+        <is>
+          <t>empty database can downgrade and upgrade again</t>
+        </is>
+      </c>
+      <c r="J138" s="29" t="inlineStr">
+        <is>
+          <t>验证：empty database can downgrade and upgrade again。</t>
+        </is>
+      </c>
+      <c r="K138" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L138" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M138" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N138" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O138" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P138" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-138</t>
+        </is>
+      </c>
+      <c r="B139" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C139" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D139" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E139" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F139" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G139" s="29" t="n">
+        <v>246</v>
+      </c>
+      <c r="H139" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_fresh_bootstrap_reaches_phase1_head_with_authorized_retirement</t>
+        </is>
+      </c>
+      <c r="I139" s="29" t="inlineStr">
+        <is>
+          <t>fresh bootstrap reaches phase1 head with authorized retirement</t>
+        </is>
+      </c>
+      <c r="J139" s="29" t="inlineStr">
+        <is>
+          <t>验证：fresh bootstrap reaches phase1 head with authorized retirement。</t>
+        </is>
+      </c>
+      <c r="K139" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L139" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M139" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N139" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O139" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P139" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-139</t>
+        </is>
+      </c>
+      <c r="B140" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C140" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D140" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E140" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F140" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G140" s="29" t="n">
+        <v>331</v>
+      </c>
+      <c r="H140" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_invalid_current_version_fails_closed_before_schema_changes</t>
+        </is>
+      </c>
+      <c r="I140" s="29" t="inlineStr">
+        <is>
+          <t>invalid current version fails closed before schema changes</t>
+        </is>
+      </c>
+      <c r="J140" s="29" t="inlineStr">
+        <is>
+          <t>验证：invalid current version fails closed before schema changes。</t>
+        </is>
+      </c>
+      <c r="K140" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L140" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M140" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N140" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O140" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P140" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-140</t>
+        </is>
+      </c>
+      <c r="B141" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C141" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D141" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E141" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F141" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G141" s="29" t="n">
+        <v>413</v>
+      </c>
+      <c r="H141" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_migration_fingerprint_is_frozen_and_matches_application_vector</t>
+        </is>
+      </c>
+      <c r="I141" s="29" t="inlineStr">
+        <is>
+          <t>migration fingerprint is frozen and matches application vector</t>
+        </is>
+      </c>
+      <c r="J141" s="29" t="inlineStr">
+        <is>
+          <t>验证：migration fingerprint is frozen and matches application vector。</t>
+        </is>
+      </c>
+      <c r="K141" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L141" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M141" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N141" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O141" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P141" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-141</t>
+        </is>
+      </c>
+      <c r="B142" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C142" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D142" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E142" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F142" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G142" s="29" t="n">
+        <v>271</v>
+      </c>
+      <c r="H142" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_phase0_data_is_backfilled_without_losing_requirement_source</t>
+        </is>
+      </c>
+      <c r="I142" s="29" t="inlineStr">
+        <is>
+          <t>phase0 data is backfilled without losing requirement source</t>
+        </is>
+      </c>
+      <c r="J142" s="29" t="inlineStr">
+        <is>
+          <t>验证：phase0 data is backfilled without losing requirement source。</t>
+        </is>
+      </c>
+      <c r="K142" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L142" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M142" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N142" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O142" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P142" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-142</t>
+        </is>
+      </c>
+      <c r="B143" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 3</t>
+        </is>
+      </c>
+      <c r="C143" s="29" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="D143" s="29" t="inlineStr">
+        <is>
+          <t>迁移集成测试</t>
+        </is>
+      </c>
+      <c r="E143" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F143" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py</t>
+        </is>
+      </c>
+      <c r="G143" s="29" t="n">
+        <v>345</v>
+      </c>
+      <c r="H143" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_phase1_migration.py::test_requirement_source_scope_mismatch_fails_closed_before_schema_changes</t>
+        </is>
+      </c>
+      <c r="I143" s="29" t="inlineStr">
+        <is>
+          <t>requirement source scope mismatch fails closed before schema changes</t>
+        </is>
+      </c>
+      <c r="J143" s="29" t="inlineStr">
+        <is>
+          <t>验证：requirement source scope mismatch fails closed before schema changes。</t>
+        </is>
+      </c>
+      <c r="K143" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L143" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M143" s="29" t="inlineStr">
+        <is>
+          <t>SQLite（真实 PostgreSQL 16 另有验证记录）</t>
+        </is>
+      </c>
+      <c r="N143" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O143" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P143" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-143</t>
+        </is>
+      </c>
+      <c r="B144" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3</t>
+        </is>
+      </c>
+      <c r="C144" s="29" t="inlineStr">
+        <is>
+          <t>Repository/事务</t>
+        </is>
+      </c>
+      <c r="D144" s="29" t="inlineStr">
+        <is>
+          <t>数据库单元测试</t>
+        </is>
+      </c>
+      <c r="E144" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F144" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_repositories.py</t>
+        </is>
+      </c>
+      <c r="G144" s="29" t="n">
+        <v>334</v>
+      </c>
+      <c r="H144" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_repositories.py::test_requirement_source_main_and_subtype_roll_back_together</t>
+        </is>
+      </c>
+      <c r="I144" s="29" t="inlineStr">
+        <is>
+          <t>requirement source main and subtype roll back together</t>
+        </is>
+      </c>
+      <c r="J144" s="29" t="inlineStr">
+        <is>
+          <t>验证：requirement source main and subtype roll back together。</t>
+        </is>
+      </c>
+      <c r="K144" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L144" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M144" s="29" t="inlineStr">
+        <is>
+          <t>SQLite foreign_keys=ON</t>
+        </is>
+      </c>
+      <c r="N144" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O144" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P144" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-144</t>
+        </is>
+      </c>
+      <c r="B145" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C145" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D145" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E145" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F145" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G145" s="29" t="n">
+        <v>126</v>
+      </c>
+      <c r="H145" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_intake_rejects_client_controlled_identity_and_governance_fields</t>
+        </is>
+      </c>
+      <c r="I145" s="29" t="inlineStr">
+        <is>
+          <t>intake rejects client controlled identity and governance fields</t>
+        </is>
+      </c>
+      <c r="J145" s="29" t="inlineStr">
+        <is>
+          <t>验证：intake rejects client controlled identity and governance fields。</t>
+        </is>
+      </c>
+      <c r="K145" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L145" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M145" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N145" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O145" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P145" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-145</t>
+        </is>
+      </c>
+      <c r="B146" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C146" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D146" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E146" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F146" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G146" s="29" t="n">
+        <v>270</v>
+      </c>
+      <c r="H146" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_list_query_has_frozen_pagination_defaults_and_limits</t>
+        </is>
+      </c>
+      <c r="I146" s="29" t="inlineStr">
+        <is>
+          <t>list query has frozen pagination defaults and limits</t>
+        </is>
+      </c>
+      <c r="J146" s="29" t="inlineStr">
+        <is>
+          <t>验证：list query has frozen pagination defaults and limits。</t>
+        </is>
+      </c>
+      <c r="K146" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L146" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M146" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N146" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O146" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P146" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-146</t>
+        </is>
+      </c>
+      <c r="B147" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C147" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D147" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E147" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F147" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G147" s="29" t="n">
+        <v>173</v>
+      </c>
+      <c r="H147" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_natural_language_content_accepts_incomplete_content</t>
+        </is>
+      </c>
+      <c r="I147" s="29" t="inlineStr">
+        <is>
+          <t>natural language content accepts incomplete content</t>
+        </is>
+      </c>
+      <c r="J147" s="29" t="inlineStr">
+        <is>
+          <t>验证：natural language content accepts incomplete content。</t>
+        </is>
+      </c>
+      <c r="K147" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L147" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M147" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N147" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O147" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P147" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-147</t>
+        </is>
+      </c>
+      <c r="B148" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C148" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D148" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E148" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F148" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G148" s="29" t="n">
+        <v>180</v>
+      </c>
+      <c r="H148" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_natural_language_content_rejects_machine_execution_payload</t>
+        </is>
+      </c>
+      <c r="I148" s="29" t="inlineStr">
+        <is>
+          <t>natural language content rejects machine execution payload</t>
+        </is>
+      </c>
+      <c r="J148" s="29" t="inlineStr">
+        <is>
+          <t>验证：natural language content rejects machine execution payload。</t>
+        </is>
+      </c>
+      <c r="K148" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L148" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M148" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N148" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O148" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P148" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-148</t>
+        </is>
+      </c>
+      <c r="B149" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C149" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D149" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E149" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F149" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G149" s="29" t="n">
+        <v>258</v>
+      </c>
+      <c r="H149" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_operation_result_contains_only_stable_public_result_summary</t>
+        </is>
+      </c>
+      <c r="I149" s="29" t="inlineStr">
+        <is>
+          <t>operation result contains only stable public result summary</t>
+        </is>
+      </c>
+      <c r="J149" s="29" t="inlineStr">
+        <is>
+          <t>验证：operation result contains only stable public result summary。</t>
+        </is>
+      </c>
+      <c r="K149" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L149" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M149" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N149" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O149" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P149" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-149</t>
+        </is>
+      </c>
+      <c r="B150" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C150" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D150" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E150" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F150" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G150" s="29" t="n">
+        <v>203</v>
+      </c>
+      <c r="H150" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_review_write_targets_explicit_version_and_current_row_version</t>
+        </is>
+      </c>
+      <c r="I150" s="29" t="inlineStr">
+        <is>
+          <t>review write targets explicit version and current row version</t>
+        </is>
+      </c>
+      <c r="J150" s="29" t="inlineStr">
+        <is>
+          <t>验证：review write targets explicit version and current row version。</t>
+        </is>
+      </c>
+      <c r="K150" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L150" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M150" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N150" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O150" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P150" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-150</t>
+        </is>
+      </c>
+      <c r="B151" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C151" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D151" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E151" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F151" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G151" s="29" t="n">
+        <v>147</v>
+      </c>
+      <c r="H151" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_source_discriminated_union_accepts_only_approved_shapes</t>
+        </is>
+      </c>
+      <c r="I151" s="29" t="inlineStr">
+        <is>
+          <t>source discriminated union accepts only approved shapes</t>
+        </is>
+      </c>
+      <c r="J151" s="29" t="inlineStr">
+        <is>
+          <t>验证：source discriminated union accepts only approved shapes。</t>
+        </is>
+      </c>
+      <c r="K151" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L151" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M151" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N151" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O151" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P151" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-151</t>
+        </is>
+      </c>
+      <c r="B152" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C152" s="29" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="D152" s="29" t="inlineStr">
+        <is>
+          <t>Schema 单元测试</t>
+        </is>
+      </c>
+      <c r="E152" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F152" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py</t>
+        </is>
+      </c>
+      <c r="G152" s="29" t="n">
+        <v>189</v>
+      </c>
+      <c r="H152" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_schemas.py::test_version_and_lifecycle_writes_require_positive_row_version</t>
+        </is>
+      </c>
+      <c r="I152" s="29" t="inlineStr">
+        <is>
+          <t>version and lifecycle writes require positive row version</t>
+        </is>
+      </c>
+      <c r="J152" s="29" t="inlineStr">
+        <is>
+          <t>验证：version and lifecycle writes require positive row version。</t>
+        </is>
+      </c>
+      <c r="K152" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L152" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M152" s="29" t="inlineStr">
+        <is>
+          <t>无数据库</t>
+        </is>
+      </c>
+      <c r="N152" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O152" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P152" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-152</t>
+        </is>
+      </c>
+      <c r="B153" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C153" s="29" t="inlineStr">
+        <is>
+          <t>User/JWT兼容</t>
+        </is>
+      </c>
+      <c r="D153" s="29" t="inlineStr">
+        <is>
+          <t>兼容性单元测试</t>
+        </is>
+      </c>
+      <c r="E153" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F153" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G153" s="29" t="n">
+        <v>49</v>
+      </c>
+      <c r="H153" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_registration_allocates_public_identity_from_shared_generator</t>
+        </is>
+      </c>
+      <c r="I153" s="29" t="inlineStr">
+        <is>
+          <t>registration allocates public identity from shared generator</t>
+        </is>
+      </c>
+      <c r="J153" s="29" t="inlineStr">
+        <is>
+          <t>验证：registration allocates public identity from shared generator。</t>
+        </is>
+      </c>
+      <c r="K153" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L153" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M153" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/无数据库</t>
+        </is>
+      </c>
+      <c r="N153" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O153" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P153" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-153</t>
+        </is>
+      </c>
+      <c r="B154" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C154" s="29" t="inlineStr">
+        <is>
+          <t>User/JWT兼容</t>
+        </is>
+      </c>
+      <c r="D154" s="29" t="inlineStr">
+        <is>
+          <t>兼容性单元测试</t>
+        </is>
+      </c>
+      <c r="E154" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F154" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G154" s="29" t="n">
+        <v>69</v>
+      </c>
+      <c r="H154" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_token_subject_remains_internal_user_id_for_compatibility</t>
+        </is>
+      </c>
+      <c r="I154" s="29" t="inlineStr">
+        <is>
+          <t>token subject remains internal user id for compatibility</t>
+        </is>
+      </c>
+      <c r="J154" s="29" t="inlineStr">
+        <is>
+          <t>验证：token subject remains internal user id for compatibility。</t>
+        </is>
+      </c>
+      <c r="K154" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L154" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M154" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/无数据库</t>
+        </is>
+      </c>
+      <c r="N154" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O154" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P154" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-154</t>
+        </is>
+      </c>
+      <c r="B155" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2</t>
+        </is>
+      </c>
+      <c r="C155" s="29" t="inlineStr">
+        <is>
+          <t>User/JWT兼容</t>
+        </is>
+      </c>
+      <c r="D155" s="29" t="inlineStr">
+        <is>
+          <t>兼容性单元测试</t>
+        </is>
+      </c>
+      <c r="E155" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F155" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G155" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="H155" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_user_create_rejects_client_supplied_public_identity</t>
+        </is>
+      </c>
+      <c r="I155" s="29" t="inlineStr">
+        <is>
+          <t>user create rejects client supplied public identity</t>
+        </is>
+      </c>
+      <c r="J155" s="29" t="inlineStr">
+        <is>
+          <t>验证：user create rejects client supplied public identity。</t>
+        </is>
+      </c>
+      <c r="K155" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L155" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M155" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/无数据库</t>
+        </is>
+      </c>
+      <c r="N155" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O155" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P155" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-155</t>
+        </is>
+      </c>
+      <c r="B156" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C156" s="29" t="inlineStr">
+        <is>
+          <t>Alembic 空库守卫</t>
+        </is>
+      </c>
+      <c r="D156" s="29" t="inlineStr">
+        <is>
+          <t>迁移安全单元测试</t>
+        </is>
+      </c>
+      <c r="E156" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F156" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_alembic_empty_database_guard.py</t>
+        </is>
+      </c>
+      <c r="G156" s="29" t="n">
+        <v>57</v>
+      </c>
+      <c r="H156" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_alembic_empty_database_guard.py::test_legacy_override_does_not_replace_deterministic_bootstrap</t>
+        </is>
+      </c>
+      <c r="I156" s="29" t="inlineStr">
+        <is>
+          <t>legacy override does not replace deterministic bootstrap</t>
+        </is>
+      </c>
+      <c r="J156" s="29" t="inlineStr">
+        <is>
+          <t>验证：legacy override does not replace deterministic bootstrap。</t>
+        </is>
+      </c>
+      <c r="K156" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L156" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M156" s="29" t="inlineStr">
+        <is>
+          <t>临时 SQLite</t>
+        </is>
+      </c>
+      <c r="N156" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O156" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P156" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-156</t>
+        </is>
+      </c>
+      <c r="B157" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C157" s="29" t="inlineStr">
+        <is>
+          <t>Bootstrap</t>
+        </is>
+      </c>
+      <c r="D157" s="29" t="inlineStr">
+        <is>
+          <t>数据库启动单元测试</t>
+        </is>
+      </c>
+      <c r="E157" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F157" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py</t>
+        </is>
+      </c>
+      <c r="G157" s="29" t="n">
+        <v>357</v>
+      </c>
+      <c r="H157" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py::test_descendant_health_check_passes_lineage_authorization_to_fingerprint</t>
+        </is>
+      </c>
+      <c r="I157" s="29" t="inlineStr">
+        <is>
+          <t>descendant health check passes lineage authorization to fingerprint</t>
+        </is>
+      </c>
+      <c r="J157" s="29" t="inlineStr">
+        <is>
+          <t>验证：descendant health check passes lineage authorization to fingerprint。</t>
+        </is>
+      </c>
+      <c r="K157" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L157" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M157" s="29" t="inlineStr">
+        <is>
+          <t>临时 SQLite</t>
+        </is>
+      </c>
+      <c r="N157" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O157" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P157" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-157</t>
+        </is>
+      </c>
+      <c r="B158" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C158" s="29" t="inlineStr">
+        <is>
+          <t>Bootstrap</t>
+        </is>
+      </c>
+      <c r="D158" s="29" t="inlineStr">
+        <is>
+          <t>数据库启动单元测试</t>
+        </is>
+      </c>
+      <c r="E158" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F158" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py</t>
+        </is>
+      </c>
+      <c r="G158" s="29" t="n">
+        <v>80</v>
+      </c>
+      <c r="H158" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py::test_empty_bootstrap_validates_schema_after_upgrade</t>
+        </is>
+      </c>
+      <c r="I158" s="29" t="inlineStr">
+        <is>
+          <t>empty bootstrap validates schema after upgrade</t>
+        </is>
+      </c>
+      <c r="J158" s="29" t="inlineStr">
+        <is>
+          <t>验证：empty bootstrap validates schema after upgrade。</t>
+        </is>
+      </c>
+      <c r="K158" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L158" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M158" s="29" t="inlineStr">
+        <is>
+          <t>临时 SQLite</t>
+        </is>
+      </c>
+      <c r="N158" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O158" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P158" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-158</t>
+        </is>
+      </c>
+      <c r="B159" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C159" s="29" t="inlineStr">
+        <is>
+          <t>Bootstrap</t>
+        </is>
+      </c>
+      <c r="D159" s="29" t="inlineStr">
+        <is>
+          <t>数据库启动单元测试</t>
+        </is>
+      </c>
+      <c r="E159" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F159" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py</t>
+        </is>
+      </c>
+      <c r="G159" s="29" t="n">
+        <v>110</v>
+      </c>
+      <c r="H159" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py::test_managed_bootstrap_validates_schema_before_and_after_upgrade</t>
+        </is>
+      </c>
+      <c r="I159" s="29" t="inlineStr">
+        <is>
+          <t>managed bootstrap validates schema before and after upgrade</t>
+        </is>
+      </c>
+      <c r="J159" s="29" t="inlineStr">
+        <is>
+          <t>验证：managed bootstrap validates schema before and after upgrade。</t>
+        </is>
+      </c>
+      <c r="K159" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L159" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M159" s="29" t="inlineStr">
+        <is>
+          <t>临时 SQLite</t>
+        </is>
+      </c>
+      <c r="N159" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O159" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P159" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-159</t>
+        </is>
+      </c>
+      <c r="B160" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C160" s="29" t="inlineStr">
+        <is>
+          <t>Bootstrap</t>
+        </is>
+      </c>
+      <c r="D160" s="29" t="inlineStr">
+        <is>
+          <t>数据库启动单元测试</t>
+        </is>
+      </c>
+      <c r="E160" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F160" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py</t>
+        </is>
+      </c>
+      <c r="G160" s="29" t="n">
+        <v>306</v>
+      </c>
+      <c r="H160" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_bootstrap_database.py::test_retirement_authorization_uses_alembic_revision_lineage</t>
+        </is>
+      </c>
+      <c r="I160" s="29" t="inlineStr">
+        <is>
+          <t>retirement authorization uses alembic revision lineage</t>
+        </is>
+      </c>
+      <c r="J160" s="29" t="inlineStr">
+        <is>
+          <t>验证：retirement authorization uses alembic revision lineage。</t>
+        </is>
+      </c>
+      <c r="K160" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L160" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M160" s="29" t="inlineStr">
+        <is>
+          <t>临时 SQLite</t>
+        </is>
+      </c>
+      <c r="N160" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O160" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P160" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-160</t>
+        </is>
+      </c>
+      <c r="B161" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C161" s="29" t="inlineStr">
+        <is>
+          <t>冻结结构</t>
+        </is>
+      </c>
+      <c r="D161" s="29" t="inlineStr">
+        <is>
+          <t>结构单元测试</t>
+        </is>
+      </c>
+      <c r="E161" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F161" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py</t>
+        </is>
+      </c>
+      <c r="G161" s="29" t="n">
+        <v>244</v>
+      </c>
+      <c r="H161" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py::test_authorized_retirement_does_not_hide_other_frozen_drift</t>
+        </is>
+      </c>
+      <c r="I161" s="29" t="inlineStr">
+        <is>
+          <t>authorized retirement does not hide other frozen drift</t>
+        </is>
+      </c>
+      <c r="J161" s="29" t="inlineStr">
+        <is>
+          <t>验证：authorized retirement does not hide other frozen drift。</t>
+        </is>
+      </c>
+      <c r="K161" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L161" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M161" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL 逻辑结构</t>
+        </is>
+      </c>
+      <c r="N161" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O161" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P161" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-161</t>
+        </is>
+      </c>
+      <c r="B162" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C162" s="29" t="inlineStr">
+        <is>
+          <t>冻结结构</t>
+        </is>
+      </c>
+      <c r="D162" s="29" t="inlineStr">
+        <is>
+          <t>结构单元测试</t>
+        </is>
+      </c>
+      <c r="E162" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F162" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py</t>
+        </is>
+      </c>
+      <c r="G162" s="29" t="n">
+        <v>377</v>
+      </c>
+      <c r="H162" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py::test_authorized_retirement_manifest_has_no_runtime_dependencies</t>
+        </is>
+      </c>
+      <c r="I162" s="29" t="inlineStr">
+        <is>
+          <t>authorized retirement manifest has no runtime dependencies</t>
+        </is>
+      </c>
+      <c r="J162" s="29" t="inlineStr">
+        <is>
+          <t>验证：authorized retirement manifest has no runtime dependencies。</t>
+        </is>
+      </c>
+      <c r="K162" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L162" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M162" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL 逻辑结构</t>
+        </is>
+      </c>
+      <c r="N162" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O162" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P162" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-162</t>
+        </is>
+      </c>
+      <c r="B163" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C163" s="29" t="inlineStr">
+        <is>
+          <t>冻结结构</t>
+        </is>
+      </c>
+      <c r="D163" s="29" t="inlineStr">
+        <is>
+          <t>结构单元测试</t>
+        </is>
+      </c>
+      <c r="E163" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F163" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py</t>
+        </is>
+      </c>
+      <c r="G163" s="29" t="n">
+        <v>261</v>
+      </c>
+      <c r="H163" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py::test_retirement_authorization_must_reference_frozen_objects</t>
+        </is>
+      </c>
+      <c r="I163" s="29" t="inlineStr">
+        <is>
+          <t>retirement authorization must reference frozen objects</t>
+        </is>
+      </c>
+      <c r="J163" s="29" t="inlineStr">
+        <is>
+          <t>验证：retirement authorization must reference frozen objects。</t>
+        </is>
+      </c>
+      <c r="K163" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L163" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M163" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL 逻辑结构</t>
+        </is>
+      </c>
+      <c r="N163" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O163" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P163" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-163</t>
+        </is>
+      </c>
+      <c r="B164" s="29" t="inlineStr">
+        <is>
+          <t>确定性数据库基线 + Slice 3</t>
+        </is>
+      </c>
+      <c r="C164" s="29" t="inlineStr">
+        <is>
+          <t>冻结结构</t>
+        </is>
+      </c>
+      <c r="D164" s="29" t="inlineStr">
+        <is>
+          <t>结构单元测试</t>
+        </is>
+      </c>
+      <c r="E164" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F164" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py</t>
+        </is>
+      </c>
+      <c r="G164" s="29" t="n">
+        <v>219</v>
+      </c>
+      <c r="H164" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/test_deterministic_baseline.py::test_sqlite_authorized_retirement_requires_its_replacement_shape</t>
+        </is>
+      </c>
+      <c r="I164" s="29" t="inlineStr">
+        <is>
+          <t>sqlite authorized retirement requires its replacement shape</t>
+        </is>
+      </c>
+      <c r="J164" s="29" t="inlineStr">
+        <is>
+          <t>验证：sqlite authorized retirement requires its replacement shape。</t>
+        </is>
+      </c>
+      <c r="K164" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L164" s="29" t="inlineStr">
+        <is>
+          <t>断言批准合同成立；违反该契约时测试失败。</t>
+        </is>
+      </c>
+      <c r="M164" s="29" t="inlineStr">
+        <is>
+          <t>SQLite/PostgreSQL 逻辑结构</t>
+        </is>
+      </c>
+      <c r="N164" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O164" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P164" s="29" t="inlineStr">
+        <is>
+          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(evie-ai): record public identity compatibility closure
</commit_message>
<xml_diff>
--- a/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
+++ b/docs/evie-ai/implementation/2026-07-14_15_EvieAi工作任务留档.xlsx
@@ -11130,7 +11130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13452,6 +13452,68 @@
       <c r="L39" s="12" t="inlineStr">
         <is>
           <t>随 Slice 2/3 原子 PR 审查合并</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>P10-COMPAT-01</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>PR #10 身份合同兼容收口</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>对齐 UserRead、UserCreate 与前端 AuthUser 公共身份合同</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>保留 A-11 不暴露内部 User.id，同时避免把身份覆盖拒绝扩大为注册 API 全量严格字段模式</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>UserCreate 保持 extra=ignore 并选择性拒绝 user_public_id/actor_or_client_id；AuthUser 改用 user_public_id；补 Router 201/422 合同测试</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>91c9221、Implementation Plan、Excel 测试台账</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>后端定向 10 passed；总定向 163 passed；前端 typecheck/build 通过；全量新增失败 0</t>
+        </is>
+      </c>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>仅认证兼容最小修正；不实现 RequestActorContext、权限、JWT 迁移或前端资产中心</t>
+        </is>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>91c9221 / PR #10</t>
+        </is>
+      </c>
+      <c r="L40" s="12" t="inlineStr">
+        <is>
+          <t>等待 CI 与评审后合并 PR #10</t>
         </is>
       </c>
     </row>
@@ -14020,7 +14082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15450,6 +15512,102 @@
       <c r="F46" s="12" t="inlineStr">
         <is>
           <t>主/子记录同事务；FK 正确；rollback 后均不存在；Repository 无 commit/rollback/独立 Session</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>P10-V01</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>P-10 后端注册兼容合同</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>UserCreate Schema + FastAPI /api/auth/register Router 测试</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>10 passed</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>普通未知字段继续忽略；两个身份覆盖字段单独或同时提交均 422；响应只含 user_public_id；JWT sub 保持内部 ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>P10-V02</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>P-10 前端公共身份合同</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>npm run typecheck &amp;&amp; npm run build</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>AuthUser 使用 user_public_id；无 AuthUser.id 消费点；Vite 仅报告既有 chunk size 警告</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>P10-V03</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>PR #10 最终定向与全量回归</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>定向 pytest + tests/unit 全量 + 0aeedde 失败节点对比</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>定向 163 passed；全量 591 passed/32 failed；failure diff=0</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="inlineStr">
+        <is>
+          <t>通过（存在已知旧链失败）</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>32 个失败节点与 0aeedde 基线完全一致；新增失败 0</t>
         </is>
       </c>
     </row>
@@ -18457,7 +18615,7 @@
         </is>
       </c>
       <c r="B4" s="29" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
@@ -18468,7 +18626,7 @@
       </c>
       <c r="F4" s="29" t="inlineStr">
         <is>
-          <t>定向 156 passed；全量 584 passed, 32 known legacy failures；相对 0aeedde 新增失败 0</t>
+          <t>定向 163 passed；全量 591 passed, 32 known legacy failures；相对 0aeedde 新增失败 0</t>
         </is>
       </c>
       <c r="G4" s="5" t="n"/>
@@ -18504,7 +18662,7 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>dev@7b0957b + Slice 2 b33844b + Slice 3 77c92fe</t>
+          <t>dev@7b0957b + Slice 2/3 + P-10 兼容修正 91c9221</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -18767,7 +18925,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -18815,7 +18973,7 @@
     <row r="29">
       <c r="A29" s="32" t="inlineStr">
         <is>
-          <t>6. Slice 2/3 已实现并完成代码提交：当前 156 个相关 pytest 节点；7 个旧节点保留为历史替换记录。</t>
+          <t>6. PR #10 最终兼容修正已完成：当前 163 个相关 pytest 节点；8 个旧节点保留为历史替换记录。</t>
         </is>
       </c>
     </row>
@@ -18851,7 +19009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P164"/>
+  <dimension ref="A1:P172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -31217,7 +31375,7 @@
       </c>
       <c r="E155" s="34" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>历史节点（已替换）</t>
         </is>
       </c>
       <c r="F155" s="29" t="inlineStr">
@@ -31265,12 +31423,12 @@
       </c>
       <c r="O155" s="29" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>不再收集</t>
         </is>
       </c>
       <c r="P155" s="29" t="inlineStr">
         <is>
-          <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+          <t>P-10 兼容修正后由普通未知字段兼容测试及选择性身份覆盖参数化测试替代。</t>
         </is>
       </c>
     </row>
@@ -31991,6 +32149,646 @@
       <c r="P164" s="29" t="inlineStr">
         <is>
           <t>Slice 2/3 定向 156 passed；全量相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-164</t>
+        </is>
+      </c>
+      <c r="B165" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C165" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D165" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E165" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F165" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G165" s="29" t="n">
+        <v>97</v>
+      </c>
+      <c r="H165" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_registration_api_ignores_unrelated_extra_fields</t>
+        </is>
+      </c>
+      <c r="I165" s="29" t="inlineStr">
+        <is>
+          <t>registration api ignores unrelated extra fields</t>
+        </is>
+      </c>
+      <c r="J165" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：registration api ignores unrelated extra fields。</t>
+        </is>
+      </c>
+      <c r="K165" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L165" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M165" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N165" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O165" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P165" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-165</t>
+        </is>
+      </c>
+      <c r="B166" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C166" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D166" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E166" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F166" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G166" s="29" t="n">
+        <v>128</v>
+      </c>
+      <c r="H166" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_registration_api_rejects_identity_overrides[identity_overrides0]</t>
+        </is>
+      </c>
+      <c r="I166" s="29" t="inlineStr">
+        <is>
+          <t>registration api rejects identity overrides</t>
+        </is>
+      </c>
+      <c r="J166" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：registration api rejects identity overrides。</t>
+        </is>
+      </c>
+      <c r="K166" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：identity_overrides0</t>
+        </is>
+      </c>
+      <c r="L166" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M166" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N166" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O166" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P166" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-166</t>
+        </is>
+      </c>
+      <c r="B167" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C167" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D167" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E167" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F167" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G167" s="29" t="n">
+        <v>128</v>
+      </c>
+      <c r="H167" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_registration_api_rejects_identity_overrides[identity_overrides1]</t>
+        </is>
+      </c>
+      <c r="I167" s="29" t="inlineStr">
+        <is>
+          <t>registration api rejects identity overrides</t>
+        </is>
+      </c>
+      <c r="J167" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：registration api rejects identity overrides。</t>
+        </is>
+      </c>
+      <c r="K167" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：identity_overrides1</t>
+        </is>
+      </c>
+      <c r="L167" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M167" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N167" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O167" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P167" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-167</t>
+        </is>
+      </c>
+      <c r="B168" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C168" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D168" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E168" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F168" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G168" s="29" t="n">
+        <v>128</v>
+      </c>
+      <c r="H168" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_registration_api_rejects_identity_overrides[identity_overrides2]</t>
+        </is>
+      </c>
+      <c r="I168" s="29" t="inlineStr">
+        <is>
+          <t>registration api rejects identity overrides</t>
+        </is>
+      </c>
+      <c r="J168" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：registration api rejects identity overrides。</t>
+        </is>
+      </c>
+      <c r="K168" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：identity_overrides2</t>
+        </is>
+      </c>
+      <c r="L168" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M168" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N168" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O168" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P168" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-168</t>
+        </is>
+      </c>
+      <c r="B169" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C169" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D169" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E169" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F169" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G169" s="29" t="n">
+        <v>59</v>
+      </c>
+      <c r="H169" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_user_create_ignores_unrelated_extra_fields</t>
+        </is>
+      </c>
+      <c r="I169" s="29" t="inlineStr">
+        <is>
+          <t>user create ignores unrelated extra fields</t>
+        </is>
+      </c>
+      <c r="J169" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：user create ignores unrelated extra fields。</t>
+        </is>
+      </c>
+      <c r="K169" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：无 fixture 参数</t>
+        </is>
+      </c>
+      <c r="L169" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M169" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N169" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O169" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P169" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-169</t>
+        </is>
+      </c>
+      <c r="B170" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C170" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D170" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E170" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F170" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G170" s="29" t="n">
+        <v>81</v>
+      </c>
+      <c r="H170" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_user_create_rejects_identity_overrides[identity_overrides0]</t>
+        </is>
+      </c>
+      <c r="I170" s="29" t="inlineStr">
+        <is>
+          <t>user create rejects identity overrides</t>
+        </is>
+      </c>
+      <c r="J170" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：user create rejects identity overrides。</t>
+        </is>
+      </c>
+      <c r="K170" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：identity_overrides0</t>
+        </is>
+      </c>
+      <c r="L170" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M170" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N170" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O170" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P170" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-170</t>
+        </is>
+      </c>
+      <c r="B171" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C171" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D171" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E171" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F171" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G171" s="29" t="n">
+        <v>81</v>
+      </c>
+      <c r="H171" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_user_create_rejects_identity_overrides[identity_overrides1]</t>
+        </is>
+      </c>
+      <c r="I171" s="29" t="inlineStr">
+        <is>
+          <t>user create rejects identity overrides</t>
+        </is>
+      </c>
+      <c r="J171" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：user create rejects identity overrides。</t>
+        </is>
+      </c>
+      <c r="K171" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：identity_overrides1</t>
+        </is>
+      </c>
+      <c r="L171" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M171" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N171" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O171" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P171" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="29" t="inlineStr">
+        <is>
+          <t>EVIE-ACT-171</t>
+        </is>
+      </c>
+      <c r="B172" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 Slice 2/3 P-10</t>
+        </is>
+      </c>
+      <c r="C172" s="29" t="inlineStr">
+        <is>
+          <t>User/API兼容</t>
+        </is>
+      </c>
+      <c r="D172" s="29" t="inlineStr">
+        <is>
+          <t>Schema/Router 单元测试</t>
+        </is>
+      </c>
+      <c r="E172" s="34" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="F172" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py</t>
+        </is>
+      </c>
+      <c r="G172" s="29" t="n">
+        <v>81</v>
+      </c>
+      <c r="H172" s="29" t="inlineStr">
+        <is>
+          <t>apps/web-ui-service/tests/unit/evie_ai/test_evie_ai_user_public_identity_compat.py::test_user_create_rejects_identity_overrides[identity_overrides2]</t>
+        </is>
+      </c>
+      <c r="I172" s="29" t="inlineStr">
+        <is>
+          <t>user create rejects identity overrides</t>
+        </is>
+      </c>
+      <c r="J172" s="29" t="inlineStr">
+        <is>
+          <t>验证 P-10 公共用户身份兼容合同：user create rejects identity overrides。</t>
+        </is>
+      </c>
+      <c r="K172" s="29" t="inlineStr">
+        <is>
+          <t>参数/前置：identity_overrides2</t>
+        </is>
+      </c>
+      <c r="L172" s="29" t="inlineStr">
+        <is>
+          <t>普通未知字段保持兼容；身份覆盖明确失败；响应不暴露内部 ID。</t>
+        </is>
+      </c>
+      <c r="M172" s="29" t="inlineStr">
+        <is>
+          <t>FastAPI TestClient/无真实数据库</t>
+        </is>
+      </c>
+      <c r="N172" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O172" s="29" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P172" s="29" t="inlineStr">
+        <is>
+          <t>P-10 定向 10 passed；总定向 163 passed；相对 0aeedde 新增失败 0。</t>
         </is>
       </c>
     </row>

</xml_diff>